<commit_message>
daily auto push: 2026-03-17 10:04 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3525"/>
+  <dimension ref="A1:D3526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63129,7 +63129,7 @@
     <row r="3484">
       <c r="A3484" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/03/17</t>
         </is>
       </c>
       <c r="B3484" t="inlineStr">
@@ -63138,7 +63138,7 @@
         </is>
       </c>
       <c r="C3484" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D3484" t="n">
         <v>201</v>
@@ -63156,7 +63156,7 @@
         </is>
       </c>
       <c r="C3485" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3485" t="n">
         <v>201</v>
@@ -63174,7 +63174,7 @@
         </is>
       </c>
       <c r="C3486" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3486" t="n">
         <v>201</v>
@@ -63192,7 +63192,7 @@
         </is>
       </c>
       <c r="C3487" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3487" t="n">
         <v>201</v>
@@ -63201,16 +63201,16 @@
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3488" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3488" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3488" t="n">
         <v>201</v>
@@ -63228,7 +63228,7 @@
         </is>
       </c>
       <c r="C3489" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3489" t="n">
         <v>201</v>
@@ -63246,7 +63246,7 @@
         </is>
       </c>
       <c r="C3490" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3490" t="n">
         <v>201</v>
@@ -63264,7 +63264,7 @@
         </is>
       </c>
       <c r="C3491" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3491" t="n">
         <v>201</v>
@@ -63282,7 +63282,7 @@
         </is>
       </c>
       <c r="C3492" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3492" t="n">
         <v>201</v>
@@ -63300,7 +63300,7 @@
         </is>
       </c>
       <c r="C3493" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3493" t="n">
         <v>201</v>
@@ -63309,16 +63309,16 @@
     <row r="3494">
       <c r="A3494" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3494" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3494" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3494" t="n">
         <v>201</v>
@@ -63336,7 +63336,7 @@
         </is>
       </c>
       <c r="C3495" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3495" t="n">
         <v>201</v>
@@ -63354,7 +63354,7 @@
         </is>
       </c>
       <c r="C3496" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3496" t="n">
         <v>201</v>
@@ -63372,7 +63372,7 @@
         </is>
       </c>
       <c r="C3497" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3497" t="n">
         <v>201</v>
@@ -63390,7 +63390,7 @@
         </is>
       </c>
       <c r="C3498" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3498" t="n">
         <v>201</v>
@@ -63408,7 +63408,7 @@
         </is>
       </c>
       <c r="C3499" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3499" t="n">
         <v>201</v>
@@ -63417,16 +63417,16 @@
     <row r="3500">
       <c r="A3500" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3500" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3500" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3500" t="n">
         <v>201</v>
@@ -63444,7 +63444,7 @@
         </is>
       </c>
       <c r="C3501" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3501" t="n">
         <v>201</v>
@@ -63462,7 +63462,7 @@
         </is>
       </c>
       <c r="C3502" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3502" t="n">
         <v>201</v>
@@ -63480,7 +63480,7 @@
         </is>
       </c>
       <c r="C3503" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3503" t="n">
         <v>201</v>
@@ -63498,7 +63498,7 @@
         </is>
       </c>
       <c r="C3504" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3504" t="n">
         <v>201</v>
@@ -63507,16 +63507,16 @@
     <row r="3505">
       <c r="A3505" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3505" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3505" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3505" t="n">
         <v>201</v>
@@ -63534,7 +63534,7 @@
         </is>
       </c>
       <c r="C3506" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3506" t="n">
         <v>201</v>
@@ -63552,7 +63552,7 @@
         </is>
       </c>
       <c r="C3507" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3507" t="n">
         <v>201</v>
@@ -63570,7 +63570,7 @@
         </is>
       </c>
       <c r="C3508" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3508" t="n">
         <v>201</v>
@@ -63588,7 +63588,7 @@
         </is>
       </c>
       <c r="C3509" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3509" t="n">
         <v>201</v>
@@ -63606,7 +63606,7 @@
         </is>
       </c>
       <c r="C3510" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3510" t="n">
         <v>201</v>
@@ -63624,7 +63624,7 @@
         </is>
       </c>
       <c r="C3511" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3511" t="n">
         <v>201</v>
@@ -63633,16 +63633,16 @@
     <row r="3512">
       <c r="A3512" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3512" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3512" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3512" t="n">
         <v>201</v>
@@ -63660,7 +63660,7 @@
         </is>
       </c>
       <c r="C3513" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3513" t="n">
         <v>201</v>
@@ -63678,7 +63678,7 @@
         </is>
       </c>
       <c r="C3514" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3514" t="n">
         <v>201</v>
@@ -63696,7 +63696,7 @@
         </is>
       </c>
       <c r="C3515" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3515" t="n">
         <v>201</v>
@@ -63714,7 +63714,7 @@
         </is>
       </c>
       <c r="C3516" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3516" t="n">
         <v>201</v>
@@ -63732,7 +63732,7 @@
         </is>
       </c>
       <c r="C3517" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3517" t="n">
         <v>201</v>
@@ -63750,7 +63750,7 @@
         </is>
       </c>
       <c r="C3518" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3518" t="n">
         <v>201</v>
@@ -63759,16 +63759,16 @@
     <row r="3519">
       <c r="A3519" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3519" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3519" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3519" t="n">
         <v>201</v>
@@ -63786,7 +63786,7 @@
         </is>
       </c>
       <c r="C3520" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3520" t="n">
         <v>201</v>
@@ -63804,7 +63804,7 @@
         </is>
       </c>
       <c r="C3521" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3521" t="n">
         <v>201</v>
@@ -63822,7 +63822,7 @@
         </is>
       </c>
       <c r="C3522" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3522" t="n">
         <v>201</v>
@@ -63840,7 +63840,7 @@
         </is>
       </c>
       <c r="C3523" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3523" t="n">
         <v>201</v>
@@ -63849,16 +63849,16 @@
     <row r="3524">
       <c r="A3524" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3524" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3524" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3524" t="n">
         <v>201</v>
@@ -63876,9 +63876,27 @@
         </is>
       </c>
       <c r="C3525" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3525" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3526">
+      <c r="A3526" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3526" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3526" t="n">
         <v>7</v>
       </c>
-      <c r="D3525" t="n">
+      <c r="D3526" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-03-26 10:10 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3585"/>
+  <dimension ref="A1:D3586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64209,16 +64209,16 @@
     <row r="3544">
       <c r="A3544" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/03/26</t>
         </is>
       </c>
       <c r="B3544" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3544" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D3544" t="n">
         <v>201</v>
@@ -64236,7 +64236,7 @@
         </is>
       </c>
       <c r="C3545" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3545" t="n">
         <v>201</v>
@@ -64254,7 +64254,7 @@
         </is>
       </c>
       <c r="C3546" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3546" t="n">
         <v>201</v>
@@ -64272,7 +64272,7 @@
         </is>
       </c>
       <c r="C3547" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3547" t="n">
         <v>201</v>
@@ -64281,16 +64281,16 @@
     <row r="3548">
       <c r="A3548" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3548" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3548" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3548" t="n">
         <v>201</v>
@@ -64308,7 +64308,7 @@
         </is>
       </c>
       <c r="C3549" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3549" t="n">
         <v>201</v>
@@ -64326,7 +64326,7 @@
         </is>
       </c>
       <c r="C3550" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3550" t="n">
         <v>201</v>
@@ -64344,7 +64344,7 @@
         </is>
       </c>
       <c r="C3551" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3551" t="n">
         <v>201</v>
@@ -64362,7 +64362,7 @@
         </is>
       </c>
       <c r="C3552" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3552" t="n">
         <v>201</v>
@@ -64380,7 +64380,7 @@
         </is>
       </c>
       <c r="C3553" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3553" t="n">
         <v>201</v>
@@ -64389,16 +64389,16 @@
     <row r="3554">
       <c r="A3554" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3554" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3554" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3554" t="n">
         <v>201</v>
@@ -64416,7 +64416,7 @@
         </is>
       </c>
       <c r="C3555" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3555" t="n">
         <v>201</v>
@@ -64434,7 +64434,7 @@
         </is>
       </c>
       <c r="C3556" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3556" t="n">
         <v>201</v>
@@ -64452,7 +64452,7 @@
         </is>
       </c>
       <c r="C3557" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3557" t="n">
         <v>201</v>
@@ -64470,7 +64470,7 @@
         </is>
       </c>
       <c r="C3558" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3558" t="n">
         <v>201</v>
@@ -64488,7 +64488,7 @@
         </is>
       </c>
       <c r="C3559" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3559" t="n">
         <v>201</v>
@@ -64497,16 +64497,16 @@
     <row r="3560">
       <c r="A3560" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3560" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3560" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3560" t="n">
         <v>201</v>
@@ -64524,7 +64524,7 @@
         </is>
       </c>
       <c r="C3561" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3561" t="n">
         <v>201</v>
@@ -64542,7 +64542,7 @@
         </is>
       </c>
       <c r="C3562" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3562" t="n">
         <v>201</v>
@@ -64560,7 +64560,7 @@
         </is>
       </c>
       <c r="C3563" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3563" t="n">
         <v>201</v>
@@ -64578,7 +64578,7 @@
         </is>
       </c>
       <c r="C3564" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3564" t="n">
         <v>201</v>
@@ -64587,16 +64587,16 @@
     <row r="3565">
       <c r="A3565" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3565" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3565" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3565" t="n">
         <v>201</v>
@@ -64614,7 +64614,7 @@
         </is>
       </c>
       <c r="C3566" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3566" t="n">
         <v>201</v>
@@ -64632,7 +64632,7 @@
         </is>
       </c>
       <c r="C3567" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3567" t="n">
         <v>201</v>
@@ -64650,7 +64650,7 @@
         </is>
       </c>
       <c r="C3568" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3568" t="n">
         <v>201</v>
@@ -64668,7 +64668,7 @@
         </is>
       </c>
       <c r="C3569" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3569" t="n">
         <v>201</v>
@@ -64686,7 +64686,7 @@
         </is>
       </c>
       <c r="C3570" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3570" t="n">
         <v>201</v>
@@ -64704,7 +64704,7 @@
         </is>
       </c>
       <c r="C3571" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3571" t="n">
         <v>201</v>
@@ -64713,16 +64713,16 @@
     <row r="3572">
       <c r="A3572" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3572" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3572" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3572" t="n">
         <v>201</v>
@@ -64740,7 +64740,7 @@
         </is>
       </c>
       <c r="C3573" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3573" t="n">
         <v>201</v>
@@ -64758,7 +64758,7 @@
         </is>
       </c>
       <c r="C3574" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3574" t="n">
         <v>201</v>
@@ -64776,7 +64776,7 @@
         </is>
       </c>
       <c r="C3575" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3575" t="n">
         <v>201</v>
@@ -64794,7 +64794,7 @@
         </is>
       </c>
       <c r="C3576" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3576" t="n">
         <v>201</v>
@@ -64812,7 +64812,7 @@
         </is>
       </c>
       <c r="C3577" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3577" t="n">
         <v>201</v>
@@ -64830,7 +64830,7 @@
         </is>
       </c>
       <c r="C3578" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3578" t="n">
         <v>201</v>
@@ -64839,16 +64839,16 @@
     <row r="3579">
       <c r="A3579" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3579" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3579" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3579" t="n">
         <v>201</v>
@@ -64866,7 +64866,7 @@
         </is>
       </c>
       <c r="C3580" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3580" t="n">
         <v>201</v>
@@ -64884,7 +64884,7 @@
         </is>
       </c>
       <c r="C3581" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3581" t="n">
         <v>201</v>
@@ -64902,7 +64902,7 @@
         </is>
       </c>
       <c r="C3582" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3582" t="n">
         <v>201</v>
@@ -64920,7 +64920,7 @@
         </is>
       </c>
       <c r="C3583" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3583" t="n">
         <v>201</v>
@@ -64929,16 +64929,16 @@
     <row r="3584">
       <c r="A3584" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3584" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3584" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3584" t="n">
         <v>201</v>
@@ -64956,9 +64956,27 @@
         </is>
       </c>
       <c r="C3585" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3585" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3586">
+      <c r="A3586" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3586" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3586" t="n">
         <v>7</v>
       </c>
-      <c r="D3585" t="n">
+      <c r="D3586" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-02 03:24 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3625"/>
+  <dimension ref="A1:D3626"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64929,16 +64929,16 @@
     <row r="3584">
       <c r="A3584" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/02</t>
         </is>
       </c>
       <c r="B3584" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3584" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3584" t="n">
         <v>201</v>
@@ -64956,7 +64956,7 @@
         </is>
       </c>
       <c r="C3585" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3585" t="n">
         <v>201</v>
@@ -64974,7 +64974,7 @@
         </is>
       </c>
       <c r="C3586" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3586" t="n">
         <v>201</v>
@@ -64992,7 +64992,7 @@
         </is>
       </c>
       <c r="C3587" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3587" t="n">
         <v>201</v>
@@ -65001,16 +65001,16 @@
     <row r="3588">
       <c r="A3588" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3588" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3588" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3588" t="n">
         <v>201</v>
@@ -65028,7 +65028,7 @@
         </is>
       </c>
       <c r="C3589" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3589" t="n">
         <v>201</v>
@@ -65046,7 +65046,7 @@
         </is>
       </c>
       <c r="C3590" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3590" t="n">
         <v>201</v>
@@ -65064,7 +65064,7 @@
         </is>
       </c>
       <c r="C3591" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3591" t="n">
         <v>201</v>
@@ -65082,7 +65082,7 @@
         </is>
       </c>
       <c r="C3592" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3592" t="n">
         <v>201</v>
@@ -65100,7 +65100,7 @@
         </is>
       </c>
       <c r="C3593" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3593" t="n">
         <v>201</v>
@@ -65109,16 +65109,16 @@
     <row r="3594">
       <c r="A3594" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3594" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3594" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3594" t="n">
         <v>201</v>
@@ -65136,7 +65136,7 @@
         </is>
       </c>
       <c r="C3595" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3595" t="n">
         <v>201</v>
@@ -65154,7 +65154,7 @@
         </is>
       </c>
       <c r="C3596" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3596" t="n">
         <v>201</v>
@@ -65172,7 +65172,7 @@
         </is>
       </c>
       <c r="C3597" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3597" t="n">
         <v>201</v>
@@ -65190,7 +65190,7 @@
         </is>
       </c>
       <c r="C3598" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3598" t="n">
         <v>201</v>
@@ -65208,7 +65208,7 @@
         </is>
       </c>
       <c r="C3599" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3599" t="n">
         <v>201</v>
@@ -65217,16 +65217,16 @@
     <row r="3600">
       <c r="A3600" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3600" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3600" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3600" t="n">
         <v>201</v>
@@ -65244,7 +65244,7 @@
         </is>
       </c>
       <c r="C3601" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3601" t="n">
         <v>201</v>
@@ -65262,7 +65262,7 @@
         </is>
       </c>
       <c r="C3602" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3602" t="n">
         <v>201</v>
@@ -65280,7 +65280,7 @@
         </is>
       </c>
       <c r="C3603" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3603" t="n">
         <v>201</v>
@@ -65298,7 +65298,7 @@
         </is>
       </c>
       <c r="C3604" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3604" t="n">
         <v>201</v>
@@ -65307,16 +65307,16 @@
     <row r="3605">
       <c r="A3605" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3605" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3605" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3605" t="n">
         <v>201</v>
@@ -65334,7 +65334,7 @@
         </is>
       </c>
       <c r="C3606" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3606" t="n">
         <v>201</v>
@@ -65352,7 +65352,7 @@
         </is>
       </c>
       <c r="C3607" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3607" t="n">
         <v>201</v>
@@ -65370,7 +65370,7 @@
         </is>
       </c>
       <c r="C3608" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3608" t="n">
         <v>201</v>
@@ -65388,7 +65388,7 @@
         </is>
       </c>
       <c r="C3609" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3609" t="n">
         <v>201</v>
@@ -65406,7 +65406,7 @@
         </is>
       </c>
       <c r="C3610" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3610" t="n">
         <v>201</v>
@@ -65424,7 +65424,7 @@
         </is>
       </c>
       <c r="C3611" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3611" t="n">
         <v>201</v>
@@ -65433,16 +65433,16 @@
     <row r="3612">
       <c r="A3612" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3612" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3612" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3612" t="n">
         <v>201</v>
@@ -65460,7 +65460,7 @@
         </is>
       </c>
       <c r="C3613" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3613" t="n">
         <v>201</v>
@@ -65478,7 +65478,7 @@
         </is>
       </c>
       <c r="C3614" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3614" t="n">
         <v>201</v>
@@ -65496,7 +65496,7 @@
         </is>
       </c>
       <c r="C3615" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3615" t="n">
         <v>201</v>
@@ -65514,7 +65514,7 @@
         </is>
       </c>
       <c r="C3616" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3616" t="n">
         <v>201</v>
@@ -65532,7 +65532,7 @@
         </is>
       </c>
       <c r="C3617" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3617" t="n">
         <v>201</v>
@@ -65550,7 +65550,7 @@
         </is>
       </c>
       <c r="C3618" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3618" t="n">
         <v>201</v>
@@ -65559,16 +65559,16 @@
     <row r="3619">
       <c r="A3619" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3619" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3619" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3619" t="n">
         <v>201</v>
@@ -65586,7 +65586,7 @@
         </is>
       </c>
       <c r="C3620" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3620" t="n">
         <v>201</v>
@@ -65604,7 +65604,7 @@
         </is>
       </c>
       <c r="C3621" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3621" t="n">
         <v>201</v>
@@ -65622,7 +65622,7 @@
         </is>
       </c>
       <c r="C3622" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3622" t="n">
         <v>201</v>
@@ -65640,7 +65640,7 @@
         </is>
       </c>
       <c r="C3623" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3623" t="n">
         <v>201</v>
@@ -65649,16 +65649,16 @@
     <row r="3624">
       <c r="A3624" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3624" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3624" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3624" t="n">
         <v>201</v>
@@ -65676,9 +65676,27 @@
         </is>
       </c>
       <c r="C3625" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3625" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3626">
+      <c r="A3626" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3626" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3626" t="n">
         <v>7</v>
       </c>
-      <c r="D3625" t="n">
+      <c r="D3626" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-07 10:15 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3657"/>
+  <dimension ref="A1:D3658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65505,7 +65505,7 @@
     <row r="3616">
       <c r="A3616" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/07</t>
         </is>
       </c>
       <c r="B3616" t="inlineStr">
@@ -65514,7 +65514,7 @@
         </is>
       </c>
       <c r="C3616" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D3616" t="n">
         <v>201</v>
@@ -65532,7 +65532,7 @@
         </is>
       </c>
       <c r="C3617" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3617" t="n">
         <v>201</v>
@@ -65550,7 +65550,7 @@
         </is>
       </c>
       <c r="C3618" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3618" t="n">
         <v>201</v>
@@ -65568,7 +65568,7 @@
         </is>
       </c>
       <c r="C3619" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3619" t="n">
         <v>201</v>
@@ -65577,16 +65577,16 @@
     <row r="3620">
       <c r="A3620" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3620" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3620" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3620" t="n">
         <v>201</v>
@@ -65604,7 +65604,7 @@
         </is>
       </c>
       <c r="C3621" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3621" t="n">
         <v>201</v>
@@ -65622,7 +65622,7 @@
         </is>
       </c>
       <c r="C3622" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3622" t="n">
         <v>201</v>
@@ -65640,7 +65640,7 @@
         </is>
       </c>
       <c r="C3623" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3623" t="n">
         <v>201</v>
@@ -65658,7 +65658,7 @@
         </is>
       </c>
       <c r="C3624" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3624" t="n">
         <v>201</v>
@@ -65676,7 +65676,7 @@
         </is>
       </c>
       <c r="C3625" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3625" t="n">
         <v>201</v>
@@ -65685,16 +65685,16 @@
     <row r="3626">
       <c r="A3626" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3626" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3626" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3626" t="n">
         <v>201</v>
@@ -65712,7 +65712,7 @@
         </is>
       </c>
       <c r="C3627" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3627" t="n">
         <v>201</v>
@@ -65730,7 +65730,7 @@
         </is>
       </c>
       <c r="C3628" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3628" t="n">
         <v>201</v>
@@ -65748,7 +65748,7 @@
         </is>
       </c>
       <c r="C3629" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3629" t="n">
         <v>201</v>
@@ -65766,7 +65766,7 @@
         </is>
       </c>
       <c r="C3630" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3630" t="n">
         <v>201</v>
@@ -65784,7 +65784,7 @@
         </is>
       </c>
       <c r="C3631" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3631" t="n">
         <v>201</v>
@@ -65793,16 +65793,16 @@
     <row r="3632">
       <c r="A3632" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3632" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3632" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3632" t="n">
         <v>201</v>
@@ -65820,7 +65820,7 @@
         </is>
       </c>
       <c r="C3633" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3633" t="n">
         <v>201</v>
@@ -65838,7 +65838,7 @@
         </is>
       </c>
       <c r="C3634" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3634" t="n">
         <v>201</v>
@@ -65856,7 +65856,7 @@
         </is>
       </c>
       <c r="C3635" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3635" t="n">
         <v>201</v>
@@ -65874,7 +65874,7 @@
         </is>
       </c>
       <c r="C3636" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3636" t="n">
         <v>201</v>
@@ -65883,16 +65883,16 @@
     <row r="3637">
       <c r="A3637" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3637" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3637" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3637" t="n">
         <v>201</v>
@@ -65910,7 +65910,7 @@
         </is>
       </c>
       <c r="C3638" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3638" t="n">
         <v>201</v>
@@ -65928,7 +65928,7 @@
         </is>
       </c>
       <c r="C3639" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3639" t="n">
         <v>201</v>
@@ -65946,7 +65946,7 @@
         </is>
       </c>
       <c r="C3640" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3640" t="n">
         <v>201</v>
@@ -65964,7 +65964,7 @@
         </is>
       </c>
       <c r="C3641" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3641" t="n">
         <v>201</v>
@@ -65982,7 +65982,7 @@
         </is>
       </c>
       <c r="C3642" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3642" t="n">
         <v>201</v>
@@ -66000,7 +66000,7 @@
         </is>
       </c>
       <c r="C3643" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3643" t="n">
         <v>201</v>
@@ -66009,16 +66009,16 @@
     <row r="3644">
       <c r="A3644" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3644" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3644" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3644" t="n">
         <v>201</v>
@@ -66036,7 +66036,7 @@
         </is>
       </c>
       <c r="C3645" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3645" t="n">
         <v>201</v>
@@ -66054,7 +66054,7 @@
         </is>
       </c>
       <c r="C3646" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3646" t="n">
         <v>201</v>
@@ -66072,7 +66072,7 @@
         </is>
       </c>
       <c r="C3647" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3647" t="n">
         <v>201</v>
@@ -66090,7 +66090,7 @@
         </is>
       </c>
       <c r="C3648" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3648" t="n">
         <v>201</v>
@@ -66108,7 +66108,7 @@
         </is>
       </c>
       <c r="C3649" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3649" t="n">
         <v>201</v>
@@ -66126,7 +66126,7 @@
         </is>
       </c>
       <c r="C3650" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3650" t="n">
         <v>201</v>
@@ -66135,16 +66135,16 @@
     <row r="3651">
       <c r="A3651" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3651" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3651" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3651" t="n">
         <v>201</v>
@@ -66162,7 +66162,7 @@
         </is>
       </c>
       <c r="C3652" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3652" t="n">
         <v>201</v>
@@ -66180,7 +66180,7 @@
         </is>
       </c>
       <c r="C3653" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3653" t="n">
         <v>201</v>
@@ -66198,7 +66198,7 @@
         </is>
       </c>
       <c r="C3654" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3654" t="n">
         <v>201</v>
@@ -66216,7 +66216,7 @@
         </is>
       </c>
       <c r="C3655" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3655" t="n">
         <v>201</v>
@@ -66225,16 +66225,16 @@
     <row r="3656">
       <c r="A3656" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3656" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3656" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3656" t="n">
         <v>201</v>
@@ -66252,9 +66252,27 @@
         </is>
       </c>
       <c r="C3657" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3657" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3658">
+      <c r="A3658" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3658" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3658" t="n">
         <v>7</v>
       </c>
-      <c r="D3657" t="n">
+      <c r="D3658" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-12 09:56 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3692"/>
+  <dimension ref="A1:D3693"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66135,16 +66135,16 @@
     <row r="3651">
       <c r="A3651" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/12</t>
         </is>
       </c>
       <c r="B3651" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3651" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D3651" t="n">
         <v>201</v>
@@ -66162,7 +66162,7 @@
         </is>
       </c>
       <c r="C3652" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3652" t="n">
         <v>201</v>
@@ -66180,7 +66180,7 @@
         </is>
       </c>
       <c r="C3653" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3653" t="n">
         <v>201</v>
@@ -66198,7 +66198,7 @@
         </is>
       </c>
       <c r="C3654" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3654" t="n">
         <v>201</v>
@@ -66207,16 +66207,16 @@
     <row r="3655">
       <c r="A3655" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3655" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3655" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3655" t="n">
         <v>201</v>
@@ -66234,7 +66234,7 @@
         </is>
       </c>
       <c r="C3656" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3656" t="n">
         <v>201</v>
@@ -66252,7 +66252,7 @@
         </is>
       </c>
       <c r="C3657" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3657" t="n">
         <v>201</v>
@@ -66270,7 +66270,7 @@
         </is>
       </c>
       <c r="C3658" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3658" t="n">
         <v>201</v>
@@ -66288,7 +66288,7 @@
         </is>
       </c>
       <c r="C3659" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3659" t="n">
         <v>201</v>
@@ -66306,7 +66306,7 @@
         </is>
       </c>
       <c r="C3660" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3660" t="n">
         <v>201</v>
@@ -66315,16 +66315,16 @@
     <row r="3661">
       <c r="A3661" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3661" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3661" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3661" t="n">
         <v>201</v>
@@ -66342,7 +66342,7 @@
         </is>
       </c>
       <c r="C3662" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3662" t="n">
         <v>201</v>
@@ -66360,7 +66360,7 @@
         </is>
       </c>
       <c r="C3663" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3663" t="n">
         <v>201</v>
@@ -66378,7 +66378,7 @@
         </is>
       </c>
       <c r="C3664" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3664" t="n">
         <v>201</v>
@@ -66396,7 +66396,7 @@
         </is>
       </c>
       <c r="C3665" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3665" t="n">
         <v>201</v>
@@ -66414,7 +66414,7 @@
         </is>
       </c>
       <c r="C3666" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3666" t="n">
         <v>201</v>
@@ -66423,16 +66423,16 @@
     <row r="3667">
       <c r="A3667" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3667" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3667" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3667" t="n">
         <v>201</v>
@@ -66450,7 +66450,7 @@
         </is>
       </c>
       <c r="C3668" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3668" t="n">
         <v>201</v>
@@ -66468,7 +66468,7 @@
         </is>
       </c>
       <c r="C3669" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3669" t="n">
         <v>201</v>
@@ -66486,7 +66486,7 @@
         </is>
       </c>
       <c r="C3670" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3670" t="n">
         <v>201</v>
@@ -66504,7 +66504,7 @@
         </is>
       </c>
       <c r="C3671" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3671" t="n">
         <v>201</v>
@@ -66513,16 +66513,16 @@
     <row r="3672">
       <c r="A3672" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3672" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3672" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3672" t="n">
         <v>201</v>
@@ -66540,7 +66540,7 @@
         </is>
       </c>
       <c r="C3673" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3673" t="n">
         <v>201</v>
@@ -66558,7 +66558,7 @@
         </is>
       </c>
       <c r="C3674" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3674" t="n">
         <v>201</v>
@@ -66576,7 +66576,7 @@
         </is>
       </c>
       <c r="C3675" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3675" t="n">
         <v>201</v>
@@ -66594,7 +66594,7 @@
         </is>
       </c>
       <c r="C3676" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3676" t="n">
         <v>201</v>
@@ -66612,7 +66612,7 @@
         </is>
       </c>
       <c r="C3677" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3677" t="n">
         <v>201</v>
@@ -66630,7 +66630,7 @@
         </is>
       </c>
       <c r="C3678" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3678" t="n">
         <v>201</v>
@@ -66639,16 +66639,16 @@
     <row r="3679">
       <c r="A3679" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3679" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3679" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3679" t="n">
         <v>201</v>
@@ -66666,7 +66666,7 @@
         </is>
       </c>
       <c r="C3680" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3680" t="n">
         <v>201</v>
@@ -66684,7 +66684,7 @@
         </is>
       </c>
       <c r="C3681" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3681" t="n">
         <v>201</v>
@@ -66702,7 +66702,7 @@
         </is>
       </c>
       <c r="C3682" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3682" t="n">
         <v>201</v>
@@ -66720,7 +66720,7 @@
         </is>
       </c>
       <c r="C3683" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3683" t="n">
         <v>201</v>
@@ -66738,7 +66738,7 @@
         </is>
       </c>
       <c r="C3684" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3684" t="n">
         <v>201</v>
@@ -66756,7 +66756,7 @@
         </is>
       </c>
       <c r="C3685" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3685" t="n">
         <v>201</v>
@@ -66765,16 +66765,16 @@
     <row r="3686">
       <c r="A3686" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3686" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3686" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3686" t="n">
         <v>201</v>
@@ -66792,7 +66792,7 @@
         </is>
       </c>
       <c r="C3687" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3687" t="n">
         <v>201</v>
@@ -66810,7 +66810,7 @@
         </is>
       </c>
       <c r="C3688" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3688" t="n">
         <v>201</v>
@@ -66828,7 +66828,7 @@
         </is>
       </c>
       <c r="C3689" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3689" t="n">
         <v>201</v>
@@ -66846,7 +66846,7 @@
         </is>
       </c>
       <c r="C3690" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3690" t="n">
         <v>201</v>
@@ -66855,16 +66855,16 @@
     <row r="3691">
       <c r="A3691" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3691" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3691" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3691" t="n">
         <v>201</v>
@@ -66882,9 +66882,27 @@
         </is>
       </c>
       <c r="C3692" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3692" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3693">
+      <c r="A3693" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3693" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3693" t="n">
         <v>7</v>
       </c>
-      <c r="D3692" t="n">
+      <c r="D3693" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-05-01 04:14 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3813"/>
+  <dimension ref="A1:D3814"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68313,19 +68313,19 @@
     <row r="3772">
       <c r="A3772" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/05/01</t>
         </is>
       </c>
       <c r="B3772" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3772" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D3772" t="n">
-        <v>201</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3773">
@@ -68340,7 +68340,7 @@
         </is>
       </c>
       <c r="C3773" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3773" t="n">
         <v>201</v>
@@ -68358,7 +68358,7 @@
         </is>
       </c>
       <c r="C3774" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3774" t="n">
         <v>201</v>
@@ -68376,7 +68376,7 @@
         </is>
       </c>
       <c r="C3775" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3775" t="n">
         <v>201</v>
@@ -68385,16 +68385,16 @@
     <row r="3776">
       <c r="A3776" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3776" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3776" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3776" t="n">
         <v>201</v>
@@ -68412,7 +68412,7 @@
         </is>
       </c>
       <c r="C3777" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3777" t="n">
         <v>201</v>
@@ -68430,7 +68430,7 @@
         </is>
       </c>
       <c r="C3778" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3778" t="n">
         <v>201</v>
@@ -68448,7 +68448,7 @@
         </is>
       </c>
       <c r="C3779" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3779" t="n">
         <v>201</v>
@@ -68466,7 +68466,7 @@
         </is>
       </c>
       <c r="C3780" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3780" t="n">
         <v>201</v>
@@ -68484,7 +68484,7 @@
         </is>
       </c>
       <c r="C3781" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3781" t="n">
         <v>201</v>
@@ -68493,16 +68493,16 @@
     <row r="3782">
       <c r="A3782" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3782" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3782" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3782" t="n">
         <v>201</v>
@@ -68520,7 +68520,7 @@
         </is>
       </c>
       <c r="C3783" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3783" t="n">
         <v>201</v>
@@ -68538,7 +68538,7 @@
         </is>
       </c>
       <c r="C3784" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3784" t="n">
         <v>201</v>
@@ -68556,7 +68556,7 @@
         </is>
       </c>
       <c r="C3785" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3785" t="n">
         <v>201</v>
@@ -68574,7 +68574,7 @@
         </is>
       </c>
       <c r="C3786" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3786" t="n">
         <v>201</v>
@@ -68592,7 +68592,7 @@
         </is>
       </c>
       <c r="C3787" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3787" t="n">
         <v>201</v>
@@ -68601,16 +68601,16 @@
     <row r="3788">
       <c r="A3788" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3788" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3788" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3788" t="n">
         <v>201</v>
@@ -68628,7 +68628,7 @@
         </is>
       </c>
       <c r="C3789" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3789" t="n">
         <v>201</v>
@@ -68646,7 +68646,7 @@
         </is>
       </c>
       <c r="C3790" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3790" t="n">
         <v>201</v>
@@ -68664,7 +68664,7 @@
         </is>
       </c>
       <c r="C3791" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3791" t="n">
         <v>201</v>
@@ -68682,7 +68682,7 @@
         </is>
       </c>
       <c r="C3792" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3792" t="n">
         <v>201</v>
@@ -68691,16 +68691,16 @@
     <row r="3793">
       <c r="A3793" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3793" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3793" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3793" t="n">
         <v>201</v>
@@ -68718,7 +68718,7 @@
         </is>
       </c>
       <c r="C3794" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3794" t="n">
         <v>201</v>
@@ -68736,7 +68736,7 @@
         </is>
       </c>
       <c r="C3795" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3795" t="n">
         <v>201</v>
@@ -68754,7 +68754,7 @@
         </is>
       </c>
       <c r="C3796" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3796" t="n">
         <v>201</v>
@@ -68772,7 +68772,7 @@
         </is>
       </c>
       <c r="C3797" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3797" t="n">
         <v>201</v>
@@ -68790,7 +68790,7 @@
         </is>
       </c>
       <c r="C3798" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3798" t="n">
         <v>201</v>
@@ -68808,7 +68808,7 @@
         </is>
       </c>
       <c r="C3799" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3799" t="n">
         <v>201</v>
@@ -68817,16 +68817,16 @@
     <row r="3800">
       <c r="A3800" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3800" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3800" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3800" t="n">
         <v>201</v>
@@ -68844,7 +68844,7 @@
         </is>
       </c>
       <c r="C3801" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3801" t="n">
         <v>201</v>
@@ -68862,7 +68862,7 @@
         </is>
       </c>
       <c r="C3802" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3802" t="n">
         <v>201</v>
@@ -68880,7 +68880,7 @@
         </is>
       </c>
       <c r="C3803" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3803" t="n">
         <v>201</v>
@@ -68898,7 +68898,7 @@
         </is>
       </c>
       <c r="C3804" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3804" t="n">
         <v>201</v>
@@ -68916,7 +68916,7 @@
         </is>
       </c>
       <c r="C3805" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3805" t="n">
         <v>201</v>
@@ -68934,7 +68934,7 @@
         </is>
       </c>
       <c r="C3806" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3806" t="n">
         <v>201</v>
@@ -68943,16 +68943,16 @@
     <row r="3807">
       <c r="A3807" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3807" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3807" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3807" t="n">
         <v>201</v>
@@ -68970,7 +68970,7 @@
         </is>
       </c>
       <c r="C3808" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3808" t="n">
         <v>201</v>
@@ -68988,7 +68988,7 @@
         </is>
       </c>
       <c r="C3809" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3809" t="n">
         <v>201</v>
@@ -69006,7 +69006,7 @@
         </is>
       </c>
       <c r="C3810" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3810" t="n">
         <v>201</v>
@@ -69024,7 +69024,7 @@
         </is>
       </c>
       <c r="C3811" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3811" t="n">
         <v>201</v>
@@ -69033,16 +69033,16 @@
     <row r="3812">
       <c r="A3812" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3812" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3812" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3812" t="n">
         <v>201</v>
@@ -69060,9 +69060,27 @@
         </is>
       </c>
       <c r="C3813" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3813" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3814">
+      <c r="A3814" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3814" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3814" t="n">
         <v>7</v>
       </c>
-      <c r="D3813" t="n">
+      <c r="D3814" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-05-12 05:46 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3887"/>
+  <dimension ref="A1:D3888"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69645,7 +69645,7 @@
     <row r="3846">
       <c r="A3846" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/05/12</t>
         </is>
       </c>
       <c r="B3846" t="inlineStr">
@@ -69654,10 +69654,10 @@
         </is>
       </c>
       <c r="C3846" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3846" t="n">
-        <v>201</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3847">
@@ -69672,7 +69672,7 @@
         </is>
       </c>
       <c r="C3847" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3847" t="n">
         <v>201</v>
@@ -69690,7 +69690,7 @@
         </is>
       </c>
       <c r="C3848" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3848" t="n">
         <v>201</v>
@@ -69708,7 +69708,7 @@
         </is>
       </c>
       <c r="C3849" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3849" t="n">
         <v>201</v>
@@ -69717,16 +69717,16 @@
     <row r="3850">
       <c r="A3850" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3850" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3850" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3850" t="n">
         <v>201</v>
@@ -69744,7 +69744,7 @@
         </is>
       </c>
       <c r="C3851" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3851" t="n">
         <v>201</v>
@@ -69762,7 +69762,7 @@
         </is>
       </c>
       <c r="C3852" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3852" t="n">
         <v>201</v>
@@ -69780,7 +69780,7 @@
         </is>
       </c>
       <c r="C3853" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3853" t="n">
         <v>201</v>
@@ -69798,7 +69798,7 @@
         </is>
       </c>
       <c r="C3854" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3854" t="n">
         <v>201</v>
@@ -69816,7 +69816,7 @@
         </is>
       </c>
       <c r="C3855" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3855" t="n">
         <v>201</v>
@@ -69825,16 +69825,16 @@
     <row r="3856">
       <c r="A3856" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3856" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3856" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3856" t="n">
         <v>201</v>
@@ -69852,7 +69852,7 @@
         </is>
       </c>
       <c r="C3857" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3857" t="n">
         <v>201</v>
@@ -69870,7 +69870,7 @@
         </is>
       </c>
       <c r="C3858" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3858" t="n">
         <v>201</v>
@@ -69888,7 +69888,7 @@
         </is>
       </c>
       <c r="C3859" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3859" t="n">
         <v>201</v>
@@ -69906,7 +69906,7 @@
         </is>
       </c>
       <c r="C3860" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3860" t="n">
         <v>201</v>
@@ -69924,7 +69924,7 @@
         </is>
       </c>
       <c r="C3861" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3861" t="n">
         <v>201</v>
@@ -69933,16 +69933,16 @@
     <row r="3862">
       <c r="A3862" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3862" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3862" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3862" t="n">
         <v>201</v>
@@ -69960,7 +69960,7 @@
         </is>
       </c>
       <c r="C3863" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3863" t="n">
         <v>201</v>
@@ -69978,7 +69978,7 @@
         </is>
       </c>
       <c r="C3864" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3864" t="n">
         <v>201</v>
@@ -69996,7 +69996,7 @@
         </is>
       </c>
       <c r="C3865" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3865" t="n">
         <v>201</v>
@@ -70014,7 +70014,7 @@
         </is>
       </c>
       <c r="C3866" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3866" t="n">
         <v>201</v>
@@ -70023,16 +70023,16 @@
     <row r="3867">
       <c r="A3867" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3867" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3867" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3867" t="n">
         <v>201</v>
@@ -70050,7 +70050,7 @@
         </is>
       </c>
       <c r="C3868" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3868" t="n">
         <v>201</v>
@@ -70068,7 +70068,7 @@
         </is>
       </c>
       <c r="C3869" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3869" t="n">
         <v>201</v>
@@ -70086,7 +70086,7 @@
         </is>
       </c>
       <c r="C3870" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3870" t="n">
         <v>201</v>
@@ -70104,7 +70104,7 @@
         </is>
       </c>
       <c r="C3871" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3871" t="n">
         <v>201</v>
@@ -70122,7 +70122,7 @@
         </is>
       </c>
       <c r="C3872" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3872" t="n">
         <v>201</v>
@@ -70140,7 +70140,7 @@
         </is>
       </c>
       <c r="C3873" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3873" t="n">
         <v>201</v>
@@ -70149,16 +70149,16 @@
     <row r="3874">
       <c r="A3874" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3874" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3874" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3874" t="n">
         <v>201</v>
@@ -70176,7 +70176,7 @@
         </is>
       </c>
       <c r="C3875" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3875" t="n">
         <v>201</v>
@@ -70194,7 +70194,7 @@
         </is>
       </c>
       <c r="C3876" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3876" t="n">
         <v>201</v>
@@ -70212,7 +70212,7 @@
         </is>
       </c>
       <c r="C3877" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3877" t="n">
         <v>201</v>
@@ -70230,7 +70230,7 @@
         </is>
       </c>
       <c r="C3878" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3878" t="n">
         <v>201</v>
@@ -70248,7 +70248,7 @@
         </is>
       </c>
       <c r="C3879" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3879" t="n">
         <v>201</v>
@@ -70266,7 +70266,7 @@
         </is>
       </c>
       <c r="C3880" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3880" t="n">
         <v>201</v>
@@ -70275,16 +70275,16 @@
     <row r="3881">
       <c r="A3881" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3881" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3881" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3881" t="n">
         <v>201</v>
@@ -70302,7 +70302,7 @@
         </is>
       </c>
       <c r="C3882" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3882" t="n">
         <v>201</v>
@@ -70320,7 +70320,7 @@
         </is>
       </c>
       <c r="C3883" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3883" t="n">
         <v>201</v>
@@ -70338,7 +70338,7 @@
         </is>
       </c>
       <c r="C3884" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3884" t="n">
         <v>201</v>
@@ -70356,7 +70356,7 @@
         </is>
       </c>
       <c r="C3885" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3885" t="n">
         <v>201</v>
@@ -70365,16 +70365,16 @@
     <row r="3886">
       <c r="A3886" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3886" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3886" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3886" t="n">
         <v>201</v>
@@ -70392,9 +70392,27 @@
         </is>
       </c>
       <c r="C3887" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3887" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3888">
+      <c r="A3888" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3888" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3888" t="n">
         <v>7</v>
       </c>
-      <c r="D3887" t="n">
+      <c r="D3888" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-05-16 03:59 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3913"/>
+  <dimension ref="A1:D3914"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70113,16 +70113,16 @@
     <row r="3872">
       <c r="A3872" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/05/16</t>
         </is>
       </c>
       <c r="B3872" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3872" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D3872" t="n">
         <v>201</v>
@@ -70140,7 +70140,7 @@
         </is>
       </c>
       <c r="C3873" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3873" t="n">
         <v>201</v>
@@ -70158,7 +70158,7 @@
         </is>
       </c>
       <c r="C3874" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3874" t="n">
         <v>201</v>
@@ -70176,7 +70176,7 @@
         </is>
       </c>
       <c r="C3875" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3875" t="n">
         <v>201</v>
@@ -70185,16 +70185,16 @@
     <row r="3876">
       <c r="A3876" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3876" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3876" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3876" t="n">
         <v>201</v>
@@ -70212,7 +70212,7 @@
         </is>
       </c>
       <c r="C3877" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3877" t="n">
         <v>201</v>
@@ -70230,7 +70230,7 @@
         </is>
       </c>
       <c r="C3878" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3878" t="n">
         <v>201</v>
@@ -70248,7 +70248,7 @@
         </is>
       </c>
       <c r="C3879" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3879" t="n">
         <v>201</v>
@@ -70266,7 +70266,7 @@
         </is>
       </c>
       <c r="C3880" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3880" t="n">
         <v>201</v>
@@ -70284,7 +70284,7 @@
         </is>
       </c>
       <c r="C3881" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3881" t="n">
         <v>201</v>
@@ -70293,16 +70293,16 @@
     <row r="3882">
       <c r="A3882" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3882" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3882" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3882" t="n">
         <v>201</v>
@@ -70320,7 +70320,7 @@
         </is>
       </c>
       <c r="C3883" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3883" t="n">
         <v>201</v>
@@ -70338,7 +70338,7 @@
         </is>
       </c>
       <c r="C3884" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3884" t="n">
         <v>201</v>
@@ -70356,7 +70356,7 @@
         </is>
       </c>
       <c r="C3885" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3885" t="n">
         <v>201</v>
@@ -70374,7 +70374,7 @@
         </is>
       </c>
       <c r="C3886" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3886" t="n">
         <v>201</v>
@@ -70392,7 +70392,7 @@
         </is>
       </c>
       <c r="C3887" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3887" t="n">
         <v>201</v>
@@ -70401,16 +70401,16 @@
     <row r="3888">
       <c r="A3888" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3888" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3888" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3888" t="n">
         <v>201</v>
@@ -70428,7 +70428,7 @@
         </is>
       </c>
       <c r="C3889" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3889" t="n">
         <v>201</v>
@@ -70446,7 +70446,7 @@
         </is>
       </c>
       <c r="C3890" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3890" t="n">
         <v>201</v>
@@ -70464,7 +70464,7 @@
         </is>
       </c>
       <c r="C3891" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3891" t="n">
         <v>201</v>
@@ -70482,7 +70482,7 @@
         </is>
       </c>
       <c r="C3892" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3892" t="n">
         <v>201</v>
@@ -70491,16 +70491,16 @@
     <row r="3893">
       <c r="A3893" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3893" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3893" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3893" t="n">
         <v>201</v>
@@ -70518,7 +70518,7 @@
         </is>
       </c>
       <c r="C3894" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3894" t="n">
         <v>201</v>
@@ -70536,7 +70536,7 @@
         </is>
       </c>
       <c r="C3895" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3895" t="n">
         <v>201</v>
@@ -70554,7 +70554,7 @@
         </is>
       </c>
       <c r="C3896" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3896" t="n">
         <v>201</v>
@@ -70572,7 +70572,7 @@
         </is>
       </c>
       <c r="C3897" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3897" t="n">
         <v>201</v>
@@ -70590,7 +70590,7 @@
         </is>
       </c>
       <c r="C3898" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3898" t="n">
         <v>201</v>
@@ -70608,7 +70608,7 @@
         </is>
       </c>
       <c r="C3899" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3899" t="n">
         <v>201</v>
@@ -70617,16 +70617,16 @@
     <row r="3900">
       <c r="A3900" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3900" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3900" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3900" t="n">
         <v>201</v>
@@ -70644,7 +70644,7 @@
         </is>
       </c>
       <c r="C3901" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3901" t="n">
         <v>201</v>
@@ -70662,7 +70662,7 @@
         </is>
       </c>
       <c r="C3902" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3902" t="n">
         <v>201</v>
@@ -70680,7 +70680,7 @@
         </is>
       </c>
       <c r="C3903" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3903" t="n">
         <v>201</v>
@@ -70698,7 +70698,7 @@
         </is>
       </c>
       <c r="C3904" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3904" t="n">
         <v>201</v>
@@ -70716,7 +70716,7 @@
         </is>
       </c>
       <c r="C3905" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3905" t="n">
         <v>201</v>
@@ -70734,7 +70734,7 @@
         </is>
       </c>
       <c r="C3906" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3906" t="n">
         <v>201</v>
@@ -70743,16 +70743,16 @@
     <row r="3907">
       <c r="A3907" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3907" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3907" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3907" t="n">
         <v>201</v>
@@ -70770,7 +70770,7 @@
         </is>
       </c>
       <c r="C3908" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3908" t="n">
         <v>201</v>
@@ -70788,7 +70788,7 @@
         </is>
       </c>
       <c r="C3909" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3909" t="n">
         <v>201</v>
@@ -70806,7 +70806,7 @@
         </is>
       </c>
       <c r="C3910" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3910" t="n">
         <v>201</v>
@@ -70824,7 +70824,7 @@
         </is>
       </c>
       <c r="C3911" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3911" t="n">
         <v>201</v>
@@ -70833,16 +70833,16 @@
     <row r="3912">
       <c r="A3912" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3912" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3912" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3912" t="n">
         <v>201</v>
@@ -70860,9 +70860,27 @@
         </is>
       </c>
       <c r="C3913" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3913" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3914">
+      <c r="A3914" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3914" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3914" t="n">
         <v>7</v>
       </c>
-      <c r="D3913" t="n">
+      <c r="D3914" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-06-05 04:44 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4037"/>
+  <dimension ref="A1:D4038"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72345,16 +72345,16 @@
     <row r="3996">
       <c r="A3996" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/06/05</t>
         </is>
       </c>
       <c r="B3996" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3996" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D3996" t="n">
         <v>201</v>
@@ -72372,7 +72372,7 @@
         </is>
       </c>
       <c r="C3997" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3997" t="n">
         <v>201</v>
@@ -72390,7 +72390,7 @@
         </is>
       </c>
       <c r="C3998" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3998" t="n">
         <v>201</v>
@@ -72408,7 +72408,7 @@
         </is>
       </c>
       <c r="C3999" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3999" t="n">
         <v>201</v>
@@ -72417,16 +72417,16 @@
     <row r="4000">
       <c r="A4000" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4000" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4000" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4000" t="n">
         <v>201</v>
@@ -72444,7 +72444,7 @@
         </is>
       </c>
       <c r="C4001" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4001" t="n">
         <v>201</v>
@@ -72462,7 +72462,7 @@
         </is>
       </c>
       <c r="C4002" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4002" t="n">
         <v>201</v>
@@ -72480,7 +72480,7 @@
         </is>
       </c>
       <c r="C4003" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4003" t="n">
         <v>201</v>
@@ -72498,7 +72498,7 @@
         </is>
       </c>
       <c r="C4004" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4004" t="n">
         <v>201</v>
@@ -72516,7 +72516,7 @@
         </is>
       </c>
       <c r="C4005" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4005" t="n">
         <v>201</v>
@@ -72525,16 +72525,16 @@
     <row r="4006">
       <c r="A4006" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4006" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4006" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4006" t="n">
         <v>201</v>
@@ -72552,7 +72552,7 @@
         </is>
       </c>
       <c r="C4007" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4007" t="n">
         <v>201</v>
@@ -72570,7 +72570,7 @@
         </is>
       </c>
       <c r="C4008" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4008" t="n">
         <v>201</v>
@@ -72588,7 +72588,7 @@
         </is>
       </c>
       <c r="C4009" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4009" t="n">
         <v>201</v>
@@ -72606,7 +72606,7 @@
         </is>
       </c>
       <c r="C4010" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4010" t="n">
         <v>201</v>
@@ -72624,7 +72624,7 @@
         </is>
       </c>
       <c r="C4011" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4011" t="n">
         <v>201</v>
@@ -72633,16 +72633,16 @@
     <row r="4012">
       <c r="A4012" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4012" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4012" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4012" t="n">
         <v>201</v>
@@ -72660,7 +72660,7 @@
         </is>
       </c>
       <c r="C4013" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4013" t="n">
         <v>201</v>
@@ -72678,7 +72678,7 @@
         </is>
       </c>
       <c r="C4014" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4014" t="n">
         <v>201</v>
@@ -72696,7 +72696,7 @@
         </is>
       </c>
       <c r="C4015" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4015" t="n">
         <v>201</v>
@@ -72714,7 +72714,7 @@
         </is>
       </c>
       <c r="C4016" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4016" t="n">
         <v>201</v>
@@ -72723,16 +72723,16 @@
     <row r="4017">
       <c r="A4017" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4017" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4017" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4017" t="n">
         <v>201</v>
@@ -72750,7 +72750,7 @@
         </is>
       </c>
       <c r="C4018" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4018" t="n">
         <v>201</v>
@@ -72768,7 +72768,7 @@
         </is>
       </c>
       <c r="C4019" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4019" t="n">
         <v>201</v>
@@ -72786,7 +72786,7 @@
         </is>
       </c>
       <c r="C4020" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4020" t="n">
         <v>201</v>
@@ -72804,7 +72804,7 @@
         </is>
       </c>
       <c r="C4021" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4021" t="n">
         <v>201</v>
@@ -72822,7 +72822,7 @@
         </is>
       </c>
       <c r="C4022" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4022" t="n">
         <v>201</v>
@@ -72840,7 +72840,7 @@
         </is>
       </c>
       <c r="C4023" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4023" t="n">
         <v>201</v>
@@ -72849,16 +72849,16 @@
     <row r="4024">
       <c r="A4024" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4024" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4024" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4024" t="n">
         <v>201</v>
@@ -72876,7 +72876,7 @@
         </is>
       </c>
       <c r="C4025" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4025" t="n">
         <v>201</v>
@@ -72894,7 +72894,7 @@
         </is>
       </c>
       <c r="C4026" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4026" t="n">
         <v>201</v>
@@ -72912,7 +72912,7 @@
         </is>
       </c>
       <c r="C4027" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4027" t="n">
         <v>201</v>
@@ -72930,7 +72930,7 @@
         </is>
       </c>
       <c r="C4028" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4028" t="n">
         <v>201</v>
@@ -72948,7 +72948,7 @@
         </is>
       </c>
       <c r="C4029" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4029" t="n">
         <v>201</v>
@@ -72966,7 +72966,7 @@
         </is>
       </c>
       <c r="C4030" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4030" t="n">
         <v>201</v>
@@ -72975,16 +72975,16 @@
     <row r="4031">
       <c r="A4031" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4031" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4031" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4031" t="n">
         <v>201</v>
@@ -73002,7 +73002,7 @@
         </is>
       </c>
       <c r="C4032" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4032" t="n">
         <v>201</v>
@@ -73020,7 +73020,7 @@
         </is>
       </c>
       <c r="C4033" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4033" t="n">
         <v>201</v>
@@ -73038,7 +73038,7 @@
         </is>
       </c>
       <c r="C4034" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4034" t="n">
         <v>201</v>
@@ -73056,7 +73056,7 @@
         </is>
       </c>
       <c r="C4035" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4035" t="n">
         <v>201</v>
@@ -73065,16 +73065,16 @@
     <row r="4036">
       <c r="A4036" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4036" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4036" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4036" t="n">
         <v>201</v>
@@ -73092,9 +73092,27 @@
         </is>
       </c>
       <c r="C4037" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4037" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4038">
+      <c r="A4038" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4038" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4038" t="n">
         <v>7</v>
       </c>
-      <c r="D4037" t="n">
+      <c r="D4038" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-06-20 04:39 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4133"/>
+  <dimension ref="A1:D4134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74073,16 +74073,16 @@
     <row r="4092">
       <c r="A4092" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/06/20</t>
         </is>
       </c>
       <c r="B4092" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4092" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D4092" t="n">
         <v>201</v>
@@ -74100,7 +74100,7 @@
         </is>
       </c>
       <c r="C4093" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4093" t="n">
         <v>201</v>
@@ -74118,7 +74118,7 @@
         </is>
       </c>
       <c r="C4094" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4094" t="n">
         <v>201</v>
@@ -74136,7 +74136,7 @@
         </is>
       </c>
       <c r="C4095" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4095" t="n">
         <v>201</v>
@@ -74145,16 +74145,16 @@
     <row r="4096">
       <c r="A4096" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4096" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4096" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4096" t="n">
         <v>201</v>
@@ -74172,7 +74172,7 @@
         </is>
       </c>
       <c r="C4097" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4097" t="n">
         <v>201</v>
@@ -74190,7 +74190,7 @@
         </is>
       </c>
       <c r="C4098" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4098" t="n">
         <v>201</v>
@@ -74208,7 +74208,7 @@
         </is>
       </c>
       <c r="C4099" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4099" t="n">
         <v>201</v>
@@ -74226,7 +74226,7 @@
         </is>
       </c>
       <c r="C4100" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4100" t="n">
         <v>201</v>
@@ -74244,7 +74244,7 @@
         </is>
       </c>
       <c r="C4101" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4101" t="n">
         <v>201</v>
@@ -74253,16 +74253,16 @@
     <row r="4102">
       <c r="A4102" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4102" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4102" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4102" t="n">
         <v>201</v>
@@ -74280,7 +74280,7 @@
         </is>
       </c>
       <c r="C4103" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4103" t="n">
         <v>201</v>
@@ -74298,7 +74298,7 @@
         </is>
       </c>
       <c r="C4104" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4104" t="n">
         <v>201</v>
@@ -74316,7 +74316,7 @@
         </is>
       </c>
       <c r="C4105" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4105" t="n">
         <v>201</v>
@@ -74334,7 +74334,7 @@
         </is>
       </c>
       <c r="C4106" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4106" t="n">
         <v>201</v>
@@ -74352,7 +74352,7 @@
         </is>
       </c>
       <c r="C4107" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4107" t="n">
         <v>201</v>
@@ -74361,16 +74361,16 @@
     <row r="4108">
       <c r="A4108" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4108" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4108" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4108" t="n">
         <v>201</v>
@@ -74388,7 +74388,7 @@
         </is>
       </c>
       <c r="C4109" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4109" t="n">
         <v>201</v>
@@ -74406,7 +74406,7 @@
         </is>
       </c>
       <c r="C4110" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4110" t="n">
         <v>201</v>
@@ -74424,7 +74424,7 @@
         </is>
       </c>
       <c r="C4111" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4111" t="n">
         <v>201</v>
@@ -74442,7 +74442,7 @@
         </is>
       </c>
       <c r="C4112" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4112" t="n">
         <v>201</v>
@@ -74451,16 +74451,16 @@
     <row r="4113">
       <c r="A4113" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4113" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4113" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4113" t="n">
         <v>201</v>
@@ -74478,7 +74478,7 @@
         </is>
       </c>
       <c r="C4114" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4114" t="n">
         <v>201</v>
@@ -74496,7 +74496,7 @@
         </is>
       </c>
       <c r="C4115" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4115" t="n">
         <v>201</v>
@@ -74514,7 +74514,7 @@
         </is>
       </c>
       <c r="C4116" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4116" t="n">
         <v>201</v>
@@ -74532,7 +74532,7 @@
         </is>
       </c>
       <c r="C4117" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4117" t="n">
         <v>201</v>
@@ -74550,7 +74550,7 @@
         </is>
       </c>
       <c r="C4118" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4118" t="n">
         <v>201</v>
@@ -74568,7 +74568,7 @@
         </is>
       </c>
       <c r="C4119" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4119" t="n">
         <v>201</v>
@@ -74577,16 +74577,16 @@
     <row r="4120">
       <c r="A4120" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4120" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4120" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4120" t="n">
         <v>201</v>
@@ -74604,7 +74604,7 @@
         </is>
       </c>
       <c r="C4121" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4121" t="n">
         <v>201</v>
@@ -74622,7 +74622,7 @@
         </is>
       </c>
       <c r="C4122" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4122" t="n">
         <v>201</v>
@@ -74640,7 +74640,7 @@
         </is>
       </c>
       <c r="C4123" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4123" t="n">
         <v>201</v>
@@ -74658,7 +74658,7 @@
         </is>
       </c>
       <c r="C4124" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4124" t="n">
         <v>201</v>
@@ -74676,7 +74676,7 @@
         </is>
       </c>
       <c r="C4125" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4125" t="n">
         <v>201</v>
@@ -74694,7 +74694,7 @@
         </is>
       </c>
       <c r="C4126" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4126" t="n">
         <v>201</v>
@@ -74703,16 +74703,16 @@
     <row r="4127">
       <c r="A4127" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4127" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4127" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4127" t="n">
         <v>201</v>
@@ -74730,7 +74730,7 @@
         </is>
       </c>
       <c r="C4128" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4128" t="n">
         <v>201</v>
@@ -74748,7 +74748,7 @@
         </is>
       </c>
       <c r="C4129" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4129" t="n">
         <v>201</v>
@@ -74766,7 +74766,7 @@
         </is>
       </c>
       <c r="C4130" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4130" t="n">
         <v>201</v>
@@ -74784,7 +74784,7 @@
         </is>
       </c>
       <c r="C4131" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4131" t="n">
         <v>201</v>
@@ -74793,16 +74793,16 @@
     <row r="4132">
       <c r="A4132" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4132" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4132" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4132" t="n">
         <v>201</v>
@@ -74820,9 +74820,27 @@
         </is>
       </c>
       <c r="C4133" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4133" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4134">
+      <c r="A4134" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4134" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4134" t="n">
         <v>7</v>
       </c>
-      <c r="D4133" t="n">
+      <c r="D4134" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-06-22 07:35 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4162"/>
+  <dimension ref="A1:D4164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74595,16 +74595,16 @@
     <row r="4121">
       <c r="A4121" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/06/22</t>
         </is>
       </c>
       <c r="B4121" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4121" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4121" t="n">
         <v>201</v>
@@ -74613,12 +74613,12 @@
     <row r="4122">
       <c r="A4122" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/06/22</t>
         </is>
       </c>
       <c r="B4122" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4122" t="n">
@@ -74640,7 +74640,7 @@
         </is>
       </c>
       <c r="C4123" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D4123" t="n">
         <v>201</v>
@@ -74658,7 +74658,7 @@
         </is>
       </c>
       <c r="C4124" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D4124" t="n">
         <v>201</v>
@@ -74667,16 +74667,16 @@
     <row r="4125">
       <c r="A4125" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4125" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4125" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D4125" t="n">
         <v>201</v>
@@ -74685,16 +74685,16 @@
     <row r="4126">
       <c r="A4126" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4126" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4126" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="D4126" t="n">
         <v>201</v>
@@ -74712,7 +74712,7 @@
         </is>
       </c>
       <c r="C4127" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D4127" t="n">
         <v>201</v>
@@ -74730,7 +74730,7 @@
         </is>
       </c>
       <c r="C4128" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4128" t="n">
         <v>201</v>
@@ -74748,7 +74748,7 @@
         </is>
       </c>
       <c r="C4129" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D4129" t="n">
         <v>201</v>
@@ -74766,7 +74766,7 @@
         </is>
       </c>
       <c r="C4130" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4130" t="n">
         <v>201</v>
@@ -74775,16 +74775,16 @@
     <row r="4131">
       <c r="A4131" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4131" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4131" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D4131" t="n">
         <v>201</v>
@@ -74793,16 +74793,16 @@
     <row r="4132">
       <c r="A4132" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4132" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4132" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D4132" t="n">
         <v>201</v>
@@ -74820,7 +74820,7 @@
         </is>
       </c>
       <c r="C4133" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D4133" t="n">
         <v>201</v>
@@ -74838,7 +74838,7 @@
         </is>
       </c>
       <c r="C4134" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D4134" t="n">
         <v>201</v>
@@ -74856,7 +74856,7 @@
         </is>
       </c>
       <c r="C4135" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D4135" t="n">
         <v>201</v>
@@ -74874,7 +74874,7 @@
         </is>
       </c>
       <c r="C4136" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D4136" t="n">
         <v>201</v>
@@ -74883,16 +74883,16 @@
     <row r="4137">
       <c r="A4137" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4137" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4137" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D4137" t="n">
         <v>201</v>
@@ -74901,16 +74901,16 @@
     <row r="4138">
       <c r="A4138" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4138" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4138" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="D4138" t="n">
         <v>201</v>
@@ -74928,7 +74928,7 @@
         </is>
       </c>
       <c r="C4139" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D4139" t="n">
         <v>201</v>
@@ -74946,7 +74946,7 @@
         </is>
       </c>
       <c r="C4140" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D4140" t="n">
         <v>201</v>
@@ -74964,7 +74964,7 @@
         </is>
       </c>
       <c r="C4141" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D4141" t="n">
         <v>201</v>
@@ -74973,16 +74973,16 @@
     <row r="4142">
       <c r="A4142" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4142" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4142" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D4142" t="n">
         <v>201</v>
@@ -74991,16 +74991,16 @@
     <row r="4143">
       <c r="A4143" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4143" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4143" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="D4143" t="n">
         <v>201</v>
@@ -75018,7 +75018,7 @@
         </is>
       </c>
       <c r="C4144" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D4144" t="n">
         <v>201</v>
@@ -75036,7 +75036,7 @@
         </is>
       </c>
       <c r="C4145" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4145" t="n">
         <v>201</v>
@@ -75054,7 +75054,7 @@
         </is>
       </c>
       <c r="C4146" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D4146" t="n">
         <v>201</v>
@@ -75072,7 +75072,7 @@
         </is>
       </c>
       <c r="C4147" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D4147" t="n">
         <v>201</v>
@@ -75090,7 +75090,7 @@
         </is>
       </c>
       <c r="C4148" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4148" t="n">
         <v>201</v>
@@ -75099,16 +75099,16 @@
     <row r="4149">
       <c r="A4149" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4149" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4149" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4149" t="n">
         <v>201</v>
@@ -75117,16 +75117,16 @@
     <row r="4150">
       <c r="A4150" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4150" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4150" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D4150" t="n">
         <v>201</v>
@@ -75144,7 +75144,7 @@
         </is>
       </c>
       <c r="C4151" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D4151" t="n">
         <v>201</v>
@@ -75162,7 +75162,7 @@
         </is>
       </c>
       <c r="C4152" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D4152" t="n">
         <v>201</v>
@@ -75180,7 +75180,7 @@
         </is>
       </c>
       <c r="C4153" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D4153" t="n">
         <v>201</v>
@@ -75198,7 +75198,7 @@
         </is>
       </c>
       <c r="C4154" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D4154" t="n">
         <v>201</v>
@@ -75216,7 +75216,7 @@
         </is>
       </c>
       <c r="C4155" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4155" t="n">
         <v>201</v>
@@ -75225,16 +75225,16 @@
     <row r="4156">
       <c r="A4156" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4156" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4156" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D4156" t="n">
         <v>201</v>
@@ -75243,16 +75243,16 @@
     <row r="4157">
       <c r="A4157" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4157" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4157" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D4157" t="n">
         <v>201</v>
@@ -75270,7 +75270,7 @@
         </is>
       </c>
       <c r="C4158" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D4158" t="n">
         <v>201</v>
@@ -75288,7 +75288,7 @@
         </is>
       </c>
       <c r="C4159" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D4159" t="n">
         <v>201</v>
@@ -75306,7 +75306,7 @@
         </is>
       </c>
       <c r="C4160" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D4160" t="n">
         <v>201</v>
@@ -75315,16 +75315,16 @@
     <row r="4161">
       <c r="A4161" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4161" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4161" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D4161" t="n">
         <v>201</v>
@@ -75333,18 +75333,54 @@
     <row r="4162">
       <c r="A4162" t="inlineStr">
         <is>
+          <t>2027/01/04</t>
+        </is>
+      </c>
+      <c r="B4162" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C4162" t="n">
+        <v>22</v>
+      </c>
+      <c r="D4162" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4163">
+      <c r="A4163" t="inlineStr">
+        <is>
           <t>2027/01/05</t>
         </is>
       </c>
-      <c r="B4162" t="inlineStr">
+      <c r="B4163" t="inlineStr">
         <is>
           <t>火</t>
         </is>
       </c>
-      <c r="C4162" t="n">
+      <c r="C4163" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4163" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4164">
+      <c r="A4164" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4164" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4164" t="n">
         <v>7</v>
       </c>
-      <c r="D4162" t="n">
+      <c r="D4164" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-06-22 13:01 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4169"/>
+  <dimension ref="A1:D4170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74721,16 +74721,16 @@
     <row r="4128">
       <c r="A4128" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/06/22</t>
         </is>
       </c>
       <c r="B4128" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4128" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D4128" t="n">
         <v>201</v>
@@ -74748,7 +74748,7 @@
         </is>
       </c>
       <c r="C4129" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4129" t="n">
         <v>201</v>
@@ -74766,7 +74766,7 @@
         </is>
       </c>
       <c r="C4130" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4130" t="n">
         <v>201</v>
@@ -74784,7 +74784,7 @@
         </is>
       </c>
       <c r="C4131" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4131" t="n">
         <v>201</v>
@@ -74793,16 +74793,16 @@
     <row r="4132">
       <c r="A4132" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4132" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4132" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4132" t="n">
         <v>201</v>
@@ -74820,7 +74820,7 @@
         </is>
       </c>
       <c r="C4133" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4133" t="n">
         <v>201</v>
@@ -74838,7 +74838,7 @@
         </is>
       </c>
       <c r="C4134" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4134" t="n">
         <v>201</v>
@@ -74856,7 +74856,7 @@
         </is>
       </c>
       <c r="C4135" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4135" t="n">
         <v>201</v>
@@ -74874,7 +74874,7 @@
         </is>
       </c>
       <c r="C4136" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4136" t="n">
         <v>201</v>
@@ -74892,7 +74892,7 @@
         </is>
       </c>
       <c r="C4137" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4137" t="n">
         <v>201</v>
@@ -74901,16 +74901,16 @@
     <row r="4138">
       <c r="A4138" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4138" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4138" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4138" t="n">
         <v>201</v>
@@ -74928,7 +74928,7 @@
         </is>
       </c>
       <c r="C4139" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4139" t="n">
         <v>201</v>
@@ -74946,7 +74946,7 @@
         </is>
       </c>
       <c r="C4140" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4140" t="n">
         <v>201</v>
@@ -74964,7 +74964,7 @@
         </is>
       </c>
       <c r="C4141" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4141" t="n">
         <v>201</v>
@@ -74982,7 +74982,7 @@
         </is>
       </c>
       <c r="C4142" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4142" t="n">
         <v>201</v>
@@ -75000,7 +75000,7 @@
         </is>
       </c>
       <c r="C4143" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4143" t="n">
         <v>201</v>
@@ -75009,16 +75009,16 @@
     <row r="4144">
       <c r="A4144" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4144" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4144" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4144" t="n">
         <v>201</v>
@@ -75036,7 +75036,7 @@
         </is>
       </c>
       <c r="C4145" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4145" t="n">
         <v>201</v>
@@ -75054,7 +75054,7 @@
         </is>
       </c>
       <c r="C4146" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4146" t="n">
         <v>201</v>
@@ -75072,7 +75072,7 @@
         </is>
       </c>
       <c r="C4147" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4147" t="n">
         <v>201</v>
@@ -75090,7 +75090,7 @@
         </is>
       </c>
       <c r="C4148" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4148" t="n">
         <v>201</v>
@@ -75099,16 +75099,16 @@
     <row r="4149">
       <c r="A4149" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4149" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4149" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4149" t="n">
         <v>201</v>
@@ -75126,7 +75126,7 @@
         </is>
       </c>
       <c r="C4150" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4150" t="n">
         <v>201</v>
@@ -75144,7 +75144,7 @@
         </is>
       </c>
       <c r="C4151" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4151" t="n">
         <v>201</v>
@@ -75162,7 +75162,7 @@
         </is>
       </c>
       <c r="C4152" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4152" t="n">
         <v>201</v>
@@ -75180,7 +75180,7 @@
         </is>
       </c>
       <c r="C4153" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4153" t="n">
         <v>201</v>
@@ -75198,7 +75198,7 @@
         </is>
       </c>
       <c r="C4154" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4154" t="n">
         <v>201</v>
@@ -75216,7 +75216,7 @@
         </is>
       </c>
       <c r="C4155" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4155" t="n">
         <v>201</v>
@@ -75225,16 +75225,16 @@
     <row r="4156">
       <c r="A4156" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4156" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4156" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4156" t="n">
         <v>201</v>
@@ -75252,7 +75252,7 @@
         </is>
       </c>
       <c r="C4157" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4157" t="n">
         <v>201</v>
@@ -75270,7 +75270,7 @@
         </is>
       </c>
       <c r="C4158" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4158" t="n">
         <v>201</v>
@@ -75288,7 +75288,7 @@
         </is>
       </c>
       <c r="C4159" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4159" t="n">
         <v>201</v>
@@ -75306,7 +75306,7 @@
         </is>
       </c>
       <c r="C4160" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4160" t="n">
         <v>201</v>
@@ -75324,7 +75324,7 @@
         </is>
       </c>
       <c r="C4161" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4161" t="n">
         <v>201</v>
@@ -75342,7 +75342,7 @@
         </is>
       </c>
       <c r="C4162" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4162" t="n">
         <v>201</v>
@@ -75351,16 +75351,16 @@
     <row r="4163">
       <c r="A4163" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4163" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4163" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4163" t="n">
         <v>201</v>
@@ -75378,7 +75378,7 @@
         </is>
       </c>
       <c r="C4164" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4164" t="n">
         <v>201</v>
@@ -75396,7 +75396,7 @@
         </is>
       </c>
       <c r="C4165" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4165" t="n">
         <v>201</v>
@@ -75414,7 +75414,7 @@
         </is>
       </c>
       <c r="C4166" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4166" t="n">
         <v>201</v>
@@ -75432,7 +75432,7 @@
         </is>
       </c>
       <c r="C4167" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4167" t="n">
         <v>201</v>
@@ -75441,16 +75441,16 @@
     <row r="4168">
       <c r="A4168" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4168" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4168" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4168" t="n">
         <v>201</v>
@@ -75468,9 +75468,27 @@
         </is>
       </c>
       <c r="C4169" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4169" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4170">
+      <c r="A4170" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4170" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4170" t="n">
         <v>7</v>
       </c>
-      <c r="D4169" t="n">
+      <c r="D4170" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-06-29 12:06 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4259"/>
+  <dimension ref="A1:D4260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76341,16 +76341,16 @@
     <row r="4218">
       <c r="A4218" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="B4218" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4218" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D4218" t="n">
         <v>201</v>
@@ -76368,7 +76368,7 @@
         </is>
       </c>
       <c r="C4219" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4219" t="n">
         <v>201</v>
@@ -76386,7 +76386,7 @@
         </is>
       </c>
       <c r="C4220" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4220" t="n">
         <v>201</v>
@@ -76404,7 +76404,7 @@
         </is>
       </c>
       <c r="C4221" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4221" t="n">
         <v>201</v>
@@ -76413,16 +76413,16 @@
     <row r="4222">
       <c r="A4222" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4222" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4222" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4222" t="n">
         <v>201</v>
@@ -76440,7 +76440,7 @@
         </is>
       </c>
       <c r="C4223" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4223" t="n">
         <v>201</v>
@@ -76458,7 +76458,7 @@
         </is>
       </c>
       <c r="C4224" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4224" t="n">
         <v>201</v>
@@ -76476,7 +76476,7 @@
         </is>
       </c>
       <c r="C4225" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4225" t="n">
         <v>201</v>
@@ -76494,7 +76494,7 @@
         </is>
       </c>
       <c r="C4226" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4226" t="n">
         <v>201</v>
@@ -76512,7 +76512,7 @@
         </is>
       </c>
       <c r="C4227" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4227" t="n">
         <v>201</v>
@@ -76521,16 +76521,16 @@
     <row r="4228">
       <c r="A4228" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4228" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4228" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4228" t="n">
         <v>201</v>
@@ -76548,7 +76548,7 @@
         </is>
       </c>
       <c r="C4229" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4229" t="n">
         <v>201</v>
@@ -76566,7 +76566,7 @@
         </is>
       </c>
       <c r="C4230" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4230" t="n">
         <v>201</v>
@@ -76584,7 +76584,7 @@
         </is>
       </c>
       <c r="C4231" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4231" t="n">
         <v>201</v>
@@ -76602,7 +76602,7 @@
         </is>
       </c>
       <c r="C4232" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4232" t="n">
         <v>201</v>
@@ -76620,7 +76620,7 @@
         </is>
       </c>
       <c r="C4233" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4233" t="n">
         <v>201</v>
@@ -76629,16 +76629,16 @@
     <row r="4234">
       <c r="A4234" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4234" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4234" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4234" t="n">
         <v>201</v>
@@ -76656,7 +76656,7 @@
         </is>
       </c>
       <c r="C4235" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4235" t="n">
         <v>201</v>
@@ -76674,7 +76674,7 @@
         </is>
       </c>
       <c r="C4236" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4236" t="n">
         <v>201</v>
@@ -76692,7 +76692,7 @@
         </is>
       </c>
       <c r="C4237" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4237" t="n">
         <v>201</v>
@@ -76710,7 +76710,7 @@
         </is>
       </c>
       <c r="C4238" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4238" t="n">
         <v>201</v>
@@ -76719,16 +76719,16 @@
     <row r="4239">
       <c r="A4239" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4239" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4239" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4239" t="n">
         <v>201</v>
@@ -76746,7 +76746,7 @@
         </is>
       </c>
       <c r="C4240" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4240" t="n">
         <v>201</v>
@@ -76764,7 +76764,7 @@
         </is>
       </c>
       <c r="C4241" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4241" t="n">
         <v>201</v>
@@ -76782,7 +76782,7 @@
         </is>
       </c>
       <c r="C4242" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4242" t="n">
         <v>201</v>
@@ -76800,7 +76800,7 @@
         </is>
       </c>
       <c r="C4243" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4243" t="n">
         <v>201</v>
@@ -76818,7 +76818,7 @@
         </is>
       </c>
       <c r="C4244" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4244" t="n">
         <v>201</v>
@@ -76836,7 +76836,7 @@
         </is>
       </c>
       <c r="C4245" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4245" t="n">
         <v>201</v>
@@ -76845,16 +76845,16 @@
     <row r="4246">
       <c r="A4246" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4246" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4246" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4246" t="n">
         <v>201</v>
@@ -76872,7 +76872,7 @@
         </is>
       </c>
       <c r="C4247" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4247" t="n">
         <v>201</v>
@@ -76890,7 +76890,7 @@
         </is>
       </c>
       <c r="C4248" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4248" t="n">
         <v>201</v>
@@ -76908,7 +76908,7 @@
         </is>
       </c>
       <c r="C4249" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4249" t="n">
         <v>201</v>
@@ -76926,7 +76926,7 @@
         </is>
       </c>
       <c r="C4250" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4250" t="n">
         <v>201</v>
@@ -76944,7 +76944,7 @@
         </is>
       </c>
       <c r="C4251" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4251" t="n">
         <v>201</v>
@@ -76962,7 +76962,7 @@
         </is>
       </c>
       <c r="C4252" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4252" t="n">
         <v>201</v>
@@ -76971,16 +76971,16 @@
     <row r="4253">
       <c r="A4253" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4253" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4253" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4253" t="n">
         <v>201</v>
@@ -76998,7 +76998,7 @@
         </is>
       </c>
       <c r="C4254" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4254" t="n">
         <v>201</v>
@@ -77016,7 +77016,7 @@
         </is>
       </c>
       <c r="C4255" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4255" t="n">
         <v>201</v>
@@ -77034,7 +77034,7 @@
         </is>
       </c>
       <c r="C4256" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4256" t="n">
         <v>201</v>
@@ -77052,7 +77052,7 @@
         </is>
       </c>
       <c r="C4257" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4257" t="n">
         <v>201</v>
@@ -77061,16 +77061,16 @@
     <row r="4258">
       <c r="A4258" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4258" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4258" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4258" t="n">
         <v>201</v>
@@ -77088,9 +77088,27 @@
         </is>
       </c>
       <c r="C4259" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4259" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4260">
+      <c r="A4260" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4260" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4260" t="n">
         <v>7</v>
       </c>
-      <c r="D4259" t="n">
+      <c r="D4260" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-06-29 13:14 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4260"/>
+  <dimension ref="A1:D4261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76359,16 +76359,16 @@
     <row r="4219">
       <c r="A4219" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="B4219" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4219" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D4219" t="n">
         <v>201</v>
@@ -76386,7 +76386,7 @@
         </is>
       </c>
       <c r="C4220" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4220" t="n">
         <v>201</v>
@@ -76404,7 +76404,7 @@
         </is>
       </c>
       <c r="C4221" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4221" t="n">
         <v>201</v>
@@ -76422,7 +76422,7 @@
         </is>
       </c>
       <c r="C4222" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4222" t="n">
         <v>201</v>
@@ -76431,16 +76431,16 @@
     <row r="4223">
       <c r="A4223" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4223" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4223" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4223" t="n">
         <v>201</v>
@@ -76458,7 +76458,7 @@
         </is>
       </c>
       <c r="C4224" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4224" t="n">
         <v>201</v>
@@ -76476,7 +76476,7 @@
         </is>
       </c>
       <c r="C4225" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4225" t="n">
         <v>201</v>
@@ -76494,7 +76494,7 @@
         </is>
       </c>
       <c r="C4226" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4226" t="n">
         <v>201</v>
@@ -76512,7 +76512,7 @@
         </is>
       </c>
       <c r="C4227" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4227" t="n">
         <v>201</v>
@@ -76530,7 +76530,7 @@
         </is>
       </c>
       <c r="C4228" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4228" t="n">
         <v>201</v>
@@ -76539,16 +76539,16 @@
     <row r="4229">
       <c r="A4229" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4229" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4229" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4229" t="n">
         <v>201</v>
@@ -76566,7 +76566,7 @@
         </is>
       </c>
       <c r="C4230" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4230" t="n">
         <v>201</v>
@@ -76584,7 +76584,7 @@
         </is>
       </c>
       <c r="C4231" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4231" t="n">
         <v>201</v>
@@ -76602,7 +76602,7 @@
         </is>
       </c>
       <c r="C4232" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4232" t="n">
         <v>201</v>
@@ -76620,7 +76620,7 @@
         </is>
       </c>
       <c r="C4233" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4233" t="n">
         <v>201</v>
@@ -76638,7 +76638,7 @@
         </is>
       </c>
       <c r="C4234" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4234" t="n">
         <v>201</v>
@@ -76647,16 +76647,16 @@
     <row r="4235">
       <c r="A4235" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4235" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4235" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4235" t="n">
         <v>201</v>
@@ -76674,7 +76674,7 @@
         </is>
       </c>
       <c r="C4236" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4236" t="n">
         <v>201</v>
@@ -76692,7 +76692,7 @@
         </is>
       </c>
       <c r="C4237" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4237" t="n">
         <v>201</v>
@@ -76710,7 +76710,7 @@
         </is>
       </c>
       <c r="C4238" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4238" t="n">
         <v>201</v>
@@ -76728,7 +76728,7 @@
         </is>
       </c>
       <c r="C4239" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4239" t="n">
         <v>201</v>
@@ -76737,16 +76737,16 @@
     <row r="4240">
       <c r="A4240" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4240" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4240" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4240" t="n">
         <v>201</v>
@@ -76764,7 +76764,7 @@
         </is>
       </c>
       <c r="C4241" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4241" t="n">
         <v>201</v>
@@ -76782,7 +76782,7 @@
         </is>
       </c>
       <c r="C4242" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4242" t="n">
         <v>201</v>
@@ -76800,7 +76800,7 @@
         </is>
       </c>
       <c r="C4243" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4243" t="n">
         <v>201</v>
@@ -76818,7 +76818,7 @@
         </is>
       </c>
       <c r="C4244" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4244" t="n">
         <v>201</v>
@@ -76836,7 +76836,7 @@
         </is>
       </c>
       <c r="C4245" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4245" t="n">
         <v>201</v>
@@ -76854,7 +76854,7 @@
         </is>
       </c>
       <c r="C4246" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4246" t="n">
         <v>201</v>
@@ -76863,16 +76863,16 @@
     <row r="4247">
       <c r="A4247" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4247" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4247" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4247" t="n">
         <v>201</v>
@@ -76890,7 +76890,7 @@
         </is>
       </c>
       <c r="C4248" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4248" t="n">
         <v>201</v>
@@ -76908,7 +76908,7 @@
         </is>
       </c>
       <c r="C4249" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4249" t="n">
         <v>201</v>
@@ -76926,7 +76926,7 @@
         </is>
       </c>
       <c r="C4250" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4250" t="n">
         <v>201</v>
@@ -76944,7 +76944,7 @@
         </is>
       </c>
       <c r="C4251" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4251" t="n">
         <v>201</v>
@@ -76962,7 +76962,7 @@
         </is>
       </c>
       <c r="C4252" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4252" t="n">
         <v>201</v>
@@ -76980,7 +76980,7 @@
         </is>
       </c>
       <c r="C4253" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4253" t="n">
         <v>201</v>
@@ -76989,16 +76989,16 @@
     <row r="4254">
       <c r="A4254" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4254" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4254" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4254" t="n">
         <v>201</v>
@@ -77016,7 +77016,7 @@
         </is>
       </c>
       <c r="C4255" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4255" t="n">
         <v>201</v>
@@ -77034,7 +77034,7 @@
         </is>
       </c>
       <c r="C4256" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4256" t="n">
         <v>201</v>
@@ -77052,7 +77052,7 @@
         </is>
       </c>
       <c r="C4257" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4257" t="n">
         <v>201</v>
@@ -77070,7 +77070,7 @@
         </is>
       </c>
       <c r="C4258" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4258" t="n">
         <v>201</v>
@@ -77079,16 +77079,16 @@
     <row r="4259">
       <c r="A4259" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4259" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4259" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4259" t="n">
         <v>201</v>
@@ -77106,9 +77106,27 @@
         </is>
       </c>
       <c r="C4260" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4260" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4261">
+      <c r="A4261" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4261" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4261" t="n">
         <v>7</v>
       </c>
-      <c r="D4260" t="n">
+      <c r="D4261" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-12 03:53 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4524"/>
+  <dimension ref="A1:D4528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81111,16 +81111,16 @@
     <row r="4483">
       <c r="A4483" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/12</t>
         </is>
       </c>
       <c r="B4483" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4483" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D4483" t="n">
         <v>201</v>
@@ -81129,16 +81129,16 @@
     <row r="4484">
       <c r="A4484" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/12</t>
         </is>
       </c>
       <c r="B4484" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4484" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D4484" t="n">
         <v>201</v>
@@ -81147,16 +81147,16 @@
     <row r="4485">
       <c r="A4485" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/12</t>
         </is>
       </c>
       <c r="B4485" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4485" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D4485" t="n">
         <v>201</v>
@@ -81165,16 +81165,16 @@
     <row r="4486">
       <c r="A4486" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/12</t>
         </is>
       </c>
       <c r="B4486" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4486" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D4486" t="n">
         <v>201</v>
@@ -81183,16 +81183,16 @@
     <row r="4487">
       <c r="A4487" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4487" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4487" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D4487" t="n">
         <v>201</v>
@@ -81201,16 +81201,16 @@
     <row r="4488">
       <c r="A4488" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4488" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4488" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D4488" t="n">
         <v>201</v>
@@ -81219,16 +81219,16 @@
     <row r="4489">
       <c r="A4489" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4489" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4489" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D4489" t="n">
         <v>201</v>
@@ -81237,16 +81237,16 @@
     <row r="4490">
       <c r="A4490" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4490" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4490" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D4490" t="n">
         <v>201</v>
@@ -81264,7 +81264,7 @@
         </is>
       </c>
       <c r="C4491" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="D4491" t="n">
         <v>201</v>
@@ -81282,7 +81282,7 @@
         </is>
       </c>
       <c r="C4492" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="D4492" t="n">
         <v>201</v>
@@ -81291,16 +81291,16 @@
     <row r="4493">
       <c r="A4493" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4493" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4493" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D4493" t="n">
         <v>201</v>
@@ -81309,16 +81309,16 @@
     <row r="4494">
       <c r="A4494" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4494" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4494" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D4494" t="n">
         <v>201</v>
@@ -81327,16 +81327,16 @@
     <row r="4495">
       <c r="A4495" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4495" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4495" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D4495" t="n">
         <v>201</v>
@@ -81345,16 +81345,16 @@
     <row r="4496">
       <c r="A4496" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4496" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4496" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D4496" t="n">
         <v>201</v>
@@ -81372,7 +81372,7 @@
         </is>
       </c>
       <c r="C4497" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D4497" t="n">
         <v>201</v>
@@ -81390,7 +81390,7 @@
         </is>
       </c>
       <c r="C4498" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="D4498" t="n">
         <v>201</v>
@@ -81399,16 +81399,16 @@
     <row r="4499">
       <c r="A4499" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4499" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4499" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D4499" t="n">
         <v>201</v>
@@ -81417,16 +81417,16 @@
     <row r="4500">
       <c r="A4500" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4500" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4500" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D4500" t="n">
         <v>201</v>
@@ -81435,16 +81435,16 @@
     <row r="4501">
       <c r="A4501" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4501" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4501" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4501" t="n">
         <v>201</v>
@@ -81453,16 +81453,16 @@
     <row r="4502">
       <c r="A4502" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4502" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4502" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D4502" t="n">
         <v>201</v>
@@ -81480,7 +81480,7 @@
         </is>
       </c>
       <c r="C4503" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D4503" t="n">
         <v>201</v>
@@ -81489,16 +81489,16 @@
     <row r="4504">
       <c r="A4504" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4504" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4504" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D4504" t="n">
         <v>201</v>
@@ -81507,16 +81507,16 @@
     <row r="4505">
       <c r="A4505" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4505" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4505" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D4505" t="n">
         <v>201</v>
@@ -81525,16 +81525,16 @@
     <row r="4506">
       <c r="A4506" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4506" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4506" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D4506" t="n">
         <v>201</v>
@@ -81543,16 +81543,16 @@
     <row r="4507">
       <c r="A4507" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4507" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4507" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D4507" t="n">
         <v>201</v>
@@ -81570,7 +81570,7 @@
         </is>
       </c>
       <c r="C4508" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D4508" t="n">
         <v>201</v>
@@ -81588,7 +81588,7 @@
         </is>
       </c>
       <c r="C4509" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="D4509" t="n">
         <v>201</v>
@@ -81606,7 +81606,7 @@
         </is>
       </c>
       <c r="C4510" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D4510" t="n">
         <v>201</v>
@@ -81615,16 +81615,16 @@
     <row r="4511">
       <c r="A4511" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4511" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4511" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D4511" t="n">
         <v>201</v>
@@ -81633,16 +81633,16 @@
     <row r="4512">
       <c r="A4512" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4512" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4512" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D4512" t="n">
         <v>201</v>
@@ -81651,16 +81651,16 @@
     <row r="4513">
       <c r="A4513" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4513" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4513" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D4513" t="n">
         <v>201</v>
@@ -81669,16 +81669,16 @@
     <row r="4514">
       <c r="A4514" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4514" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4514" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D4514" t="n">
         <v>201</v>
@@ -81696,7 +81696,7 @@
         </is>
       </c>
       <c r="C4515" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D4515" t="n">
         <v>201</v>
@@ -81714,7 +81714,7 @@
         </is>
       </c>
       <c r="C4516" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D4516" t="n">
         <v>201</v>
@@ -81732,7 +81732,7 @@
         </is>
       </c>
       <c r="C4517" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D4517" t="n">
         <v>201</v>
@@ -81741,16 +81741,16 @@
     <row r="4518">
       <c r="A4518" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4518" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4518" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D4518" t="n">
         <v>201</v>
@@ -81759,16 +81759,16 @@
     <row r="4519">
       <c r="A4519" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4519" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4519" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D4519" t="n">
         <v>201</v>
@@ -81777,16 +81777,16 @@
     <row r="4520">
       <c r="A4520" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4520" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4520" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D4520" t="n">
         <v>201</v>
@@ -81795,16 +81795,16 @@
     <row r="4521">
       <c r="A4521" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4521" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4521" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D4521" t="n">
         <v>201</v>
@@ -81822,7 +81822,7 @@
         </is>
       </c>
       <c r="C4522" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D4522" t="n">
         <v>201</v>
@@ -81831,16 +81831,16 @@
     <row r="4523">
       <c r="A4523" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4523" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4523" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D4523" t="n">
         <v>201</v>
@@ -81849,18 +81849,90 @@
     <row r="4524">
       <c r="A4524" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4524" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4524" t="n">
         <v>7</v>
       </c>
       <c r="D4524" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4525">
+      <c r="A4525" t="inlineStr">
+        <is>
+          <t>2027/01/04</t>
+        </is>
+      </c>
+      <c r="B4525" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C4525" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4525" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4526">
+      <c r="A4526" t="inlineStr">
+        <is>
+          <t>2027/01/04</t>
+        </is>
+      </c>
+      <c r="B4526" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C4526" t="n">
+        <v>22</v>
+      </c>
+      <c r="D4526" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4527">
+      <c r="A4527" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4527" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4527" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4527" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4528">
+      <c r="A4528" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4528" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4528" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4528" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-12 06:11 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4530"/>
+  <dimension ref="A1:D4531"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81219,16 +81219,16 @@
     <row r="4489">
       <c r="A4489" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/12</t>
         </is>
       </c>
       <c r="B4489" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4489" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4489" t="n">
         <v>201</v>
@@ -81246,7 +81246,7 @@
         </is>
       </c>
       <c r="C4490" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4490" t="n">
         <v>201</v>
@@ -81264,7 +81264,7 @@
         </is>
       </c>
       <c r="C4491" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4491" t="n">
         <v>201</v>
@@ -81282,7 +81282,7 @@
         </is>
       </c>
       <c r="C4492" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4492" t="n">
         <v>201</v>
@@ -81291,16 +81291,16 @@
     <row r="4493">
       <c r="A4493" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4493" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4493" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4493" t="n">
         <v>201</v>
@@ -81318,7 +81318,7 @@
         </is>
       </c>
       <c r="C4494" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4494" t="n">
         <v>201</v>
@@ -81336,7 +81336,7 @@
         </is>
       </c>
       <c r="C4495" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4495" t="n">
         <v>201</v>
@@ -81354,7 +81354,7 @@
         </is>
       </c>
       <c r="C4496" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4496" t="n">
         <v>201</v>
@@ -81372,7 +81372,7 @@
         </is>
       </c>
       <c r="C4497" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4497" t="n">
         <v>201</v>
@@ -81390,7 +81390,7 @@
         </is>
       </c>
       <c r="C4498" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4498" t="n">
         <v>201</v>
@@ -81399,16 +81399,16 @@
     <row r="4499">
       <c r="A4499" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4499" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4499" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4499" t="n">
         <v>201</v>
@@ -81426,7 +81426,7 @@
         </is>
       </c>
       <c r="C4500" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4500" t="n">
         <v>201</v>
@@ -81444,7 +81444,7 @@
         </is>
       </c>
       <c r="C4501" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4501" t="n">
         <v>201</v>
@@ -81462,7 +81462,7 @@
         </is>
       </c>
       <c r="C4502" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4502" t="n">
         <v>201</v>
@@ -81480,7 +81480,7 @@
         </is>
       </c>
       <c r="C4503" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4503" t="n">
         <v>201</v>
@@ -81498,7 +81498,7 @@
         </is>
       </c>
       <c r="C4504" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4504" t="n">
         <v>201</v>
@@ -81507,16 +81507,16 @@
     <row r="4505">
       <c r="A4505" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4505" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4505" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4505" t="n">
         <v>201</v>
@@ -81534,7 +81534,7 @@
         </is>
       </c>
       <c r="C4506" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4506" t="n">
         <v>201</v>
@@ -81552,7 +81552,7 @@
         </is>
       </c>
       <c r="C4507" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4507" t="n">
         <v>201</v>
@@ -81570,7 +81570,7 @@
         </is>
       </c>
       <c r="C4508" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4508" t="n">
         <v>201</v>
@@ -81588,7 +81588,7 @@
         </is>
       </c>
       <c r="C4509" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4509" t="n">
         <v>201</v>
@@ -81597,16 +81597,16 @@
     <row r="4510">
       <c r="A4510" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4510" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4510" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4510" t="n">
         <v>201</v>
@@ -81624,7 +81624,7 @@
         </is>
       </c>
       <c r="C4511" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4511" t="n">
         <v>201</v>
@@ -81642,7 +81642,7 @@
         </is>
       </c>
       <c r="C4512" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4512" t="n">
         <v>201</v>
@@ -81660,7 +81660,7 @@
         </is>
       </c>
       <c r="C4513" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4513" t="n">
         <v>201</v>
@@ -81678,7 +81678,7 @@
         </is>
       </c>
       <c r="C4514" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4514" t="n">
         <v>201</v>
@@ -81696,7 +81696,7 @@
         </is>
       </c>
       <c r="C4515" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4515" t="n">
         <v>201</v>
@@ -81714,7 +81714,7 @@
         </is>
       </c>
       <c r="C4516" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4516" t="n">
         <v>201</v>
@@ -81723,16 +81723,16 @@
     <row r="4517">
       <c r="A4517" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4517" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4517" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4517" t="n">
         <v>201</v>
@@ -81750,7 +81750,7 @@
         </is>
       </c>
       <c r="C4518" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4518" t="n">
         <v>201</v>
@@ -81768,7 +81768,7 @@
         </is>
       </c>
       <c r="C4519" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4519" t="n">
         <v>201</v>
@@ -81786,7 +81786,7 @@
         </is>
       </c>
       <c r="C4520" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4520" t="n">
         <v>201</v>
@@ -81804,7 +81804,7 @@
         </is>
       </c>
       <c r="C4521" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4521" t="n">
         <v>201</v>
@@ -81822,7 +81822,7 @@
         </is>
       </c>
       <c r="C4522" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4522" t="n">
         <v>201</v>
@@ -81840,7 +81840,7 @@
         </is>
       </c>
       <c r="C4523" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4523" t="n">
         <v>201</v>
@@ -81849,16 +81849,16 @@
     <row r="4524">
       <c r="A4524" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4524" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4524" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4524" t="n">
         <v>201</v>
@@ -81876,7 +81876,7 @@
         </is>
       </c>
       <c r="C4525" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4525" t="n">
         <v>201</v>
@@ -81894,7 +81894,7 @@
         </is>
       </c>
       <c r="C4526" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4526" t="n">
         <v>201</v>
@@ -81912,7 +81912,7 @@
         </is>
       </c>
       <c r="C4527" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4527" t="n">
         <v>201</v>
@@ -81930,7 +81930,7 @@
         </is>
       </c>
       <c r="C4528" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4528" t="n">
         <v>201</v>
@@ -81939,16 +81939,16 @@
     <row r="4529">
       <c r="A4529" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4529" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4529" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4529" t="n">
         <v>201</v>
@@ -81966,9 +81966,27 @@
         </is>
       </c>
       <c r="C4530" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4530" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4531">
+      <c r="A4531" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4531" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4531" t="n">
         <v>7</v>
       </c>
-      <c r="D4530" t="n">
+      <c r="D4531" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-12 09:10 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4533"/>
+  <dimension ref="A1:D4534"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81273,16 +81273,16 @@
     <row r="4492">
       <c r="A4492" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/12</t>
         </is>
       </c>
       <c r="B4492" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4492" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D4492" t="n">
         <v>201</v>
@@ -81300,7 +81300,7 @@
         </is>
       </c>
       <c r="C4493" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4493" t="n">
         <v>201</v>
@@ -81318,7 +81318,7 @@
         </is>
       </c>
       <c r="C4494" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4494" t="n">
         <v>201</v>
@@ -81336,7 +81336,7 @@
         </is>
       </c>
       <c r="C4495" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4495" t="n">
         <v>201</v>
@@ -81345,16 +81345,16 @@
     <row r="4496">
       <c r="A4496" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4496" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4496" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4496" t="n">
         <v>201</v>
@@ -81372,7 +81372,7 @@
         </is>
       </c>
       <c r="C4497" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4497" t="n">
         <v>201</v>
@@ -81390,7 +81390,7 @@
         </is>
       </c>
       <c r="C4498" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4498" t="n">
         <v>201</v>
@@ -81408,7 +81408,7 @@
         </is>
       </c>
       <c r="C4499" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4499" t="n">
         <v>201</v>
@@ -81426,7 +81426,7 @@
         </is>
       </c>
       <c r="C4500" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4500" t="n">
         <v>201</v>
@@ -81444,7 +81444,7 @@
         </is>
       </c>
       <c r="C4501" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4501" t="n">
         <v>201</v>
@@ -81453,16 +81453,16 @@
     <row r="4502">
       <c r="A4502" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4502" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4502" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4502" t="n">
         <v>201</v>
@@ -81480,7 +81480,7 @@
         </is>
       </c>
       <c r="C4503" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4503" t="n">
         <v>201</v>
@@ -81498,7 +81498,7 @@
         </is>
       </c>
       <c r="C4504" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4504" t="n">
         <v>201</v>
@@ -81516,7 +81516,7 @@
         </is>
       </c>
       <c r="C4505" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4505" t="n">
         <v>201</v>
@@ -81534,7 +81534,7 @@
         </is>
       </c>
       <c r="C4506" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4506" t="n">
         <v>201</v>
@@ -81552,7 +81552,7 @@
         </is>
       </c>
       <c r="C4507" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4507" t="n">
         <v>201</v>
@@ -81561,16 +81561,16 @@
     <row r="4508">
       <c r="A4508" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4508" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4508" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4508" t="n">
         <v>201</v>
@@ -81588,7 +81588,7 @@
         </is>
       </c>
       <c r="C4509" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4509" t="n">
         <v>201</v>
@@ -81606,7 +81606,7 @@
         </is>
       </c>
       <c r="C4510" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4510" t="n">
         <v>201</v>
@@ -81624,7 +81624,7 @@
         </is>
       </c>
       <c r="C4511" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4511" t="n">
         <v>201</v>
@@ -81642,7 +81642,7 @@
         </is>
       </c>
       <c r="C4512" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4512" t="n">
         <v>201</v>
@@ -81651,16 +81651,16 @@
     <row r="4513">
       <c r="A4513" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4513" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4513" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4513" t="n">
         <v>201</v>
@@ -81678,7 +81678,7 @@
         </is>
       </c>
       <c r="C4514" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4514" t="n">
         <v>201</v>
@@ -81696,7 +81696,7 @@
         </is>
       </c>
       <c r="C4515" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4515" t="n">
         <v>201</v>
@@ -81714,7 +81714,7 @@
         </is>
       </c>
       <c r="C4516" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4516" t="n">
         <v>201</v>
@@ -81732,7 +81732,7 @@
         </is>
       </c>
       <c r="C4517" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4517" t="n">
         <v>201</v>
@@ -81750,7 +81750,7 @@
         </is>
       </c>
       <c r="C4518" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4518" t="n">
         <v>201</v>
@@ -81768,7 +81768,7 @@
         </is>
       </c>
       <c r="C4519" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4519" t="n">
         <v>201</v>
@@ -81777,16 +81777,16 @@
     <row r="4520">
       <c r="A4520" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4520" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4520" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4520" t="n">
         <v>201</v>
@@ -81804,7 +81804,7 @@
         </is>
       </c>
       <c r="C4521" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4521" t="n">
         <v>201</v>
@@ -81822,7 +81822,7 @@
         </is>
       </c>
       <c r="C4522" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4522" t="n">
         <v>201</v>
@@ -81840,7 +81840,7 @@
         </is>
       </c>
       <c r="C4523" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4523" t="n">
         <v>201</v>
@@ -81858,7 +81858,7 @@
         </is>
       </c>
       <c r="C4524" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4524" t="n">
         <v>201</v>
@@ -81876,7 +81876,7 @@
         </is>
       </c>
       <c r="C4525" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4525" t="n">
         <v>201</v>
@@ -81894,7 +81894,7 @@
         </is>
       </c>
       <c r="C4526" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4526" t="n">
         <v>201</v>
@@ -81903,16 +81903,16 @@
     <row r="4527">
       <c r="A4527" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4527" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4527" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4527" t="n">
         <v>201</v>
@@ -81930,7 +81930,7 @@
         </is>
       </c>
       <c r="C4528" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4528" t="n">
         <v>201</v>
@@ -81948,7 +81948,7 @@
         </is>
       </c>
       <c r="C4529" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4529" t="n">
         <v>201</v>
@@ -81966,7 +81966,7 @@
         </is>
       </c>
       <c r="C4530" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4530" t="n">
         <v>201</v>
@@ -81984,7 +81984,7 @@
         </is>
       </c>
       <c r="C4531" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4531" t="n">
         <v>201</v>
@@ -81993,16 +81993,16 @@
     <row r="4532">
       <c r="A4532" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4532" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4532" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4532" t="n">
         <v>201</v>
@@ -82020,9 +82020,27 @@
         </is>
       </c>
       <c r="C4533" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4533" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4534">
+      <c r="A4534" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4534" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4534" t="n">
         <v>7</v>
       </c>
-      <c r="D4533" t="n">
+      <c r="D4534" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-13 12:15 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4553"/>
+  <dimension ref="A1:D4554"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81633,16 +81633,16 @@
     <row r="4512">
       <c r="A4512" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/13</t>
         </is>
       </c>
       <c r="B4512" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4512" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D4512" t="n">
         <v>201</v>
@@ -81660,7 +81660,7 @@
         </is>
       </c>
       <c r="C4513" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4513" t="n">
         <v>201</v>
@@ -81678,7 +81678,7 @@
         </is>
       </c>
       <c r="C4514" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4514" t="n">
         <v>201</v>
@@ -81696,7 +81696,7 @@
         </is>
       </c>
       <c r="C4515" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4515" t="n">
         <v>201</v>
@@ -81705,16 +81705,16 @@
     <row r="4516">
       <c r="A4516" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4516" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4516" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4516" t="n">
         <v>201</v>
@@ -81732,7 +81732,7 @@
         </is>
       </c>
       <c r="C4517" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4517" t="n">
         <v>201</v>
@@ -81750,7 +81750,7 @@
         </is>
       </c>
       <c r="C4518" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4518" t="n">
         <v>201</v>
@@ -81768,7 +81768,7 @@
         </is>
       </c>
       <c r="C4519" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4519" t="n">
         <v>201</v>
@@ -81786,7 +81786,7 @@
         </is>
       </c>
       <c r="C4520" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4520" t="n">
         <v>201</v>
@@ -81804,7 +81804,7 @@
         </is>
       </c>
       <c r="C4521" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4521" t="n">
         <v>201</v>
@@ -81813,16 +81813,16 @@
     <row r="4522">
       <c r="A4522" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4522" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4522" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4522" t="n">
         <v>201</v>
@@ -81840,7 +81840,7 @@
         </is>
       </c>
       <c r="C4523" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4523" t="n">
         <v>201</v>
@@ -81858,7 +81858,7 @@
         </is>
       </c>
       <c r="C4524" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4524" t="n">
         <v>201</v>
@@ -81876,7 +81876,7 @@
         </is>
       </c>
       <c r="C4525" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4525" t="n">
         <v>201</v>
@@ -81894,7 +81894,7 @@
         </is>
       </c>
       <c r="C4526" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4526" t="n">
         <v>201</v>
@@ -81912,7 +81912,7 @@
         </is>
       </c>
       <c r="C4527" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4527" t="n">
         <v>201</v>
@@ -81921,16 +81921,16 @@
     <row r="4528">
       <c r="A4528" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4528" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4528" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4528" t="n">
         <v>201</v>
@@ -81948,7 +81948,7 @@
         </is>
       </c>
       <c r="C4529" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4529" t="n">
         <v>201</v>
@@ -81966,7 +81966,7 @@
         </is>
       </c>
       <c r="C4530" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4530" t="n">
         <v>201</v>
@@ -81984,7 +81984,7 @@
         </is>
       </c>
       <c r="C4531" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4531" t="n">
         <v>201</v>
@@ -82002,7 +82002,7 @@
         </is>
       </c>
       <c r="C4532" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4532" t="n">
         <v>201</v>
@@ -82011,16 +82011,16 @@
     <row r="4533">
       <c r="A4533" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4533" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4533" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4533" t="n">
         <v>201</v>
@@ -82038,7 +82038,7 @@
         </is>
       </c>
       <c r="C4534" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4534" t="n">
         <v>201</v>
@@ -82056,7 +82056,7 @@
         </is>
       </c>
       <c r="C4535" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4535" t="n">
         <v>201</v>
@@ -82074,7 +82074,7 @@
         </is>
       </c>
       <c r="C4536" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4536" t="n">
         <v>201</v>
@@ -82092,7 +82092,7 @@
         </is>
       </c>
       <c r="C4537" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4537" t="n">
         <v>201</v>
@@ -82110,7 +82110,7 @@
         </is>
       </c>
       <c r="C4538" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4538" t="n">
         <v>201</v>
@@ -82128,7 +82128,7 @@
         </is>
       </c>
       <c r="C4539" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4539" t="n">
         <v>201</v>
@@ -82137,16 +82137,16 @@
     <row r="4540">
       <c r="A4540" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4540" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4540" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4540" t="n">
         <v>201</v>
@@ -82164,7 +82164,7 @@
         </is>
       </c>
       <c r="C4541" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4541" t="n">
         <v>201</v>
@@ -82182,7 +82182,7 @@
         </is>
       </c>
       <c r="C4542" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4542" t="n">
         <v>201</v>
@@ -82200,7 +82200,7 @@
         </is>
       </c>
       <c r="C4543" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4543" t="n">
         <v>201</v>
@@ -82218,7 +82218,7 @@
         </is>
       </c>
       <c r="C4544" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4544" t="n">
         <v>201</v>
@@ -82236,7 +82236,7 @@
         </is>
       </c>
       <c r="C4545" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4545" t="n">
         <v>201</v>
@@ -82254,7 +82254,7 @@
         </is>
       </c>
       <c r="C4546" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4546" t="n">
         <v>201</v>
@@ -82263,16 +82263,16 @@
     <row r="4547">
       <c r="A4547" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4547" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4547" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4547" t="n">
         <v>201</v>
@@ -82290,7 +82290,7 @@
         </is>
       </c>
       <c r="C4548" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4548" t="n">
         <v>201</v>
@@ -82308,7 +82308,7 @@
         </is>
       </c>
       <c r="C4549" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4549" t="n">
         <v>201</v>
@@ -82326,7 +82326,7 @@
         </is>
       </c>
       <c r="C4550" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4550" t="n">
         <v>201</v>
@@ -82344,7 +82344,7 @@
         </is>
       </c>
       <c r="C4551" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4551" t="n">
         <v>201</v>
@@ -82353,16 +82353,16 @@
     <row r="4552">
       <c r="A4552" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4552" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4552" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4552" t="n">
         <v>201</v>
@@ -82380,9 +82380,27 @@
         </is>
       </c>
       <c r="C4553" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4553" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4554">
+      <c r="A4554" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4554" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4554" t="n">
         <v>7</v>
       </c>
-      <c r="D4553" t="n">
+      <c r="D4554" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-17 03:33 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4577"/>
+  <dimension ref="A1:D4578"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82065,16 +82065,16 @@
     <row r="4536">
       <c r="A4536" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/17</t>
         </is>
       </c>
       <c r="B4536" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4536" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D4536" t="n">
         <v>201</v>
@@ -82092,7 +82092,7 @@
         </is>
       </c>
       <c r="C4537" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4537" t="n">
         <v>201</v>
@@ -82110,7 +82110,7 @@
         </is>
       </c>
       <c r="C4538" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4538" t="n">
         <v>201</v>
@@ -82128,7 +82128,7 @@
         </is>
       </c>
       <c r="C4539" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4539" t="n">
         <v>201</v>
@@ -82137,16 +82137,16 @@
     <row r="4540">
       <c r="A4540" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4540" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4540" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4540" t="n">
         <v>201</v>
@@ -82164,7 +82164,7 @@
         </is>
       </c>
       <c r="C4541" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4541" t="n">
         <v>201</v>
@@ -82182,7 +82182,7 @@
         </is>
       </c>
       <c r="C4542" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4542" t="n">
         <v>201</v>
@@ -82200,7 +82200,7 @@
         </is>
       </c>
       <c r="C4543" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4543" t="n">
         <v>201</v>
@@ -82218,7 +82218,7 @@
         </is>
       </c>
       <c r="C4544" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4544" t="n">
         <v>201</v>
@@ -82236,7 +82236,7 @@
         </is>
       </c>
       <c r="C4545" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4545" t="n">
         <v>201</v>
@@ -82245,16 +82245,16 @@
     <row r="4546">
       <c r="A4546" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4546" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4546" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4546" t="n">
         <v>201</v>
@@ -82272,7 +82272,7 @@
         </is>
       </c>
       <c r="C4547" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4547" t="n">
         <v>201</v>
@@ -82290,7 +82290,7 @@
         </is>
       </c>
       <c r="C4548" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4548" t="n">
         <v>201</v>
@@ -82308,7 +82308,7 @@
         </is>
       </c>
       <c r="C4549" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4549" t="n">
         <v>201</v>
@@ -82326,7 +82326,7 @@
         </is>
       </c>
       <c r="C4550" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4550" t="n">
         <v>201</v>
@@ -82344,7 +82344,7 @@
         </is>
       </c>
       <c r="C4551" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4551" t="n">
         <v>201</v>
@@ -82353,16 +82353,16 @@
     <row r="4552">
       <c r="A4552" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4552" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4552" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4552" t="n">
         <v>201</v>
@@ -82380,7 +82380,7 @@
         </is>
       </c>
       <c r="C4553" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4553" t="n">
         <v>201</v>
@@ -82398,7 +82398,7 @@
         </is>
       </c>
       <c r="C4554" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4554" t="n">
         <v>201</v>
@@ -82416,7 +82416,7 @@
         </is>
       </c>
       <c r="C4555" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4555" t="n">
         <v>201</v>
@@ -82434,7 +82434,7 @@
         </is>
       </c>
       <c r="C4556" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4556" t="n">
         <v>201</v>
@@ -82443,16 +82443,16 @@
     <row r="4557">
       <c r="A4557" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4557" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4557" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4557" t="n">
         <v>201</v>
@@ -82470,7 +82470,7 @@
         </is>
       </c>
       <c r="C4558" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4558" t="n">
         <v>201</v>
@@ -82488,7 +82488,7 @@
         </is>
       </c>
       <c r="C4559" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4559" t="n">
         <v>201</v>
@@ -82506,7 +82506,7 @@
         </is>
       </c>
       <c r="C4560" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4560" t="n">
         <v>201</v>
@@ -82524,7 +82524,7 @@
         </is>
       </c>
       <c r="C4561" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4561" t="n">
         <v>201</v>
@@ -82542,7 +82542,7 @@
         </is>
       </c>
       <c r="C4562" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4562" t="n">
         <v>201</v>
@@ -82560,7 +82560,7 @@
         </is>
       </c>
       <c r="C4563" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4563" t="n">
         <v>201</v>
@@ -82569,16 +82569,16 @@
     <row r="4564">
       <c r="A4564" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4564" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4564" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4564" t="n">
         <v>201</v>
@@ -82596,7 +82596,7 @@
         </is>
       </c>
       <c r="C4565" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4565" t="n">
         <v>201</v>
@@ -82614,7 +82614,7 @@
         </is>
       </c>
       <c r="C4566" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4566" t="n">
         <v>201</v>
@@ -82632,7 +82632,7 @@
         </is>
       </c>
       <c r="C4567" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4567" t="n">
         <v>201</v>
@@ -82650,7 +82650,7 @@
         </is>
       </c>
       <c r="C4568" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4568" t="n">
         <v>201</v>
@@ -82668,7 +82668,7 @@
         </is>
       </c>
       <c r="C4569" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4569" t="n">
         <v>201</v>
@@ -82686,7 +82686,7 @@
         </is>
       </c>
       <c r="C4570" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4570" t="n">
         <v>201</v>
@@ -82695,16 +82695,16 @@
     <row r="4571">
       <c r="A4571" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4571" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4571" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4571" t="n">
         <v>201</v>
@@ -82722,7 +82722,7 @@
         </is>
       </c>
       <c r="C4572" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4572" t="n">
         <v>201</v>
@@ -82740,7 +82740,7 @@
         </is>
       </c>
       <c r="C4573" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4573" t="n">
         <v>201</v>
@@ -82758,7 +82758,7 @@
         </is>
       </c>
       <c r="C4574" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4574" t="n">
         <v>201</v>
@@ -82776,7 +82776,7 @@
         </is>
       </c>
       <c r="C4575" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4575" t="n">
         <v>201</v>
@@ -82785,16 +82785,16 @@
     <row r="4576">
       <c r="A4576" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4576" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4576" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4576" t="n">
         <v>201</v>
@@ -82812,9 +82812,27 @@
         </is>
       </c>
       <c r="C4577" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4577" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4578">
+      <c r="A4578" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4578" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4578" t="n">
         <v>7</v>
       </c>
-      <c r="D4577" t="n">
+      <c r="D4578" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-18 03:28 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4584"/>
+  <dimension ref="A1:D4585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82191,16 +82191,16 @@
     <row r="4543">
       <c r="A4543" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/18</t>
         </is>
       </c>
       <c r="B4543" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4543" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D4543" t="n">
         <v>201</v>
@@ -82218,7 +82218,7 @@
         </is>
       </c>
       <c r="C4544" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4544" t="n">
         <v>201</v>
@@ -82236,7 +82236,7 @@
         </is>
       </c>
       <c r="C4545" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4545" t="n">
         <v>201</v>
@@ -82254,7 +82254,7 @@
         </is>
       </c>
       <c r="C4546" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4546" t="n">
         <v>201</v>
@@ -82263,16 +82263,16 @@
     <row r="4547">
       <c r="A4547" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4547" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4547" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4547" t="n">
         <v>201</v>
@@ -82290,7 +82290,7 @@
         </is>
       </c>
       <c r="C4548" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4548" t="n">
         <v>201</v>
@@ -82308,7 +82308,7 @@
         </is>
       </c>
       <c r="C4549" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4549" t="n">
         <v>201</v>
@@ -82326,7 +82326,7 @@
         </is>
       </c>
       <c r="C4550" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4550" t="n">
         <v>201</v>
@@ -82344,7 +82344,7 @@
         </is>
       </c>
       <c r="C4551" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4551" t="n">
         <v>201</v>
@@ -82362,7 +82362,7 @@
         </is>
       </c>
       <c r="C4552" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4552" t="n">
         <v>201</v>
@@ -82371,16 +82371,16 @@
     <row r="4553">
       <c r="A4553" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4553" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4553" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4553" t="n">
         <v>201</v>
@@ -82398,7 +82398,7 @@
         </is>
       </c>
       <c r="C4554" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4554" t="n">
         <v>201</v>
@@ -82416,7 +82416,7 @@
         </is>
       </c>
       <c r="C4555" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4555" t="n">
         <v>201</v>
@@ -82434,7 +82434,7 @@
         </is>
       </c>
       <c r="C4556" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4556" t="n">
         <v>201</v>
@@ -82452,7 +82452,7 @@
         </is>
       </c>
       <c r="C4557" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4557" t="n">
         <v>201</v>
@@ -82470,7 +82470,7 @@
         </is>
       </c>
       <c r="C4558" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4558" t="n">
         <v>201</v>
@@ -82479,16 +82479,16 @@
     <row r="4559">
       <c r="A4559" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4559" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4559" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4559" t="n">
         <v>201</v>
@@ -82506,7 +82506,7 @@
         </is>
       </c>
       <c r="C4560" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4560" t="n">
         <v>201</v>
@@ -82524,7 +82524,7 @@
         </is>
       </c>
       <c r="C4561" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4561" t="n">
         <v>201</v>
@@ -82542,7 +82542,7 @@
         </is>
       </c>
       <c r="C4562" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4562" t="n">
         <v>201</v>
@@ -82560,7 +82560,7 @@
         </is>
       </c>
       <c r="C4563" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4563" t="n">
         <v>201</v>
@@ -82569,16 +82569,16 @@
     <row r="4564">
       <c r="A4564" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4564" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4564" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4564" t="n">
         <v>201</v>
@@ -82596,7 +82596,7 @@
         </is>
       </c>
       <c r="C4565" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4565" t="n">
         <v>201</v>
@@ -82614,7 +82614,7 @@
         </is>
       </c>
       <c r="C4566" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4566" t="n">
         <v>201</v>
@@ -82632,7 +82632,7 @@
         </is>
       </c>
       <c r="C4567" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4567" t="n">
         <v>201</v>
@@ -82650,7 +82650,7 @@
         </is>
       </c>
       <c r="C4568" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4568" t="n">
         <v>201</v>
@@ -82668,7 +82668,7 @@
         </is>
       </c>
       <c r="C4569" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4569" t="n">
         <v>201</v>
@@ -82686,7 +82686,7 @@
         </is>
       </c>
       <c r="C4570" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4570" t="n">
         <v>201</v>
@@ -82695,16 +82695,16 @@
     <row r="4571">
       <c r="A4571" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4571" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4571" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4571" t="n">
         <v>201</v>
@@ -82722,7 +82722,7 @@
         </is>
       </c>
       <c r="C4572" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4572" t="n">
         <v>201</v>
@@ -82740,7 +82740,7 @@
         </is>
       </c>
       <c r="C4573" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4573" t="n">
         <v>201</v>
@@ -82758,7 +82758,7 @@
         </is>
       </c>
       <c r="C4574" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4574" t="n">
         <v>201</v>
@@ -82776,7 +82776,7 @@
         </is>
       </c>
       <c r="C4575" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4575" t="n">
         <v>201</v>
@@ -82794,7 +82794,7 @@
         </is>
       </c>
       <c r="C4576" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4576" t="n">
         <v>201</v>
@@ -82812,7 +82812,7 @@
         </is>
       </c>
       <c r="C4577" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4577" t="n">
         <v>201</v>
@@ -82821,16 +82821,16 @@
     <row r="4578">
       <c r="A4578" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4578" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4578" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4578" t="n">
         <v>201</v>
@@ -82848,7 +82848,7 @@
         </is>
       </c>
       <c r="C4579" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4579" t="n">
         <v>201</v>
@@ -82866,7 +82866,7 @@
         </is>
       </c>
       <c r="C4580" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4580" t="n">
         <v>201</v>
@@ -82884,7 +82884,7 @@
         </is>
       </c>
       <c r="C4581" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4581" t="n">
         <v>201</v>
@@ -82902,7 +82902,7 @@
         </is>
       </c>
       <c r="C4582" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4582" t="n">
         <v>201</v>
@@ -82911,16 +82911,16 @@
     <row r="4583">
       <c r="A4583" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4583" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4583" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4583" t="n">
         <v>201</v>
@@ -82938,9 +82938,27 @@
         </is>
       </c>
       <c r="C4584" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4584" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4585">
+      <c r="A4585" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4585" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4585" t="n">
         <v>7</v>
       </c>
-      <c r="D4584" t="n">
+      <c r="D4585" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-20 05:47 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4599"/>
+  <dimension ref="A1:D4600"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82461,16 +82461,16 @@
     <row r="4558">
       <c r="A4558" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/20</t>
         </is>
       </c>
       <c r="B4558" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4558" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4558" t="n">
         <v>201</v>
@@ -82488,7 +82488,7 @@
         </is>
       </c>
       <c r="C4559" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4559" t="n">
         <v>201</v>
@@ -82506,7 +82506,7 @@
         </is>
       </c>
       <c r="C4560" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4560" t="n">
         <v>201</v>
@@ -82524,7 +82524,7 @@
         </is>
       </c>
       <c r="C4561" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4561" t="n">
         <v>201</v>
@@ -82533,16 +82533,16 @@
     <row r="4562">
       <c r="A4562" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4562" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4562" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4562" t="n">
         <v>201</v>
@@ -82560,7 +82560,7 @@
         </is>
       </c>
       <c r="C4563" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4563" t="n">
         <v>201</v>
@@ -82578,7 +82578,7 @@
         </is>
       </c>
       <c r="C4564" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4564" t="n">
         <v>201</v>
@@ -82596,7 +82596,7 @@
         </is>
       </c>
       <c r="C4565" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4565" t="n">
         <v>201</v>
@@ -82614,7 +82614,7 @@
         </is>
       </c>
       <c r="C4566" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4566" t="n">
         <v>201</v>
@@ -82632,7 +82632,7 @@
         </is>
       </c>
       <c r="C4567" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4567" t="n">
         <v>201</v>
@@ -82641,16 +82641,16 @@
     <row r="4568">
       <c r="A4568" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4568" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4568" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4568" t="n">
         <v>201</v>
@@ -82668,7 +82668,7 @@
         </is>
       </c>
       <c r="C4569" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4569" t="n">
         <v>201</v>
@@ -82686,7 +82686,7 @@
         </is>
       </c>
       <c r="C4570" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4570" t="n">
         <v>201</v>
@@ -82704,7 +82704,7 @@
         </is>
       </c>
       <c r="C4571" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4571" t="n">
         <v>201</v>
@@ -82722,7 +82722,7 @@
         </is>
       </c>
       <c r="C4572" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4572" t="n">
         <v>201</v>
@@ -82740,7 +82740,7 @@
         </is>
       </c>
       <c r="C4573" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4573" t="n">
         <v>201</v>
@@ -82749,16 +82749,16 @@
     <row r="4574">
       <c r="A4574" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4574" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4574" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4574" t="n">
         <v>201</v>
@@ -82776,7 +82776,7 @@
         </is>
       </c>
       <c r="C4575" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4575" t="n">
         <v>201</v>
@@ -82794,7 +82794,7 @@
         </is>
       </c>
       <c r="C4576" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4576" t="n">
         <v>201</v>
@@ -82812,7 +82812,7 @@
         </is>
       </c>
       <c r="C4577" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4577" t="n">
         <v>201</v>
@@ -82830,7 +82830,7 @@
         </is>
       </c>
       <c r="C4578" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4578" t="n">
         <v>201</v>
@@ -82839,16 +82839,16 @@
     <row r="4579">
       <c r="A4579" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4579" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4579" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4579" t="n">
         <v>201</v>
@@ -82866,7 +82866,7 @@
         </is>
       </c>
       <c r="C4580" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4580" t="n">
         <v>201</v>
@@ -82884,7 +82884,7 @@
         </is>
       </c>
       <c r="C4581" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4581" t="n">
         <v>201</v>
@@ -82902,7 +82902,7 @@
         </is>
       </c>
       <c r="C4582" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4582" t="n">
         <v>201</v>
@@ -82920,7 +82920,7 @@
         </is>
       </c>
       <c r="C4583" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4583" t="n">
         <v>201</v>
@@ -82938,7 +82938,7 @@
         </is>
       </c>
       <c r="C4584" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4584" t="n">
         <v>201</v>
@@ -82956,7 +82956,7 @@
         </is>
       </c>
       <c r="C4585" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4585" t="n">
         <v>201</v>
@@ -82965,16 +82965,16 @@
     <row r="4586">
       <c r="A4586" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4586" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4586" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4586" t="n">
         <v>201</v>
@@ -82992,7 +82992,7 @@
         </is>
       </c>
       <c r="C4587" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4587" t="n">
         <v>201</v>
@@ -83010,7 +83010,7 @@
         </is>
       </c>
       <c r="C4588" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4588" t="n">
         <v>201</v>
@@ -83028,7 +83028,7 @@
         </is>
       </c>
       <c r="C4589" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4589" t="n">
         <v>201</v>
@@ -83046,7 +83046,7 @@
         </is>
       </c>
       <c r="C4590" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4590" t="n">
         <v>201</v>
@@ -83064,7 +83064,7 @@
         </is>
       </c>
       <c r="C4591" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4591" t="n">
         <v>201</v>
@@ -83082,7 +83082,7 @@
         </is>
       </c>
       <c r="C4592" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4592" t="n">
         <v>201</v>
@@ -83091,16 +83091,16 @@
     <row r="4593">
       <c r="A4593" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4593" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4593" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4593" t="n">
         <v>201</v>
@@ -83118,7 +83118,7 @@
         </is>
       </c>
       <c r="C4594" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4594" t="n">
         <v>201</v>
@@ -83136,7 +83136,7 @@
         </is>
       </c>
       <c r="C4595" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4595" t="n">
         <v>201</v>
@@ -83154,7 +83154,7 @@
         </is>
       </c>
       <c r="C4596" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4596" t="n">
         <v>201</v>
@@ -83172,7 +83172,7 @@
         </is>
       </c>
       <c r="C4597" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4597" t="n">
         <v>201</v>
@@ -83181,16 +83181,16 @@
     <row r="4598">
       <c r="A4598" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4598" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4598" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4598" t="n">
         <v>201</v>
@@ -83208,9 +83208,27 @@
         </is>
       </c>
       <c r="C4599" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4599" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4600">
+      <c r="A4600" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4600" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4600" t="n">
         <v>7</v>
       </c>
-      <c r="D4599" t="n">
+      <c r="D4600" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-20 11:53 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4602"/>
+  <dimension ref="A1:D4603"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82515,16 +82515,16 @@
     <row r="4561">
       <c r="A4561" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/20</t>
         </is>
       </c>
       <c r="B4561" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4561" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D4561" t="n">
         <v>201</v>
@@ -82542,7 +82542,7 @@
         </is>
       </c>
       <c r="C4562" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4562" t="n">
         <v>201</v>
@@ -82560,7 +82560,7 @@
         </is>
       </c>
       <c r="C4563" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4563" t="n">
         <v>201</v>
@@ -82578,7 +82578,7 @@
         </is>
       </c>
       <c r="C4564" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4564" t="n">
         <v>201</v>
@@ -82587,16 +82587,16 @@
     <row r="4565">
       <c r="A4565" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4565" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4565" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4565" t="n">
         <v>201</v>
@@ -82614,7 +82614,7 @@
         </is>
       </c>
       <c r="C4566" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4566" t="n">
         <v>201</v>
@@ -82632,7 +82632,7 @@
         </is>
       </c>
       <c r="C4567" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4567" t="n">
         <v>201</v>
@@ -82650,7 +82650,7 @@
         </is>
       </c>
       <c r="C4568" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4568" t="n">
         <v>201</v>
@@ -82668,7 +82668,7 @@
         </is>
       </c>
       <c r="C4569" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4569" t="n">
         <v>201</v>
@@ -82686,7 +82686,7 @@
         </is>
       </c>
       <c r="C4570" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4570" t="n">
         <v>201</v>
@@ -82695,16 +82695,16 @@
     <row r="4571">
       <c r="A4571" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4571" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4571" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4571" t="n">
         <v>201</v>
@@ -82722,7 +82722,7 @@
         </is>
       </c>
       <c r="C4572" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4572" t="n">
         <v>201</v>
@@ -82740,7 +82740,7 @@
         </is>
       </c>
       <c r="C4573" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4573" t="n">
         <v>201</v>
@@ -82758,7 +82758,7 @@
         </is>
       </c>
       <c r="C4574" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4574" t="n">
         <v>201</v>
@@ -82776,7 +82776,7 @@
         </is>
       </c>
       <c r="C4575" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4575" t="n">
         <v>201</v>
@@ -82794,7 +82794,7 @@
         </is>
       </c>
       <c r="C4576" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4576" t="n">
         <v>201</v>
@@ -82803,16 +82803,16 @@
     <row r="4577">
       <c r="A4577" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4577" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4577" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4577" t="n">
         <v>201</v>
@@ -82830,7 +82830,7 @@
         </is>
       </c>
       <c r="C4578" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4578" t="n">
         <v>201</v>
@@ -82848,7 +82848,7 @@
         </is>
       </c>
       <c r="C4579" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4579" t="n">
         <v>201</v>
@@ -82866,7 +82866,7 @@
         </is>
       </c>
       <c r="C4580" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4580" t="n">
         <v>201</v>
@@ -82884,7 +82884,7 @@
         </is>
       </c>
       <c r="C4581" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4581" t="n">
         <v>201</v>
@@ -82893,16 +82893,16 @@
     <row r="4582">
       <c r="A4582" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4582" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4582" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4582" t="n">
         <v>201</v>
@@ -82920,7 +82920,7 @@
         </is>
       </c>
       <c r="C4583" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4583" t="n">
         <v>201</v>
@@ -82938,7 +82938,7 @@
         </is>
       </c>
       <c r="C4584" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4584" t="n">
         <v>201</v>
@@ -82956,7 +82956,7 @@
         </is>
       </c>
       <c r="C4585" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4585" t="n">
         <v>201</v>
@@ -82974,7 +82974,7 @@
         </is>
       </c>
       <c r="C4586" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4586" t="n">
         <v>201</v>
@@ -82992,7 +82992,7 @@
         </is>
       </c>
       <c r="C4587" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4587" t="n">
         <v>201</v>
@@ -83010,7 +83010,7 @@
         </is>
       </c>
       <c r="C4588" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4588" t="n">
         <v>201</v>
@@ -83019,16 +83019,16 @@
     <row r="4589">
       <c r="A4589" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4589" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4589" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4589" t="n">
         <v>201</v>
@@ -83046,7 +83046,7 @@
         </is>
       </c>
       <c r="C4590" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4590" t="n">
         <v>201</v>
@@ -83064,7 +83064,7 @@
         </is>
       </c>
       <c r="C4591" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4591" t="n">
         <v>201</v>
@@ -83082,7 +83082,7 @@
         </is>
       </c>
       <c r="C4592" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4592" t="n">
         <v>201</v>
@@ -83100,7 +83100,7 @@
         </is>
       </c>
       <c r="C4593" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4593" t="n">
         <v>201</v>
@@ -83118,7 +83118,7 @@
         </is>
       </c>
       <c r="C4594" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4594" t="n">
         <v>201</v>
@@ -83136,7 +83136,7 @@
         </is>
       </c>
       <c r="C4595" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4595" t="n">
         <v>201</v>
@@ -83145,16 +83145,16 @@
     <row r="4596">
       <c r="A4596" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4596" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4596" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4596" t="n">
         <v>201</v>
@@ -83172,7 +83172,7 @@
         </is>
       </c>
       <c r="C4597" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4597" t="n">
         <v>201</v>
@@ -83190,7 +83190,7 @@
         </is>
       </c>
       <c r="C4598" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4598" t="n">
         <v>201</v>
@@ -83208,7 +83208,7 @@
         </is>
       </c>
       <c r="C4599" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4599" t="n">
         <v>201</v>
@@ -83226,7 +83226,7 @@
         </is>
       </c>
       <c r="C4600" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4600" t="n">
         <v>201</v>
@@ -83235,16 +83235,16 @@
     <row r="4601">
       <c r="A4601" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4601" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4601" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4601" t="n">
         <v>201</v>
@@ -83262,9 +83262,27 @@
         </is>
       </c>
       <c r="C4602" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4602" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4603">
+      <c r="A4603" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4603" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4603" t="n">
         <v>7</v>
       </c>
-      <c r="D4602" t="n">
+      <c r="D4603" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-07-27 12:35 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4649"/>
+  <dimension ref="A1:D4650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83361,16 +83361,16 @@
     <row r="4608">
       <c r="A4608" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/27</t>
         </is>
       </c>
       <c r="B4608" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4608" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D4608" t="n">
         <v>201</v>
@@ -83388,7 +83388,7 @@
         </is>
       </c>
       <c r="C4609" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4609" t="n">
         <v>201</v>
@@ -83406,7 +83406,7 @@
         </is>
       </c>
       <c r="C4610" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4610" t="n">
         <v>201</v>
@@ -83424,7 +83424,7 @@
         </is>
       </c>
       <c r="C4611" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4611" t="n">
         <v>201</v>
@@ -83433,16 +83433,16 @@
     <row r="4612">
       <c r="A4612" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4612" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4612" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4612" t="n">
         <v>201</v>
@@ -83460,7 +83460,7 @@
         </is>
       </c>
       <c r="C4613" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4613" t="n">
         <v>201</v>
@@ -83478,7 +83478,7 @@
         </is>
       </c>
       <c r="C4614" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4614" t="n">
         <v>201</v>
@@ -83496,7 +83496,7 @@
         </is>
       </c>
       <c r="C4615" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4615" t="n">
         <v>201</v>
@@ -83514,7 +83514,7 @@
         </is>
       </c>
       <c r="C4616" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4616" t="n">
         <v>201</v>
@@ -83532,7 +83532,7 @@
         </is>
       </c>
       <c r="C4617" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4617" t="n">
         <v>201</v>
@@ -83541,16 +83541,16 @@
     <row r="4618">
       <c r="A4618" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4618" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4618" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4618" t="n">
         <v>201</v>
@@ -83568,7 +83568,7 @@
         </is>
       </c>
       <c r="C4619" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4619" t="n">
         <v>201</v>
@@ -83586,7 +83586,7 @@
         </is>
       </c>
       <c r="C4620" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4620" t="n">
         <v>201</v>
@@ -83604,7 +83604,7 @@
         </is>
       </c>
       <c r="C4621" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4621" t="n">
         <v>201</v>
@@ -83622,7 +83622,7 @@
         </is>
       </c>
       <c r="C4622" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4622" t="n">
         <v>201</v>
@@ -83640,7 +83640,7 @@
         </is>
       </c>
       <c r="C4623" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4623" t="n">
         <v>201</v>
@@ -83649,16 +83649,16 @@
     <row r="4624">
       <c r="A4624" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4624" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4624" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4624" t="n">
         <v>201</v>
@@ -83676,7 +83676,7 @@
         </is>
       </c>
       <c r="C4625" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4625" t="n">
         <v>201</v>
@@ -83694,7 +83694,7 @@
         </is>
       </c>
       <c r="C4626" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4626" t="n">
         <v>201</v>
@@ -83712,7 +83712,7 @@
         </is>
       </c>
       <c r="C4627" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4627" t="n">
         <v>201</v>
@@ -83730,7 +83730,7 @@
         </is>
       </c>
       <c r="C4628" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4628" t="n">
         <v>201</v>
@@ -83739,16 +83739,16 @@
     <row r="4629">
       <c r="A4629" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4629" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4629" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4629" t="n">
         <v>201</v>
@@ -83766,7 +83766,7 @@
         </is>
       </c>
       <c r="C4630" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4630" t="n">
         <v>201</v>
@@ -83784,7 +83784,7 @@
         </is>
       </c>
       <c r="C4631" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4631" t="n">
         <v>201</v>
@@ -83802,7 +83802,7 @@
         </is>
       </c>
       <c r="C4632" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4632" t="n">
         <v>201</v>
@@ -83820,7 +83820,7 @@
         </is>
       </c>
       <c r="C4633" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4633" t="n">
         <v>201</v>
@@ -83838,7 +83838,7 @@
         </is>
       </c>
       <c r="C4634" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4634" t="n">
         <v>201</v>
@@ -83856,7 +83856,7 @@
         </is>
       </c>
       <c r="C4635" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4635" t="n">
         <v>201</v>
@@ -83865,16 +83865,16 @@
     <row r="4636">
       <c r="A4636" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4636" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4636" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4636" t="n">
         <v>201</v>
@@ -83892,7 +83892,7 @@
         </is>
       </c>
       <c r="C4637" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4637" t="n">
         <v>201</v>
@@ -83910,7 +83910,7 @@
         </is>
       </c>
       <c r="C4638" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4638" t="n">
         <v>201</v>
@@ -83928,7 +83928,7 @@
         </is>
       </c>
       <c r="C4639" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4639" t="n">
         <v>201</v>
@@ -83946,7 +83946,7 @@
         </is>
       </c>
       <c r="C4640" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4640" t="n">
         <v>201</v>
@@ -83964,7 +83964,7 @@
         </is>
       </c>
       <c r="C4641" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4641" t="n">
         <v>201</v>
@@ -83982,7 +83982,7 @@
         </is>
       </c>
       <c r="C4642" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4642" t="n">
         <v>201</v>
@@ -83991,16 +83991,16 @@
     <row r="4643">
       <c r="A4643" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4643" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4643" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4643" t="n">
         <v>201</v>
@@ -84018,7 +84018,7 @@
         </is>
       </c>
       <c r="C4644" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4644" t="n">
         <v>201</v>
@@ -84036,7 +84036,7 @@
         </is>
       </c>
       <c r="C4645" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4645" t="n">
         <v>201</v>
@@ -84054,7 +84054,7 @@
         </is>
       </c>
       <c r="C4646" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4646" t="n">
         <v>201</v>
@@ -84072,7 +84072,7 @@
         </is>
       </c>
       <c r="C4647" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4647" t="n">
         <v>201</v>
@@ -84081,16 +84081,16 @@
     <row r="4648">
       <c r="A4648" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4648" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4648" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4648" t="n">
         <v>201</v>
@@ -84108,9 +84108,27 @@
         </is>
       </c>
       <c r="C4649" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4649" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4650">
+      <c r="A4650" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4650" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4650" t="n">
         <v>7</v>
       </c>
-      <c r="D4649" t="n">
+      <c r="D4650" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-05 03:29 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4706"/>
+  <dimension ref="A1:D4707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -84387,16 +84387,16 @@
     <row r="4665">
       <c r="A4665" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/05</t>
         </is>
       </c>
       <c r="B4665" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4665" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D4665" t="n">
         <v>201</v>
@@ -84414,7 +84414,7 @@
         </is>
       </c>
       <c r="C4666" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4666" t="n">
         <v>201</v>
@@ -84432,7 +84432,7 @@
         </is>
       </c>
       <c r="C4667" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4667" t="n">
         <v>201</v>
@@ -84450,7 +84450,7 @@
         </is>
       </c>
       <c r="C4668" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4668" t="n">
         <v>201</v>
@@ -84459,16 +84459,16 @@
     <row r="4669">
       <c r="A4669" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4669" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4669" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4669" t="n">
         <v>201</v>
@@ -84486,7 +84486,7 @@
         </is>
       </c>
       <c r="C4670" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4670" t="n">
         <v>201</v>
@@ -84504,7 +84504,7 @@
         </is>
       </c>
       <c r="C4671" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4671" t="n">
         <v>201</v>
@@ -84522,7 +84522,7 @@
         </is>
       </c>
       <c r="C4672" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4672" t="n">
         <v>201</v>
@@ -84540,7 +84540,7 @@
         </is>
       </c>
       <c r="C4673" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4673" t="n">
         <v>201</v>
@@ -84558,7 +84558,7 @@
         </is>
       </c>
       <c r="C4674" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4674" t="n">
         <v>201</v>
@@ -84567,16 +84567,16 @@
     <row r="4675">
       <c r="A4675" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4675" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4675" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4675" t="n">
         <v>201</v>
@@ -84594,7 +84594,7 @@
         </is>
       </c>
       <c r="C4676" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4676" t="n">
         <v>201</v>
@@ -84612,7 +84612,7 @@
         </is>
       </c>
       <c r="C4677" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4677" t="n">
         <v>201</v>
@@ -84630,7 +84630,7 @@
         </is>
       </c>
       <c r="C4678" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4678" t="n">
         <v>201</v>
@@ -84648,7 +84648,7 @@
         </is>
       </c>
       <c r="C4679" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4679" t="n">
         <v>201</v>
@@ -84666,7 +84666,7 @@
         </is>
       </c>
       <c r="C4680" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4680" t="n">
         <v>201</v>
@@ -84675,16 +84675,16 @@
     <row r="4681">
       <c r="A4681" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4681" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4681" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4681" t="n">
         <v>201</v>
@@ -84702,7 +84702,7 @@
         </is>
       </c>
       <c r="C4682" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4682" t="n">
         <v>201</v>
@@ -84720,7 +84720,7 @@
         </is>
       </c>
       <c r="C4683" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4683" t="n">
         <v>201</v>
@@ -84738,7 +84738,7 @@
         </is>
       </c>
       <c r="C4684" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4684" t="n">
         <v>201</v>
@@ -84756,7 +84756,7 @@
         </is>
       </c>
       <c r="C4685" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4685" t="n">
         <v>201</v>
@@ -84765,16 +84765,16 @@
     <row r="4686">
       <c r="A4686" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4686" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4686" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4686" t="n">
         <v>201</v>
@@ -84792,7 +84792,7 @@
         </is>
       </c>
       <c r="C4687" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4687" t="n">
         <v>201</v>
@@ -84810,7 +84810,7 @@
         </is>
       </c>
       <c r="C4688" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4688" t="n">
         <v>201</v>
@@ -84828,7 +84828,7 @@
         </is>
       </c>
       <c r="C4689" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4689" t="n">
         <v>201</v>
@@ -84846,7 +84846,7 @@
         </is>
       </c>
       <c r="C4690" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4690" t="n">
         <v>201</v>
@@ -84864,7 +84864,7 @@
         </is>
       </c>
       <c r="C4691" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4691" t="n">
         <v>201</v>
@@ -84882,7 +84882,7 @@
         </is>
       </c>
       <c r="C4692" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4692" t="n">
         <v>201</v>
@@ -84891,16 +84891,16 @@
     <row r="4693">
       <c r="A4693" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4693" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4693" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4693" t="n">
         <v>201</v>
@@ -84918,7 +84918,7 @@
         </is>
       </c>
       <c r="C4694" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4694" t="n">
         <v>201</v>
@@ -84936,7 +84936,7 @@
         </is>
       </c>
       <c r="C4695" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4695" t="n">
         <v>201</v>
@@ -84954,7 +84954,7 @@
         </is>
       </c>
       <c r="C4696" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4696" t="n">
         <v>201</v>
@@ -84972,7 +84972,7 @@
         </is>
       </c>
       <c r="C4697" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4697" t="n">
         <v>201</v>
@@ -84990,7 +84990,7 @@
         </is>
       </c>
       <c r="C4698" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4698" t="n">
         <v>201</v>
@@ -85008,7 +85008,7 @@
         </is>
       </c>
       <c r="C4699" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4699" t="n">
         <v>201</v>
@@ -85017,16 +85017,16 @@
     <row r="4700">
       <c r="A4700" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4700" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4700" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4700" t="n">
         <v>201</v>
@@ -85044,7 +85044,7 @@
         </is>
       </c>
       <c r="C4701" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4701" t="n">
         <v>201</v>
@@ -85062,7 +85062,7 @@
         </is>
       </c>
       <c r="C4702" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4702" t="n">
         <v>201</v>
@@ -85080,7 +85080,7 @@
         </is>
       </c>
       <c r="C4703" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4703" t="n">
         <v>201</v>
@@ -85098,7 +85098,7 @@
         </is>
       </c>
       <c r="C4704" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4704" t="n">
         <v>201</v>
@@ -85107,16 +85107,16 @@
     <row r="4705">
       <c r="A4705" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4705" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4705" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4705" t="n">
         <v>201</v>
@@ -85134,9 +85134,27 @@
         </is>
       </c>
       <c r="C4706" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4706" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4707">
+      <c r="A4707" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4707" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4707" t="n">
         <v>7</v>
       </c>
-      <c r="D4706" t="n">
+      <c r="D4707" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-07 05:01 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4721"/>
+  <dimension ref="A1:D4722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -84657,16 +84657,16 @@
     <row r="4680">
       <c r="A4680" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="B4680" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4680" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4680" t="n">
         <v>201</v>
@@ -84684,7 +84684,7 @@
         </is>
       </c>
       <c r="C4681" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4681" t="n">
         <v>201</v>
@@ -84702,7 +84702,7 @@
         </is>
       </c>
       <c r="C4682" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4682" t="n">
         <v>201</v>
@@ -84720,7 +84720,7 @@
         </is>
       </c>
       <c r="C4683" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4683" t="n">
         <v>201</v>
@@ -84729,16 +84729,16 @@
     <row r="4684">
       <c r="A4684" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4684" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4684" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4684" t="n">
         <v>201</v>
@@ -84756,7 +84756,7 @@
         </is>
       </c>
       <c r="C4685" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4685" t="n">
         <v>201</v>
@@ -84774,7 +84774,7 @@
         </is>
       </c>
       <c r="C4686" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4686" t="n">
         <v>201</v>
@@ -84792,7 +84792,7 @@
         </is>
       </c>
       <c r="C4687" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4687" t="n">
         <v>201</v>
@@ -84810,7 +84810,7 @@
         </is>
       </c>
       <c r="C4688" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4688" t="n">
         <v>201</v>
@@ -84828,7 +84828,7 @@
         </is>
       </c>
       <c r="C4689" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4689" t="n">
         <v>201</v>
@@ -84837,16 +84837,16 @@
     <row r="4690">
       <c r="A4690" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4690" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4690" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4690" t="n">
         <v>201</v>
@@ -84864,7 +84864,7 @@
         </is>
       </c>
       <c r="C4691" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4691" t="n">
         <v>201</v>
@@ -84882,7 +84882,7 @@
         </is>
       </c>
       <c r="C4692" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4692" t="n">
         <v>201</v>
@@ -84900,7 +84900,7 @@
         </is>
       </c>
       <c r="C4693" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4693" t="n">
         <v>201</v>
@@ -84918,7 +84918,7 @@
         </is>
       </c>
       <c r="C4694" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4694" t="n">
         <v>201</v>
@@ -84936,7 +84936,7 @@
         </is>
       </c>
       <c r="C4695" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4695" t="n">
         <v>201</v>
@@ -84945,16 +84945,16 @@
     <row r="4696">
       <c r="A4696" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4696" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4696" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4696" t="n">
         <v>201</v>
@@ -84972,7 +84972,7 @@
         </is>
       </c>
       <c r="C4697" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4697" t="n">
         <v>201</v>
@@ -84990,7 +84990,7 @@
         </is>
       </c>
       <c r="C4698" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4698" t="n">
         <v>201</v>
@@ -85008,7 +85008,7 @@
         </is>
       </c>
       <c r="C4699" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4699" t="n">
         <v>201</v>
@@ -85026,7 +85026,7 @@
         </is>
       </c>
       <c r="C4700" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4700" t="n">
         <v>201</v>
@@ -85035,16 +85035,16 @@
     <row r="4701">
       <c r="A4701" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4701" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4701" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4701" t="n">
         <v>201</v>
@@ -85062,7 +85062,7 @@
         </is>
       </c>
       <c r="C4702" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4702" t="n">
         <v>201</v>
@@ -85080,7 +85080,7 @@
         </is>
       </c>
       <c r="C4703" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4703" t="n">
         <v>201</v>
@@ -85098,7 +85098,7 @@
         </is>
       </c>
       <c r="C4704" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4704" t="n">
         <v>201</v>
@@ -85116,7 +85116,7 @@
         </is>
       </c>
       <c r="C4705" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4705" t="n">
         <v>201</v>
@@ -85134,7 +85134,7 @@
         </is>
       </c>
       <c r="C4706" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4706" t="n">
         <v>201</v>
@@ -85152,7 +85152,7 @@
         </is>
       </c>
       <c r="C4707" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4707" t="n">
         <v>201</v>
@@ -85161,16 +85161,16 @@
     <row r="4708">
       <c r="A4708" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4708" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4708" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4708" t="n">
         <v>201</v>
@@ -85188,7 +85188,7 @@
         </is>
       </c>
       <c r="C4709" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4709" t="n">
         <v>201</v>
@@ -85206,7 +85206,7 @@
         </is>
       </c>
       <c r="C4710" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4710" t="n">
         <v>201</v>
@@ -85224,7 +85224,7 @@
         </is>
       </c>
       <c r="C4711" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4711" t="n">
         <v>201</v>
@@ -85242,7 +85242,7 @@
         </is>
       </c>
       <c r="C4712" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4712" t="n">
         <v>201</v>
@@ -85260,7 +85260,7 @@
         </is>
       </c>
       <c r="C4713" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4713" t="n">
         <v>201</v>
@@ -85278,7 +85278,7 @@
         </is>
       </c>
       <c r="C4714" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4714" t="n">
         <v>201</v>
@@ -85287,16 +85287,16 @@
     <row r="4715">
       <c r="A4715" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4715" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4715" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4715" t="n">
         <v>201</v>
@@ -85314,7 +85314,7 @@
         </is>
       </c>
       <c r="C4716" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4716" t="n">
         <v>201</v>
@@ -85332,7 +85332,7 @@
         </is>
       </c>
       <c r="C4717" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4717" t="n">
         <v>201</v>
@@ -85350,7 +85350,7 @@
         </is>
       </c>
       <c r="C4718" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4718" t="n">
         <v>201</v>
@@ -85368,7 +85368,7 @@
         </is>
       </c>
       <c r="C4719" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4719" t="n">
         <v>201</v>
@@ -85377,16 +85377,16 @@
     <row r="4720">
       <c r="A4720" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4720" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4720" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4720" t="n">
         <v>201</v>
@@ -85404,9 +85404,27 @@
         </is>
       </c>
       <c r="C4721" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4721" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4722">
+      <c r="A4722" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4722" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4722" t="n">
         <v>7</v>
       </c>
-      <c r="D4721" t="n">
+      <c r="D4722" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-08 07:10 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4728"/>
+  <dimension ref="A1:D4729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -84783,16 +84783,16 @@
     <row r="4687">
       <c r="A4687" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/08</t>
         </is>
       </c>
       <c r="B4687" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4687" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4687" t="n">
         <v>201</v>
@@ -84810,7 +84810,7 @@
         </is>
       </c>
       <c r="C4688" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4688" t="n">
         <v>201</v>
@@ -84828,7 +84828,7 @@
         </is>
       </c>
       <c r="C4689" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4689" t="n">
         <v>201</v>
@@ -84846,7 +84846,7 @@
         </is>
       </c>
       <c r="C4690" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4690" t="n">
         <v>201</v>
@@ -84855,16 +84855,16 @@
     <row r="4691">
       <c r="A4691" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4691" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4691" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4691" t="n">
         <v>201</v>
@@ -84882,7 +84882,7 @@
         </is>
       </c>
       <c r="C4692" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4692" t="n">
         <v>201</v>
@@ -84900,7 +84900,7 @@
         </is>
       </c>
       <c r="C4693" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4693" t="n">
         <v>201</v>
@@ -84918,7 +84918,7 @@
         </is>
       </c>
       <c r="C4694" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4694" t="n">
         <v>201</v>
@@ -84936,7 +84936,7 @@
         </is>
       </c>
       <c r="C4695" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4695" t="n">
         <v>201</v>
@@ -84954,7 +84954,7 @@
         </is>
       </c>
       <c r="C4696" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4696" t="n">
         <v>201</v>
@@ -84963,16 +84963,16 @@
     <row r="4697">
       <c r="A4697" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4697" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4697" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4697" t="n">
         <v>201</v>
@@ -84990,7 +84990,7 @@
         </is>
       </c>
       <c r="C4698" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4698" t="n">
         <v>201</v>
@@ -85008,7 +85008,7 @@
         </is>
       </c>
       <c r="C4699" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4699" t="n">
         <v>201</v>
@@ -85026,7 +85026,7 @@
         </is>
       </c>
       <c r="C4700" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4700" t="n">
         <v>201</v>
@@ -85044,7 +85044,7 @@
         </is>
       </c>
       <c r="C4701" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4701" t="n">
         <v>201</v>
@@ -85062,7 +85062,7 @@
         </is>
       </c>
       <c r="C4702" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4702" t="n">
         <v>201</v>
@@ -85071,16 +85071,16 @@
     <row r="4703">
       <c r="A4703" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4703" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4703" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4703" t="n">
         <v>201</v>
@@ -85098,7 +85098,7 @@
         </is>
       </c>
       <c r="C4704" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4704" t="n">
         <v>201</v>
@@ -85116,7 +85116,7 @@
         </is>
       </c>
       <c r="C4705" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4705" t="n">
         <v>201</v>
@@ -85134,7 +85134,7 @@
         </is>
       </c>
       <c r="C4706" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4706" t="n">
         <v>201</v>
@@ -85152,7 +85152,7 @@
         </is>
       </c>
       <c r="C4707" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4707" t="n">
         <v>201</v>
@@ -85161,16 +85161,16 @@
     <row r="4708">
       <c r="A4708" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4708" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4708" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4708" t="n">
         <v>201</v>
@@ -85188,7 +85188,7 @@
         </is>
       </c>
       <c r="C4709" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4709" t="n">
         <v>201</v>
@@ -85206,7 +85206,7 @@
         </is>
       </c>
       <c r="C4710" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4710" t="n">
         <v>201</v>
@@ -85224,7 +85224,7 @@
         </is>
       </c>
       <c r="C4711" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4711" t="n">
         <v>201</v>
@@ -85242,7 +85242,7 @@
         </is>
       </c>
       <c r="C4712" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4712" t="n">
         <v>201</v>
@@ -85260,7 +85260,7 @@
         </is>
       </c>
       <c r="C4713" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4713" t="n">
         <v>201</v>
@@ -85278,7 +85278,7 @@
         </is>
       </c>
       <c r="C4714" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4714" t="n">
         <v>201</v>
@@ -85287,16 +85287,16 @@
     <row r="4715">
       <c r="A4715" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4715" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4715" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4715" t="n">
         <v>201</v>
@@ -85314,7 +85314,7 @@
         </is>
       </c>
       <c r="C4716" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4716" t="n">
         <v>201</v>
@@ -85332,7 +85332,7 @@
         </is>
       </c>
       <c r="C4717" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4717" t="n">
         <v>201</v>
@@ -85350,7 +85350,7 @@
         </is>
       </c>
       <c r="C4718" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4718" t="n">
         <v>201</v>
@@ -85368,7 +85368,7 @@
         </is>
       </c>
       <c r="C4719" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4719" t="n">
         <v>201</v>
@@ -85386,7 +85386,7 @@
         </is>
       </c>
       <c r="C4720" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4720" t="n">
         <v>201</v>
@@ -85404,7 +85404,7 @@
         </is>
       </c>
       <c r="C4721" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4721" t="n">
         <v>201</v>
@@ -85413,16 +85413,16 @@
     <row r="4722">
       <c r="A4722" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4722" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4722" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4722" t="n">
         <v>201</v>
@@ -85440,7 +85440,7 @@
         </is>
       </c>
       <c r="C4723" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4723" t="n">
         <v>201</v>
@@ -85458,7 +85458,7 @@
         </is>
       </c>
       <c r="C4724" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4724" t="n">
         <v>201</v>
@@ -85476,7 +85476,7 @@
         </is>
       </c>
       <c r="C4725" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4725" t="n">
         <v>201</v>
@@ -85494,7 +85494,7 @@
         </is>
       </c>
       <c r="C4726" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4726" t="n">
         <v>201</v>
@@ -85503,16 +85503,16 @@
     <row r="4727">
       <c r="A4727" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4727" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4727" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4727" t="n">
         <v>201</v>
@@ -85530,9 +85530,27 @@
         </is>
       </c>
       <c r="C4728" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4728" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4729">
+      <c r="A4729" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4729" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4729" t="n">
         <v>7</v>
       </c>
-      <c r="D4728" t="n">
+      <c r="D4729" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-10 08:00 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4743"/>
+  <dimension ref="A1:D4744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85053,16 +85053,16 @@
     <row r="4702">
       <c r="A4702" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/10</t>
         </is>
       </c>
       <c r="B4702" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4702" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4702" t="n">
         <v>201</v>
@@ -85080,7 +85080,7 @@
         </is>
       </c>
       <c r="C4703" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4703" t="n">
         <v>201</v>
@@ -85098,7 +85098,7 @@
         </is>
       </c>
       <c r="C4704" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4704" t="n">
         <v>201</v>
@@ -85116,7 +85116,7 @@
         </is>
       </c>
       <c r="C4705" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4705" t="n">
         <v>201</v>
@@ -85125,16 +85125,16 @@
     <row r="4706">
       <c r="A4706" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4706" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4706" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4706" t="n">
         <v>201</v>
@@ -85152,7 +85152,7 @@
         </is>
       </c>
       <c r="C4707" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4707" t="n">
         <v>201</v>
@@ -85170,7 +85170,7 @@
         </is>
       </c>
       <c r="C4708" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4708" t="n">
         <v>201</v>
@@ -85188,7 +85188,7 @@
         </is>
       </c>
       <c r="C4709" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4709" t="n">
         <v>201</v>
@@ -85206,7 +85206,7 @@
         </is>
       </c>
       <c r="C4710" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4710" t="n">
         <v>201</v>
@@ -85224,7 +85224,7 @@
         </is>
       </c>
       <c r="C4711" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4711" t="n">
         <v>201</v>
@@ -85233,16 +85233,16 @@
     <row r="4712">
       <c r="A4712" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4712" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4712" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4712" t="n">
         <v>201</v>
@@ -85260,7 +85260,7 @@
         </is>
       </c>
       <c r="C4713" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4713" t="n">
         <v>201</v>
@@ -85278,7 +85278,7 @@
         </is>
       </c>
       <c r="C4714" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4714" t="n">
         <v>201</v>
@@ -85296,7 +85296,7 @@
         </is>
       </c>
       <c r="C4715" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4715" t="n">
         <v>201</v>
@@ -85314,7 +85314,7 @@
         </is>
       </c>
       <c r="C4716" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4716" t="n">
         <v>201</v>
@@ -85332,7 +85332,7 @@
         </is>
       </c>
       <c r="C4717" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4717" t="n">
         <v>201</v>
@@ -85341,16 +85341,16 @@
     <row r="4718">
       <c r="A4718" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4718" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4718" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4718" t="n">
         <v>201</v>
@@ -85368,7 +85368,7 @@
         </is>
       </c>
       <c r="C4719" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4719" t="n">
         <v>201</v>
@@ -85386,7 +85386,7 @@
         </is>
       </c>
       <c r="C4720" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4720" t="n">
         <v>201</v>
@@ -85404,7 +85404,7 @@
         </is>
       </c>
       <c r="C4721" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4721" t="n">
         <v>201</v>
@@ -85422,7 +85422,7 @@
         </is>
       </c>
       <c r="C4722" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4722" t="n">
         <v>201</v>
@@ -85431,16 +85431,16 @@
     <row r="4723">
       <c r="A4723" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4723" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4723" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4723" t="n">
         <v>201</v>
@@ -85458,7 +85458,7 @@
         </is>
       </c>
       <c r="C4724" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4724" t="n">
         <v>201</v>
@@ -85476,7 +85476,7 @@
         </is>
       </c>
       <c r="C4725" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4725" t="n">
         <v>201</v>
@@ -85494,7 +85494,7 @@
         </is>
       </c>
       <c r="C4726" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4726" t="n">
         <v>201</v>
@@ -85512,7 +85512,7 @@
         </is>
       </c>
       <c r="C4727" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4727" t="n">
         <v>201</v>
@@ -85530,7 +85530,7 @@
         </is>
       </c>
       <c r="C4728" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4728" t="n">
         <v>201</v>
@@ -85548,7 +85548,7 @@
         </is>
       </c>
       <c r="C4729" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4729" t="n">
         <v>201</v>
@@ -85557,16 +85557,16 @@
     <row r="4730">
       <c r="A4730" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4730" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4730" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4730" t="n">
         <v>201</v>
@@ -85584,7 +85584,7 @@
         </is>
       </c>
       <c r="C4731" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4731" t="n">
         <v>201</v>
@@ -85602,7 +85602,7 @@
         </is>
       </c>
       <c r="C4732" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4732" t="n">
         <v>201</v>
@@ -85620,7 +85620,7 @@
         </is>
       </c>
       <c r="C4733" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4733" t="n">
         <v>201</v>
@@ -85638,7 +85638,7 @@
         </is>
       </c>
       <c r="C4734" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4734" t="n">
         <v>201</v>
@@ -85656,7 +85656,7 @@
         </is>
       </c>
       <c r="C4735" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4735" t="n">
         <v>201</v>
@@ -85674,7 +85674,7 @@
         </is>
       </c>
       <c r="C4736" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4736" t="n">
         <v>201</v>
@@ -85683,16 +85683,16 @@
     <row r="4737">
       <c r="A4737" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4737" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4737" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4737" t="n">
         <v>201</v>
@@ -85710,7 +85710,7 @@
         </is>
       </c>
       <c r="C4738" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4738" t="n">
         <v>201</v>
@@ -85728,7 +85728,7 @@
         </is>
       </c>
       <c r="C4739" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4739" t="n">
         <v>201</v>
@@ -85746,7 +85746,7 @@
         </is>
       </c>
       <c r="C4740" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4740" t="n">
         <v>201</v>
@@ -85764,7 +85764,7 @@
         </is>
       </c>
       <c r="C4741" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4741" t="n">
         <v>201</v>
@@ -85773,16 +85773,16 @@
     <row r="4742">
       <c r="A4742" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4742" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4742" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4742" t="n">
         <v>201</v>
@@ -85800,9 +85800,27 @@
         </is>
       </c>
       <c r="C4743" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4743" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4744">
+      <c r="A4744" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4744" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4744" t="n">
         <v>7</v>
       </c>
-      <c r="D4743" t="n">
+      <c r="D4744" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-13 02:44 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4761"/>
+  <dimension ref="A1:D4762"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85377,16 +85377,16 @@
     <row r="4720">
       <c r="A4720" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/13</t>
         </is>
       </c>
       <c r="B4720" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4720" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4720" t="n">
         <v>201</v>
@@ -85404,7 +85404,7 @@
         </is>
       </c>
       <c r="C4721" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4721" t="n">
         <v>201</v>
@@ -85422,7 +85422,7 @@
         </is>
       </c>
       <c r="C4722" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4722" t="n">
         <v>201</v>
@@ -85440,7 +85440,7 @@
         </is>
       </c>
       <c r="C4723" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4723" t="n">
         <v>201</v>
@@ -85449,16 +85449,16 @@
     <row r="4724">
       <c r="A4724" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4724" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4724" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4724" t="n">
         <v>201</v>
@@ -85476,7 +85476,7 @@
         </is>
       </c>
       <c r="C4725" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4725" t="n">
         <v>201</v>
@@ -85494,7 +85494,7 @@
         </is>
       </c>
       <c r="C4726" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4726" t="n">
         <v>201</v>
@@ -85512,7 +85512,7 @@
         </is>
       </c>
       <c r="C4727" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4727" t="n">
         <v>201</v>
@@ -85530,7 +85530,7 @@
         </is>
       </c>
       <c r="C4728" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4728" t="n">
         <v>201</v>
@@ -85548,7 +85548,7 @@
         </is>
       </c>
       <c r="C4729" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4729" t="n">
         <v>201</v>
@@ -85557,16 +85557,16 @@
     <row r="4730">
       <c r="A4730" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4730" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4730" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4730" t="n">
         <v>201</v>
@@ -85584,7 +85584,7 @@
         </is>
       </c>
       <c r="C4731" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4731" t="n">
         <v>201</v>
@@ -85602,7 +85602,7 @@
         </is>
       </c>
       <c r="C4732" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4732" t="n">
         <v>201</v>
@@ -85620,7 +85620,7 @@
         </is>
       </c>
       <c r="C4733" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4733" t="n">
         <v>201</v>
@@ -85638,7 +85638,7 @@
         </is>
       </c>
       <c r="C4734" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4734" t="n">
         <v>201</v>
@@ -85656,7 +85656,7 @@
         </is>
       </c>
       <c r="C4735" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4735" t="n">
         <v>201</v>
@@ -85665,16 +85665,16 @@
     <row r="4736">
       <c r="A4736" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4736" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4736" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4736" t="n">
         <v>201</v>
@@ -85692,7 +85692,7 @@
         </is>
       </c>
       <c r="C4737" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4737" t="n">
         <v>201</v>
@@ -85710,7 +85710,7 @@
         </is>
       </c>
       <c r="C4738" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4738" t="n">
         <v>201</v>
@@ -85728,7 +85728,7 @@
         </is>
       </c>
       <c r="C4739" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4739" t="n">
         <v>201</v>
@@ -85746,7 +85746,7 @@
         </is>
       </c>
       <c r="C4740" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4740" t="n">
         <v>201</v>
@@ -85755,16 +85755,16 @@
     <row r="4741">
       <c r="A4741" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4741" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4741" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4741" t="n">
         <v>201</v>
@@ -85782,7 +85782,7 @@
         </is>
       </c>
       <c r="C4742" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4742" t="n">
         <v>201</v>
@@ -85800,7 +85800,7 @@
         </is>
       </c>
       <c r="C4743" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4743" t="n">
         <v>201</v>
@@ -85818,7 +85818,7 @@
         </is>
       </c>
       <c r="C4744" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4744" t="n">
         <v>201</v>
@@ -85836,7 +85836,7 @@
         </is>
       </c>
       <c r="C4745" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4745" t="n">
         <v>201</v>
@@ -85854,7 +85854,7 @@
         </is>
       </c>
       <c r="C4746" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4746" t="n">
         <v>201</v>
@@ -85872,7 +85872,7 @@
         </is>
       </c>
       <c r="C4747" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4747" t="n">
         <v>201</v>
@@ -85881,16 +85881,16 @@
     <row r="4748">
       <c r="A4748" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4748" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4748" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4748" t="n">
         <v>201</v>
@@ -85908,7 +85908,7 @@
         </is>
       </c>
       <c r="C4749" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4749" t="n">
         <v>201</v>
@@ -85926,7 +85926,7 @@
         </is>
       </c>
       <c r="C4750" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4750" t="n">
         <v>201</v>
@@ -85944,7 +85944,7 @@
         </is>
       </c>
       <c r="C4751" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4751" t="n">
         <v>201</v>
@@ -85962,7 +85962,7 @@
         </is>
       </c>
       <c r="C4752" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4752" t="n">
         <v>201</v>
@@ -85980,7 +85980,7 @@
         </is>
       </c>
       <c r="C4753" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4753" t="n">
         <v>201</v>
@@ -85998,7 +85998,7 @@
         </is>
       </c>
       <c r="C4754" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4754" t="n">
         <v>201</v>
@@ -86007,16 +86007,16 @@
     <row r="4755">
       <c r="A4755" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4755" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4755" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4755" t="n">
         <v>201</v>
@@ -86034,7 +86034,7 @@
         </is>
       </c>
       <c r="C4756" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4756" t="n">
         <v>201</v>
@@ -86052,7 +86052,7 @@
         </is>
       </c>
       <c r="C4757" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4757" t="n">
         <v>201</v>
@@ -86070,7 +86070,7 @@
         </is>
       </c>
       <c r="C4758" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4758" t="n">
         <v>201</v>
@@ -86088,7 +86088,7 @@
         </is>
       </c>
       <c r="C4759" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4759" t="n">
         <v>201</v>
@@ -86097,16 +86097,16 @@
     <row r="4760">
       <c r="A4760" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4760" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4760" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4760" t="n">
         <v>201</v>
@@ -86124,9 +86124,27 @@
         </is>
       </c>
       <c r="C4761" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4761" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4762">
+      <c r="A4762" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4762" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4762" t="n">
         <v>7</v>
       </c>
-      <c r="D4761" t="n">
+      <c r="D4762" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-14 08:34 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4770"/>
+  <dimension ref="A1:D4771"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85539,16 +85539,16 @@
     <row r="4729">
       <c r="A4729" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/14</t>
         </is>
       </c>
       <c r="B4729" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4729" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D4729" t="n">
         <v>201</v>
@@ -85566,7 +85566,7 @@
         </is>
       </c>
       <c r="C4730" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4730" t="n">
         <v>201</v>
@@ -85584,7 +85584,7 @@
         </is>
       </c>
       <c r="C4731" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4731" t="n">
         <v>201</v>
@@ -85602,7 +85602,7 @@
         </is>
       </c>
       <c r="C4732" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4732" t="n">
         <v>201</v>
@@ -85611,16 +85611,16 @@
     <row r="4733">
       <c r="A4733" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4733" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4733" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4733" t="n">
         <v>201</v>
@@ -85638,7 +85638,7 @@
         </is>
       </c>
       <c r="C4734" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4734" t="n">
         <v>201</v>
@@ -85656,7 +85656,7 @@
         </is>
       </c>
       <c r="C4735" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4735" t="n">
         <v>201</v>
@@ -85674,7 +85674,7 @@
         </is>
       </c>
       <c r="C4736" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4736" t="n">
         <v>201</v>
@@ -85692,7 +85692,7 @@
         </is>
       </c>
       <c r="C4737" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4737" t="n">
         <v>201</v>
@@ -85710,7 +85710,7 @@
         </is>
       </c>
       <c r="C4738" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4738" t="n">
         <v>201</v>
@@ -85719,16 +85719,16 @@
     <row r="4739">
       <c r="A4739" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4739" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4739" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4739" t="n">
         <v>201</v>
@@ -85746,7 +85746,7 @@
         </is>
       </c>
       <c r="C4740" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4740" t="n">
         <v>201</v>
@@ -85764,7 +85764,7 @@
         </is>
       </c>
       <c r="C4741" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4741" t="n">
         <v>201</v>
@@ -85782,7 +85782,7 @@
         </is>
       </c>
       <c r="C4742" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4742" t="n">
         <v>201</v>
@@ -85800,7 +85800,7 @@
         </is>
       </c>
       <c r="C4743" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4743" t="n">
         <v>201</v>
@@ -85818,7 +85818,7 @@
         </is>
       </c>
       <c r="C4744" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4744" t="n">
         <v>201</v>
@@ -85827,16 +85827,16 @@
     <row r="4745">
       <c r="A4745" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4745" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4745" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4745" t="n">
         <v>201</v>
@@ -85854,7 +85854,7 @@
         </is>
       </c>
       <c r="C4746" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4746" t="n">
         <v>201</v>
@@ -85872,7 +85872,7 @@
         </is>
       </c>
       <c r="C4747" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4747" t="n">
         <v>201</v>
@@ -85890,7 +85890,7 @@
         </is>
       </c>
       <c r="C4748" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4748" t="n">
         <v>201</v>
@@ -85908,7 +85908,7 @@
         </is>
       </c>
       <c r="C4749" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4749" t="n">
         <v>201</v>
@@ -85917,16 +85917,16 @@
     <row r="4750">
       <c r="A4750" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4750" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4750" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4750" t="n">
         <v>201</v>
@@ -85944,7 +85944,7 @@
         </is>
       </c>
       <c r="C4751" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4751" t="n">
         <v>201</v>
@@ -85962,7 +85962,7 @@
         </is>
       </c>
       <c r="C4752" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4752" t="n">
         <v>201</v>
@@ -85980,7 +85980,7 @@
         </is>
       </c>
       <c r="C4753" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4753" t="n">
         <v>201</v>
@@ -85998,7 +85998,7 @@
         </is>
       </c>
       <c r="C4754" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4754" t="n">
         <v>201</v>
@@ -86016,7 +86016,7 @@
         </is>
       </c>
       <c r="C4755" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4755" t="n">
         <v>201</v>
@@ -86034,7 +86034,7 @@
         </is>
       </c>
       <c r="C4756" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4756" t="n">
         <v>201</v>
@@ -86043,16 +86043,16 @@
     <row r="4757">
       <c r="A4757" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4757" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4757" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4757" t="n">
         <v>201</v>
@@ -86070,7 +86070,7 @@
         </is>
       </c>
       <c r="C4758" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4758" t="n">
         <v>201</v>
@@ -86088,7 +86088,7 @@
         </is>
       </c>
       <c r="C4759" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4759" t="n">
         <v>201</v>
@@ -86106,7 +86106,7 @@
         </is>
       </c>
       <c r="C4760" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4760" t="n">
         <v>201</v>
@@ -86124,7 +86124,7 @@
         </is>
       </c>
       <c r="C4761" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4761" t="n">
         <v>201</v>
@@ -86142,7 +86142,7 @@
         </is>
       </c>
       <c r="C4762" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4762" t="n">
         <v>201</v>
@@ -86160,7 +86160,7 @@
         </is>
       </c>
       <c r="C4763" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4763" t="n">
         <v>201</v>
@@ -86169,16 +86169,16 @@
     <row r="4764">
       <c r="A4764" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4764" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4764" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4764" t="n">
         <v>201</v>
@@ -86196,7 +86196,7 @@
         </is>
       </c>
       <c r="C4765" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4765" t="n">
         <v>201</v>
@@ -86214,7 +86214,7 @@
         </is>
       </c>
       <c r="C4766" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4766" t="n">
         <v>201</v>
@@ -86232,7 +86232,7 @@
         </is>
       </c>
       <c r="C4767" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4767" t="n">
         <v>201</v>
@@ -86250,7 +86250,7 @@
         </is>
       </c>
       <c r="C4768" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4768" t="n">
         <v>201</v>
@@ -86259,16 +86259,16 @@
     <row r="4769">
       <c r="A4769" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4769" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4769" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4769" t="n">
         <v>201</v>
@@ -86286,9 +86286,27 @@
         </is>
       </c>
       <c r="C4770" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4770" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4771">
+      <c r="A4771" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4771" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4771" t="n">
         <v>7</v>
       </c>
-      <c r="D4770" t="n">
+      <c r="D4771" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-18 18:52 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4803"/>
+  <dimension ref="A1:D4804"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86133,7 +86133,7 @@
     <row r="4762">
       <c r="A4762" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/18</t>
         </is>
       </c>
       <c r="B4762" t="inlineStr">
@@ -86142,7 +86142,7 @@
         </is>
       </c>
       <c r="C4762" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D4762" t="n">
         <v>201</v>
@@ -86160,7 +86160,7 @@
         </is>
       </c>
       <c r="C4763" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4763" t="n">
         <v>201</v>
@@ -86178,7 +86178,7 @@
         </is>
       </c>
       <c r="C4764" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4764" t="n">
         <v>201</v>
@@ -86196,7 +86196,7 @@
         </is>
       </c>
       <c r="C4765" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4765" t="n">
         <v>201</v>
@@ -86205,16 +86205,16 @@
     <row r="4766">
       <c r="A4766" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4766" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4766" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4766" t="n">
         <v>201</v>
@@ -86232,7 +86232,7 @@
         </is>
       </c>
       <c r="C4767" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4767" t="n">
         <v>201</v>
@@ -86250,7 +86250,7 @@
         </is>
       </c>
       <c r="C4768" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4768" t="n">
         <v>201</v>
@@ -86268,7 +86268,7 @@
         </is>
       </c>
       <c r="C4769" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4769" t="n">
         <v>201</v>
@@ -86286,7 +86286,7 @@
         </is>
       </c>
       <c r="C4770" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4770" t="n">
         <v>201</v>
@@ -86304,7 +86304,7 @@
         </is>
       </c>
       <c r="C4771" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4771" t="n">
         <v>201</v>
@@ -86313,16 +86313,16 @@
     <row r="4772">
       <c r="A4772" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4772" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4772" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4772" t="n">
         <v>201</v>
@@ -86340,7 +86340,7 @@
         </is>
       </c>
       <c r="C4773" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4773" t="n">
         <v>201</v>
@@ -86358,7 +86358,7 @@
         </is>
       </c>
       <c r="C4774" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4774" t="n">
         <v>201</v>
@@ -86376,7 +86376,7 @@
         </is>
       </c>
       <c r="C4775" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4775" t="n">
         <v>201</v>
@@ -86394,7 +86394,7 @@
         </is>
       </c>
       <c r="C4776" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4776" t="n">
         <v>201</v>
@@ -86412,7 +86412,7 @@
         </is>
       </c>
       <c r="C4777" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4777" t="n">
         <v>201</v>
@@ -86421,16 +86421,16 @@
     <row r="4778">
       <c r="A4778" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4778" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4778" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4778" t="n">
         <v>201</v>
@@ -86448,7 +86448,7 @@
         </is>
       </c>
       <c r="C4779" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4779" t="n">
         <v>201</v>
@@ -86466,7 +86466,7 @@
         </is>
       </c>
       <c r="C4780" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4780" t="n">
         <v>201</v>
@@ -86484,7 +86484,7 @@
         </is>
       </c>
       <c r="C4781" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4781" t="n">
         <v>201</v>
@@ -86502,7 +86502,7 @@
         </is>
       </c>
       <c r="C4782" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4782" t="n">
         <v>201</v>
@@ -86511,16 +86511,16 @@
     <row r="4783">
       <c r="A4783" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4783" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4783" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4783" t="n">
         <v>201</v>
@@ -86538,7 +86538,7 @@
         </is>
       </c>
       <c r="C4784" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4784" t="n">
         <v>201</v>
@@ -86556,7 +86556,7 @@
         </is>
       </c>
       <c r="C4785" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4785" t="n">
         <v>201</v>
@@ -86574,7 +86574,7 @@
         </is>
       </c>
       <c r="C4786" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4786" t="n">
         <v>201</v>
@@ -86592,7 +86592,7 @@
         </is>
       </c>
       <c r="C4787" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4787" t="n">
         <v>201</v>
@@ -86610,7 +86610,7 @@
         </is>
       </c>
       <c r="C4788" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4788" t="n">
         <v>201</v>
@@ -86628,7 +86628,7 @@
         </is>
       </c>
       <c r="C4789" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4789" t="n">
         <v>201</v>
@@ -86637,16 +86637,16 @@
     <row r="4790">
       <c r="A4790" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4790" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4790" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4790" t="n">
         <v>201</v>
@@ -86664,7 +86664,7 @@
         </is>
       </c>
       <c r="C4791" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4791" t="n">
         <v>201</v>
@@ -86682,7 +86682,7 @@
         </is>
       </c>
       <c r="C4792" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4792" t="n">
         <v>201</v>
@@ -86700,7 +86700,7 @@
         </is>
       </c>
       <c r="C4793" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4793" t="n">
         <v>201</v>
@@ -86718,7 +86718,7 @@
         </is>
       </c>
       <c r="C4794" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4794" t="n">
         <v>201</v>
@@ -86736,7 +86736,7 @@
         </is>
       </c>
       <c r="C4795" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4795" t="n">
         <v>201</v>
@@ -86754,7 +86754,7 @@
         </is>
       </c>
       <c r="C4796" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4796" t="n">
         <v>201</v>
@@ -86763,16 +86763,16 @@
     <row r="4797">
       <c r="A4797" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4797" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4797" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4797" t="n">
         <v>201</v>
@@ -86790,7 +86790,7 @@
         </is>
       </c>
       <c r="C4798" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4798" t="n">
         <v>201</v>
@@ -86808,7 +86808,7 @@
         </is>
       </c>
       <c r="C4799" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4799" t="n">
         <v>201</v>
@@ -86826,7 +86826,7 @@
         </is>
       </c>
       <c r="C4800" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4800" t="n">
         <v>201</v>
@@ -86844,7 +86844,7 @@
         </is>
       </c>
       <c r="C4801" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4801" t="n">
         <v>201</v>
@@ -86853,16 +86853,16 @@
     <row r="4802">
       <c r="A4802" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4802" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4802" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4802" t="n">
         <v>201</v>
@@ -86880,9 +86880,27 @@
         </is>
       </c>
       <c r="C4803" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4803" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4804">
+      <c r="A4804" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4804" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4804" t="n">
         <v>7</v>
       </c>
-      <c r="D4803" t="n">
+      <c r="D4804" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-20 09:46 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4814"/>
+  <dimension ref="A1:D4815"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86331,16 +86331,16 @@
     <row r="4773">
       <c r="A4773" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/20</t>
         </is>
       </c>
       <c r="B4773" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4773" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D4773" t="n">
         <v>201</v>
@@ -86358,7 +86358,7 @@
         </is>
       </c>
       <c r="C4774" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4774" t="n">
         <v>201</v>
@@ -86376,7 +86376,7 @@
         </is>
       </c>
       <c r="C4775" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4775" t="n">
         <v>201</v>
@@ -86394,7 +86394,7 @@
         </is>
       </c>
       <c r="C4776" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4776" t="n">
         <v>201</v>
@@ -86403,16 +86403,16 @@
     <row r="4777">
       <c r="A4777" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4777" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4777" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4777" t="n">
         <v>201</v>
@@ -86430,7 +86430,7 @@
         </is>
       </c>
       <c r="C4778" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4778" t="n">
         <v>201</v>
@@ -86448,7 +86448,7 @@
         </is>
       </c>
       <c r="C4779" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4779" t="n">
         <v>201</v>
@@ -86466,7 +86466,7 @@
         </is>
       </c>
       <c r="C4780" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4780" t="n">
         <v>201</v>
@@ -86484,7 +86484,7 @@
         </is>
       </c>
       <c r="C4781" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4781" t="n">
         <v>201</v>
@@ -86502,7 +86502,7 @@
         </is>
       </c>
       <c r="C4782" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4782" t="n">
         <v>201</v>
@@ -86511,16 +86511,16 @@
     <row r="4783">
       <c r="A4783" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4783" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4783" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4783" t="n">
         <v>201</v>
@@ -86538,7 +86538,7 @@
         </is>
       </c>
       <c r="C4784" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4784" t="n">
         <v>201</v>
@@ -86556,7 +86556,7 @@
         </is>
       </c>
       <c r="C4785" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4785" t="n">
         <v>201</v>
@@ -86574,7 +86574,7 @@
         </is>
       </c>
       <c r="C4786" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4786" t="n">
         <v>201</v>
@@ -86592,7 +86592,7 @@
         </is>
       </c>
       <c r="C4787" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4787" t="n">
         <v>201</v>
@@ -86610,7 +86610,7 @@
         </is>
       </c>
       <c r="C4788" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4788" t="n">
         <v>201</v>
@@ -86619,16 +86619,16 @@
     <row r="4789">
       <c r="A4789" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4789" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4789" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4789" t="n">
         <v>201</v>
@@ -86646,7 +86646,7 @@
         </is>
       </c>
       <c r="C4790" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4790" t="n">
         <v>201</v>
@@ -86664,7 +86664,7 @@
         </is>
       </c>
       <c r="C4791" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4791" t="n">
         <v>201</v>
@@ -86682,7 +86682,7 @@
         </is>
       </c>
       <c r="C4792" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4792" t="n">
         <v>201</v>
@@ -86700,7 +86700,7 @@
         </is>
       </c>
       <c r="C4793" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4793" t="n">
         <v>201</v>
@@ -86709,16 +86709,16 @@
     <row r="4794">
       <c r="A4794" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4794" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4794" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4794" t="n">
         <v>201</v>
@@ -86736,7 +86736,7 @@
         </is>
       </c>
       <c r="C4795" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4795" t="n">
         <v>201</v>
@@ -86754,7 +86754,7 @@
         </is>
       </c>
       <c r="C4796" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4796" t="n">
         <v>201</v>
@@ -86772,7 +86772,7 @@
         </is>
       </c>
       <c r="C4797" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4797" t="n">
         <v>201</v>
@@ -86790,7 +86790,7 @@
         </is>
       </c>
       <c r="C4798" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4798" t="n">
         <v>201</v>
@@ -86808,7 +86808,7 @@
         </is>
       </c>
       <c r="C4799" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4799" t="n">
         <v>201</v>
@@ -86826,7 +86826,7 @@
         </is>
       </c>
       <c r="C4800" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4800" t="n">
         <v>201</v>
@@ -86835,16 +86835,16 @@
     <row r="4801">
       <c r="A4801" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4801" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4801" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4801" t="n">
         <v>201</v>
@@ -86862,7 +86862,7 @@
         </is>
       </c>
       <c r="C4802" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4802" t="n">
         <v>201</v>
@@ -86880,7 +86880,7 @@
         </is>
       </c>
       <c r="C4803" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4803" t="n">
         <v>201</v>
@@ -86898,7 +86898,7 @@
         </is>
       </c>
       <c r="C4804" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4804" t="n">
         <v>201</v>
@@ -86916,7 +86916,7 @@
         </is>
       </c>
       <c r="C4805" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4805" t="n">
         <v>201</v>
@@ -86934,7 +86934,7 @@
         </is>
       </c>
       <c r="C4806" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4806" t="n">
         <v>201</v>
@@ -86952,7 +86952,7 @@
         </is>
       </c>
       <c r="C4807" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4807" t="n">
         <v>201</v>
@@ -86961,16 +86961,16 @@
     <row r="4808">
       <c r="A4808" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4808" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4808" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4808" t="n">
         <v>201</v>
@@ -86988,7 +86988,7 @@
         </is>
       </c>
       <c r="C4809" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4809" t="n">
         <v>201</v>
@@ -87006,7 +87006,7 @@
         </is>
       </c>
       <c r="C4810" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4810" t="n">
         <v>201</v>
@@ -87024,7 +87024,7 @@
         </is>
       </c>
       <c r="C4811" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4811" t="n">
         <v>201</v>
@@ -87042,7 +87042,7 @@
         </is>
       </c>
       <c r="C4812" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4812" t="n">
         <v>201</v>
@@ -87051,16 +87051,16 @@
     <row r="4813">
       <c r="A4813" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4813" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4813" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4813" t="n">
         <v>201</v>
@@ -87078,9 +87078,27 @@
         </is>
       </c>
       <c r="C4814" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4814" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4815">
+      <c r="A4815" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4815" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4815" t="n">
         <v>7</v>
       </c>
-      <c r="D4814" t="n">
+      <c r="D4815" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-24 08:02 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4842"/>
+  <dimension ref="A1:D4843"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86835,16 +86835,16 @@
     <row r="4801">
       <c r="A4801" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/24</t>
         </is>
       </c>
       <c r="B4801" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4801" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D4801" t="n">
         <v>201</v>
@@ -86862,7 +86862,7 @@
         </is>
       </c>
       <c r="C4802" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4802" t="n">
         <v>201</v>
@@ -86880,7 +86880,7 @@
         </is>
       </c>
       <c r="C4803" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4803" t="n">
         <v>201</v>
@@ -86898,7 +86898,7 @@
         </is>
       </c>
       <c r="C4804" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4804" t="n">
         <v>201</v>
@@ -86907,16 +86907,16 @@
     <row r="4805">
       <c r="A4805" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4805" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4805" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4805" t="n">
         <v>201</v>
@@ -86934,7 +86934,7 @@
         </is>
       </c>
       <c r="C4806" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4806" t="n">
         <v>201</v>
@@ -86952,7 +86952,7 @@
         </is>
       </c>
       <c r="C4807" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4807" t="n">
         <v>201</v>
@@ -86970,7 +86970,7 @@
         </is>
       </c>
       <c r="C4808" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4808" t="n">
         <v>201</v>
@@ -86988,7 +86988,7 @@
         </is>
       </c>
       <c r="C4809" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4809" t="n">
         <v>201</v>
@@ -87006,7 +87006,7 @@
         </is>
       </c>
       <c r="C4810" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4810" t="n">
         <v>201</v>
@@ -87015,16 +87015,16 @@
     <row r="4811">
       <c r="A4811" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4811" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4811" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4811" t="n">
         <v>201</v>
@@ -87042,7 +87042,7 @@
         </is>
       </c>
       <c r="C4812" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4812" t="n">
         <v>201</v>
@@ -87060,7 +87060,7 @@
         </is>
       </c>
       <c r="C4813" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4813" t="n">
         <v>201</v>
@@ -87078,7 +87078,7 @@
         </is>
       </c>
       <c r="C4814" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4814" t="n">
         <v>201</v>
@@ -87096,7 +87096,7 @@
         </is>
       </c>
       <c r="C4815" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4815" t="n">
         <v>201</v>
@@ -87114,7 +87114,7 @@
         </is>
       </c>
       <c r="C4816" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4816" t="n">
         <v>201</v>
@@ -87123,16 +87123,16 @@
     <row r="4817">
       <c r="A4817" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4817" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4817" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4817" t="n">
         <v>201</v>
@@ -87150,7 +87150,7 @@
         </is>
       </c>
       <c r="C4818" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4818" t="n">
         <v>201</v>
@@ -87168,7 +87168,7 @@
         </is>
       </c>
       <c r="C4819" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4819" t="n">
         <v>201</v>
@@ -87186,7 +87186,7 @@
         </is>
       </c>
       <c r="C4820" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4820" t="n">
         <v>201</v>
@@ -87204,7 +87204,7 @@
         </is>
       </c>
       <c r="C4821" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4821" t="n">
         <v>201</v>
@@ -87213,16 +87213,16 @@
     <row r="4822">
       <c r="A4822" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4822" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4822" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4822" t="n">
         <v>201</v>
@@ -87240,7 +87240,7 @@
         </is>
       </c>
       <c r="C4823" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4823" t="n">
         <v>201</v>
@@ -87258,7 +87258,7 @@
         </is>
       </c>
       <c r="C4824" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4824" t="n">
         <v>201</v>
@@ -87276,7 +87276,7 @@
         </is>
       </c>
       <c r="C4825" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4825" t="n">
         <v>201</v>
@@ -87294,7 +87294,7 @@
         </is>
       </c>
       <c r="C4826" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4826" t="n">
         <v>201</v>
@@ -87312,7 +87312,7 @@
         </is>
       </c>
       <c r="C4827" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4827" t="n">
         <v>201</v>
@@ -87330,7 +87330,7 @@
         </is>
       </c>
       <c r="C4828" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4828" t="n">
         <v>201</v>
@@ -87339,16 +87339,16 @@
     <row r="4829">
       <c r="A4829" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4829" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4829" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4829" t="n">
         <v>201</v>
@@ -87366,7 +87366,7 @@
         </is>
       </c>
       <c r="C4830" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4830" t="n">
         <v>201</v>
@@ -87384,7 +87384,7 @@
         </is>
       </c>
       <c r="C4831" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4831" t="n">
         <v>201</v>
@@ -87402,7 +87402,7 @@
         </is>
       </c>
       <c r="C4832" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4832" t="n">
         <v>201</v>
@@ -87420,7 +87420,7 @@
         </is>
       </c>
       <c r="C4833" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4833" t="n">
         <v>201</v>
@@ -87438,7 +87438,7 @@
         </is>
       </c>
       <c r="C4834" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4834" t="n">
         <v>201</v>
@@ -87456,7 +87456,7 @@
         </is>
       </c>
       <c r="C4835" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4835" t="n">
         <v>201</v>
@@ -87465,16 +87465,16 @@
     <row r="4836">
       <c r="A4836" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4836" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4836" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4836" t="n">
         <v>201</v>
@@ -87492,7 +87492,7 @@
         </is>
       </c>
       <c r="C4837" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4837" t="n">
         <v>201</v>
@@ -87510,7 +87510,7 @@
         </is>
       </c>
       <c r="C4838" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4838" t="n">
         <v>201</v>
@@ -87528,7 +87528,7 @@
         </is>
       </c>
       <c r="C4839" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4839" t="n">
         <v>201</v>
@@ -87546,7 +87546,7 @@
         </is>
       </c>
       <c r="C4840" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4840" t="n">
         <v>201</v>
@@ -87555,16 +87555,16 @@
     <row r="4841">
       <c r="A4841" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4841" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4841" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4841" t="n">
         <v>201</v>
@@ -87582,9 +87582,27 @@
         </is>
       </c>
       <c r="C4842" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4842" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4843">
+      <c r="A4843" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4843" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4843" t="n">
         <v>7</v>
       </c>
-      <c r="D4842" t="n">
+      <c r="D4843" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-04 16:50 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4922"/>
+  <dimension ref="A1:D4923"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88275,16 +88275,16 @@
     <row r="4881">
       <c r="A4881" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/04</t>
         </is>
       </c>
       <c r="B4881" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4881" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D4881" t="n">
         <v>201</v>
@@ -88302,7 +88302,7 @@
         </is>
       </c>
       <c r="C4882" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4882" t="n">
         <v>201</v>
@@ -88320,7 +88320,7 @@
         </is>
       </c>
       <c r="C4883" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4883" t="n">
         <v>201</v>
@@ -88338,7 +88338,7 @@
         </is>
       </c>
       <c r="C4884" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4884" t="n">
         <v>201</v>
@@ -88347,16 +88347,16 @@
     <row r="4885">
       <c r="A4885" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4885" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4885" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4885" t="n">
         <v>201</v>
@@ -88374,7 +88374,7 @@
         </is>
       </c>
       <c r="C4886" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4886" t="n">
         <v>201</v>
@@ -88392,7 +88392,7 @@
         </is>
       </c>
       <c r="C4887" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4887" t="n">
         <v>201</v>
@@ -88410,7 +88410,7 @@
         </is>
       </c>
       <c r="C4888" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4888" t="n">
         <v>201</v>
@@ -88428,7 +88428,7 @@
         </is>
       </c>
       <c r="C4889" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4889" t="n">
         <v>201</v>
@@ -88446,7 +88446,7 @@
         </is>
       </c>
       <c r="C4890" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4890" t="n">
         <v>201</v>
@@ -88455,16 +88455,16 @@
     <row r="4891">
       <c r="A4891" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4891" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4891" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4891" t="n">
         <v>201</v>
@@ -88482,7 +88482,7 @@
         </is>
       </c>
       <c r="C4892" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4892" t="n">
         <v>201</v>
@@ -88500,7 +88500,7 @@
         </is>
       </c>
       <c r="C4893" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4893" t="n">
         <v>201</v>
@@ -88518,7 +88518,7 @@
         </is>
       </c>
       <c r="C4894" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4894" t="n">
         <v>201</v>
@@ -88536,7 +88536,7 @@
         </is>
       </c>
       <c r="C4895" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4895" t="n">
         <v>201</v>
@@ -88554,7 +88554,7 @@
         </is>
       </c>
       <c r="C4896" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4896" t="n">
         <v>201</v>
@@ -88563,16 +88563,16 @@
     <row r="4897">
       <c r="A4897" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4897" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4897" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4897" t="n">
         <v>201</v>
@@ -88590,7 +88590,7 @@
         </is>
       </c>
       <c r="C4898" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4898" t="n">
         <v>201</v>
@@ -88608,7 +88608,7 @@
         </is>
       </c>
       <c r="C4899" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4899" t="n">
         <v>201</v>
@@ -88626,7 +88626,7 @@
         </is>
       </c>
       <c r="C4900" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4900" t="n">
         <v>201</v>
@@ -88644,7 +88644,7 @@
         </is>
       </c>
       <c r="C4901" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4901" t="n">
         <v>201</v>
@@ -88653,16 +88653,16 @@
     <row r="4902">
       <c r="A4902" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4902" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4902" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4902" t="n">
         <v>201</v>
@@ -88680,7 +88680,7 @@
         </is>
       </c>
       <c r="C4903" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4903" t="n">
         <v>201</v>
@@ -88698,7 +88698,7 @@
         </is>
       </c>
       <c r="C4904" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4904" t="n">
         <v>201</v>
@@ -88716,7 +88716,7 @@
         </is>
       </c>
       <c r="C4905" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4905" t="n">
         <v>201</v>
@@ -88734,7 +88734,7 @@
         </is>
       </c>
       <c r="C4906" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4906" t="n">
         <v>201</v>
@@ -88752,7 +88752,7 @@
         </is>
       </c>
       <c r="C4907" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4907" t="n">
         <v>201</v>
@@ -88770,7 +88770,7 @@
         </is>
       </c>
       <c r="C4908" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4908" t="n">
         <v>201</v>
@@ -88779,16 +88779,16 @@
     <row r="4909">
       <c r="A4909" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4909" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4909" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4909" t="n">
         <v>201</v>
@@ -88806,7 +88806,7 @@
         </is>
       </c>
       <c r="C4910" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4910" t="n">
         <v>201</v>
@@ -88824,7 +88824,7 @@
         </is>
       </c>
       <c r="C4911" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4911" t="n">
         <v>201</v>
@@ -88842,7 +88842,7 @@
         </is>
       </c>
       <c r="C4912" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4912" t="n">
         <v>201</v>
@@ -88860,7 +88860,7 @@
         </is>
       </c>
       <c r="C4913" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4913" t="n">
         <v>201</v>
@@ -88878,7 +88878,7 @@
         </is>
       </c>
       <c r="C4914" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4914" t="n">
         <v>201</v>
@@ -88896,7 +88896,7 @@
         </is>
       </c>
       <c r="C4915" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4915" t="n">
         <v>201</v>
@@ -88905,16 +88905,16 @@
     <row r="4916">
       <c r="A4916" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4916" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4916" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4916" t="n">
         <v>201</v>
@@ -88932,7 +88932,7 @@
         </is>
       </c>
       <c r="C4917" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4917" t="n">
         <v>201</v>
@@ -88950,7 +88950,7 @@
         </is>
       </c>
       <c r="C4918" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4918" t="n">
         <v>201</v>
@@ -88968,7 +88968,7 @@
         </is>
       </c>
       <c r="C4919" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4919" t="n">
         <v>201</v>
@@ -88986,7 +88986,7 @@
         </is>
       </c>
       <c r="C4920" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4920" t="n">
         <v>201</v>
@@ -88995,16 +88995,16 @@
     <row r="4921">
       <c r="A4921" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4921" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4921" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4921" t="n">
         <v>201</v>
@@ -89022,9 +89022,27 @@
         </is>
       </c>
       <c r="C4922" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4922" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4923">
+      <c r="A4923" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4923" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4923" t="n">
         <v>7</v>
       </c>
-      <c r="D4922" t="n">
+      <c r="D4923" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-09 07:20 UTC
</commit_message>
<xml_diff>
--- a/excel/apple2.xlsx
+++ b/excel/apple2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4956"/>
+  <dimension ref="A1:D4957"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88887,16 +88887,16 @@
     <row r="4915">
       <c r="A4915" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/09</t>
         </is>
       </c>
       <c r="B4915" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4915" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4915" t="n">
         <v>201</v>
@@ -88914,7 +88914,7 @@
         </is>
       </c>
       <c r="C4916" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4916" t="n">
         <v>201</v>
@@ -88932,7 +88932,7 @@
         </is>
       </c>
       <c r="C4917" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4917" t="n">
         <v>201</v>
@@ -88950,7 +88950,7 @@
         </is>
       </c>
       <c r="C4918" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4918" t="n">
         <v>201</v>
@@ -88959,16 +88959,16 @@
     <row r="4919">
       <c r="A4919" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4919" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4919" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4919" t="n">
         <v>201</v>
@@ -88986,7 +88986,7 @@
         </is>
       </c>
       <c r="C4920" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4920" t="n">
         <v>201</v>
@@ -89004,7 +89004,7 @@
         </is>
       </c>
       <c r="C4921" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4921" t="n">
         <v>201</v>
@@ -89022,7 +89022,7 @@
         </is>
       </c>
       <c r="C4922" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4922" t="n">
         <v>201</v>
@@ -89040,7 +89040,7 @@
         </is>
       </c>
       <c r="C4923" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4923" t="n">
         <v>201</v>
@@ -89058,7 +89058,7 @@
         </is>
       </c>
       <c r="C4924" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4924" t="n">
         <v>201</v>
@@ -89067,16 +89067,16 @@
     <row r="4925">
       <c r="A4925" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4925" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4925" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4925" t="n">
         <v>201</v>
@@ -89094,7 +89094,7 @@
         </is>
       </c>
       <c r="C4926" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4926" t="n">
         <v>201</v>
@@ -89112,7 +89112,7 @@
         </is>
       </c>
       <c r="C4927" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4927" t="n">
         <v>201</v>
@@ -89130,7 +89130,7 @@
         </is>
       </c>
       <c r="C4928" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4928" t="n">
         <v>201</v>
@@ -89148,7 +89148,7 @@
         </is>
       </c>
       <c r="C4929" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4929" t="n">
         <v>201</v>
@@ -89166,7 +89166,7 @@
         </is>
       </c>
       <c r="C4930" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4930" t="n">
         <v>201</v>
@@ -89175,16 +89175,16 @@
     <row r="4931">
       <c r="A4931" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4931" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4931" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4931" t="n">
         <v>201</v>
@@ -89202,7 +89202,7 @@
         </is>
       </c>
       <c r="C4932" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4932" t="n">
         <v>201</v>
@@ -89220,7 +89220,7 @@
         </is>
       </c>
       <c r="C4933" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4933" t="n">
         <v>201</v>
@@ -89238,7 +89238,7 @@
         </is>
       </c>
       <c r="C4934" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4934" t="n">
         <v>201</v>
@@ -89256,7 +89256,7 @@
         </is>
       </c>
       <c r="C4935" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4935" t="n">
         <v>201</v>
@@ -89265,16 +89265,16 @@
     <row r="4936">
       <c r="A4936" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4936" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4936" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4936" t="n">
         <v>201</v>
@@ -89292,7 +89292,7 @@
         </is>
       </c>
       <c r="C4937" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4937" t="n">
         <v>201</v>
@@ -89310,7 +89310,7 @@
         </is>
       </c>
       <c r="C4938" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4938" t="n">
         <v>201</v>
@@ -89328,7 +89328,7 @@
         </is>
       </c>
       <c r="C4939" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4939" t="n">
         <v>201</v>
@@ -89346,7 +89346,7 @@
         </is>
       </c>
       <c r="C4940" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4940" t="n">
         <v>201</v>
@@ -89364,7 +89364,7 @@
         </is>
       </c>
       <c r="C4941" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4941" t="n">
         <v>201</v>
@@ -89382,7 +89382,7 @@
         </is>
       </c>
       <c r="C4942" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4942" t="n">
         <v>201</v>
@@ -89391,16 +89391,16 @@
     <row r="4943">
       <c r="A4943" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4943" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4943" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4943" t="n">
         <v>201</v>
@@ -89418,7 +89418,7 @@
         </is>
       </c>
       <c r="C4944" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4944" t="n">
         <v>201</v>
@@ -89436,7 +89436,7 @@
         </is>
       </c>
       <c r="C4945" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4945" t="n">
         <v>201</v>
@@ -89454,7 +89454,7 @@
         </is>
       </c>
       <c r="C4946" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4946" t="n">
         <v>201</v>
@@ -89472,7 +89472,7 @@
         </is>
       </c>
       <c r="C4947" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4947" t="n">
         <v>201</v>
@@ -89490,7 +89490,7 @@
         </is>
       </c>
       <c r="C4948" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4948" t="n">
         <v>201</v>
@@ -89508,7 +89508,7 @@
         </is>
       </c>
       <c r="C4949" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4949" t="n">
         <v>201</v>
@@ -89517,16 +89517,16 @@
     <row r="4950">
       <c r="A4950" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4950" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4950" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4950" t="n">
         <v>201</v>
@@ -89544,7 +89544,7 @@
         </is>
       </c>
       <c r="C4951" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4951" t="n">
         <v>201</v>
@@ -89562,7 +89562,7 @@
         </is>
       </c>
       <c r="C4952" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4952" t="n">
         <v>201</v>
@@ -89580,7 +89580,7 @@
         </is>
       </c>
       <c r="C4953" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4953" t="n">
         <v>201</v>
@@ -89598,7 +89598,7 @@
         </is>
       </c>
       <c r="C4954" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4954" t="n">
         <v>201</v>
@@ -89607,16 +89607,16 @@
     <row r="4955">
       <c r="A4955" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4955" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4955" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4955" t="n">
         <v>201</v>
@@ -89634,9 +89634,27 @@
         </is>
       </c>
       <c r="C4956" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4956" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4957">
+      <c r="A4957" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4957" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4957" t="n">
         <v>7</v>
       </c>
-      <c r="D4956" t="n">
+      <c r="D4957" t="n">
         <v>201</v>
       </c>
     </row>

</xml_diff>